<commit_message>
İç link gerekçeleri, anlaşılır yönerge dili ve iç referans kodlarının kaldırılması
- İç link önerileri 2-4 arası; her bağlantıda anchor metninin gövdede ya da
  yazı planında geçip geçmediği ve buna göre ne yapılacağı yazılı
- Genel açıklama cümlesi kaldırıldı, yerini kelime bazlı gerekçe aldı
- İçerik yönergesi maddeleri tam cümleye çevrildi
- Tablolardaki P/K/G iç referans kodları kaldırıldı

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -4439,9 +4439,9 @@
       <c r="L4" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-2. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. 4.5 g ile 5g arasındaki : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -4467,11 +4467,11 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>• 192.168.1.1 ve 192.168.0.1 farkı; 
-  • marka bazında varsayılan kullanıcı adı ve şifre tablosu; 
-  • arayüze girilemediğinde kontrol listesi; 
-  • WiFi adı ve şifresi değiştirme; 
-  • modem sıfırlama.</t>
+          <t>1. 192.168.1.1 ve 192.168.0.1 farkı açıklanır
+2. Marka bazında varsayılan kullanıcı adı ve şifre tablosu verilir
+3. Arayüze girilemediğinde kontrol listesi verilir
+4. WiFi adı ve şifresi değiştirme adım adım anlatılır
+5. Modem sıfırlama adım adım anlatılır</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -4575,9 +4575,9 @@
       <c r="L5" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -4620,11 +4620,11 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>• Numara gizleme kodu ve operatör ayarı; 
-  • gizli numaradan gelen aramayı engelleme; 
-  • iPhone ve Android ayrı adımlar; 
-  • operatör servisiyle kalıcı engelleme; 
-  • yasal sınırlar.</t>
+          <t>1. Numara gizleme kodu ve operatör ayarı açıklanır
+2. Gizli numaradan gelen aramayı engelleme adım adım anlatılır
+3. IPhone ve Android ayrı adımlar adım adım anlatılır
+4. Operatör servisiyle kalıcı engelleme adım adım anlatılır
+5. Yasal sınırlar açıklanır</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -4735,9 +4735,9 @@
       <c r="L6" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -4797,11 +4797,11 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>• Kayıt ücreti ve geçerli yılın harç tutarı tablo hâlinde; 
-  • e-Devlet ve BTK üzerinden sorgulama adımları; 
-  • kayıtsız telefonun kaç gün kullanılabildiği; 
-  • IMEI numarasının telefondan öğrenilmesi; 
-  • kayıt sonrası bekleme süresi.</t>
+          <t>1. Kayıt ücreti ve geçerli yılın harç tutarı tablo hâlinde açıklanır
+2. E-Devlet ve BTK üzerinden sorgulama adımları adım adım anlatılır
+3. Kayıtsız telefonun kaç gün kullanılabildiği açıklanır
+4. IMEI numarasının telefondan öğrenilmesi adım adım anlatılır
+5. Kayıt sonrası bekleme süresi açıklanır</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
@@ -4833,7 +4833,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="115" customHeight="1">
+    <row r="7" ht="128.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Google Güvenli Arama: Açma, Kapatma ve Aile Filtresi</t>
@@ -4894,9 +4894,9 @@
       <c r="L7" s="4" t="inlineStr">
         <is>
           <t>1. turkcell chatgpt : https://www.turkcell.com.tr/blog/chatgpt-yeni-google-mi-internette-arama-aliskanliklari-nasil-degisiyor
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-3. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-4. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -4956,10 +4956,10 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>• Google güvenli aramanın ne yaptığı; 
-  • açma ve kapatma adımları; 
-  • kilitli olduğunda yapılabilecekler; 
-  • çocuk hesaplarında aile bağlantısı ayarı.</t>
+          <t>1. Google güvenli aramanın ne yaptığı açıklanır
+2. Açma ve kapatma adımları adım adım anlatılır
+3. Kilitli olduğunda yapılabilecekler açıklanır
+4. Çocuk hesaplarında aile bağlantısı ayarı açıklanır</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
@@ -5055,9 +5055,9 @@
       <c r="L8" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -5083,10 +5083,10 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>• PUK kodunun nereden öğrenileceği; 
-  • PIN değiştirme ve kaldırma; 
-  • üç kez yanlış PIN girildiğinde izlenecek yol; 
-  • SIM blokesinin kaldırılması.</t>
+          <t>1. PUK kodunun nereden öğrenileceği açıklanır
+2. PIN değiştirme ve kaldırma adım adım anlatılır
+3. Üç kez yanlış PIN girildiğinde izlenecek yol açıklanır
+4. SIM blokesinin kaldırılması adım adım anlatılır</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
@@ -5118,7 +5118,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="115" customHeight="1">
+    <row r="9" ht="128.5" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Ekran Yansıtma: Telefondan Televizyona Görüntü Aktarma</t>
@@ -5179,9 +5179,9 @@
       <c r="L9" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -5207,10 +5207,10 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>• Kablosuz yansıtma için gereken koşullar; 
-  • iPhone ve Android adımları; 
-  • kablo ile yansıtma; 
-  • televizyon bulunamadığında kontrol listesi.</t>
+          <t>1. Kablosuz yansıtma için gereken koşullar açıklanır
+2. IPhone ve Android adımları adım adım anlatılır
+3. Kablo ile yansıtma adım adım anlatılır
+4. Televizyon bulunamadığında kontrol listesi verilir</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
@@ -5301,10 +5301,10 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-2. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu</t>
+          <t>1. mac adresi nedir : https://www.turkcell.com.tr/blog/mac-adresi-her-cihazin-kendine-ozgu-dijital-imzasi
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
@@ -5330,10 +5330,10 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>• IP adresinin ne olduğu; 
-  • kendi IP adresini öğrenme; 
-  • statik ve dinamik IP farkı; 
-  • IP adresi değiştirme yolları ve sınırları.</t>
+          <t>1. IP adresinin ne olduğu açıklanır
+2. Kendi IP adresini öğrenme adım adım anlatılır
+3. Statik ve dinamik IP farkı açıklanır
+4. IP adresi değiştirme yolları ve sınırları açıklanır</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
@@ -5365,7 +5365,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="115" customHeight="1">
+    <row r="11" ht="128.5" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>İndirilenler Klasörü: Telefonda ve Bilgisayarda Dosya Bulma</t>
@@ -5425,10 +5425,10 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
-2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+          <t>1. wifi direct nedir : https://www.turkcell.com.tr/blog/wi-fi-direct-ile-dosya-paylasimi
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. ftp nedir : https://www.turkcell.com.tr/blog/ftp-nedir-dosya-transfer-protokolunun-temel-prensipleri
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -5454,10 +5454,10 @@
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>• Android ve iPhone'da indirilenler klasörünün yeri; 
-  • tarayıcıya göre değişen konumlar; 
-  • indirilen dosyanın bulunamaması durumu; 
-  • depolama temizliği.</t>
+          <t>1. Android ve iPhone'da indirilenler klasörünün yeri açıklanır
+2. Tarayıcıya göre değişen konumlar açıklanır
+3. Indirilen dosyanın bulunamaması durumu açıklanır
+4. Depolama temizliği açıklanır</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -5489,7 +5489,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="115" customHeight="1">
+    <row r="12" ht="128.5" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Instagram Hesabı: Dondurma, Giriş Sorunları ve Açılmama Nedenleri</t>
@@ -5551,9 +5551,9 @@
       <c r="L12" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
@@ -5596,11 +5596,11 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>• Hesabı geçici dondurma adımları ve kalıcı silmeden farkı; 
-  • dondurulan hesabın geri açılması; 
-  • uygulama açılmadığında kontrol listesi; 
-  • giriş yapılamadığında doğrulama adımları; 
-  • gönderilen takip isteklerinin görülmesi.</t>
+          <t>1. Hesabı geçici dondurma adımları ve kalıcı silmeden farkı açıklanır
+2. Dondurulan hesabın geri açılması adım adım anlatılır
+3. Uygulama açılmadığında kontrol listesi verilir
+4. Giriş yapılamadığında doğrulama adımları adım adım anlatılır
+5. Gönderilen takip isteklerinin görülmesi adım adım anlatılır</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
@@ -5632,7 +5632,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="115" customHeight="1">
+    <row r="13" ht="128.5" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Spam Ne Demek? Spam Mesaj ve Aramaları Engelleme</t>
@@ -5687,10 +5687,10 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>1. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
-2. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-3. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir
-4. wlan nedir : https://www.turkcell.com.tr/blog/wlan-nedir-kablosuz-aglarin-calisma-mantigi-ve-guvenlik-rehberi</t>
+          <t>1. phishing nedir : https://www.turkcell.com.tr/blog/bu-mesaj-tuzak-olabilir-phishing-nedir-ve-nasil-anlasilir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -5716,9 +5716,9 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>• Spam tanımı; 
-  • spam mesaj ve arama engelleme adımları; 
-  • operatör tarafındaki engelleme servisleri.</t>
+          <t>1. Spam tanımı açıklanır
+2. Spam mesaj ve arama engelleme adımları adım adım anlatılır
+3. Operatör tarafındaki engelleme servisleri açıklanır</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -5750,7 +5750,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="115" customHeight="1">
+    <row r="14" ht="128.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>SSD, RAM ve Ekran Kartı: Bilgisayar Donanımı Rehberi</t>
@@ -5811,10 +5811,10 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>1. kotlin nedir kotlin : https://www.turkcell.com.tr/blog/kotlin-nedir-kotlin-ne-ise-yarar
-2. turkcell hosting : https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. iss : https://www.turkcell.com.tr/blog/iss-internet-servis-saglayicisi-nedir-ne-ise-yarar</t>
+          <t>1. kuantum bilgisayar : https://www.turkcell.com.tr/blog/kuantum-bilgisayar-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -5840,11 +5840,11 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>• SSD ile HDD farkı; 
-  • RAM'in görevi ve yeterli kapasite; 
-  • ekran kartının ne işe yaradığı; 
-  • anakartın rolü; 
-  • bilgisayar yavaşladığında hangi bileşene bakılacağı.</t>
+          <t>1. SSD ile HDD farkı açıklanır
+2. RAM'in görevi ve yeterli kapasite açıklanır
+3. Ekran kartının ne işe yaradığı açıklanır
+4. Anakartın rolü açıklanır
+5. Bilgisayar yavaşladığında hangi bileşene bakılacağı açıklanır</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -5876,7 +5876,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="115" customHeight="1">
+    <row r="15" ht="128.5" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>E-İmza Nasıl Alınır?</t>
@@ -5931,9 +5931,9 @@
       <c r="L15" s="4" t="inlineStr">
         <is>
           <t>1. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-3. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir
-4. wlan nedir : https://www.turkcell.com.tr/blog/wlan-nedir-kablosuz-aglarin-calisma-mantigi-ve-guvenlik-rehberi</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
@@ -5959,9 +5959,9 @@
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>• E-imza tanımı; 
-  • başvuru adımları; 
-  • mobil imza ile farkı.</t>
+          <t>1. E-imza tanımı açıklanır
+2. Başvuru adımları adım adım anlatılır
+3. Mobil imza ile farkı açıklanır</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -6050,9 +6050,9 @@
       <c r="L16" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -6062,10 +6062,10 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>• Taahhüdün tanımı; 
-  • taahhütlü ve taahhütsüz farkı; 
-  • taahhüt süresi dolmadan çıkışta ne olduğu; 
-  • taahhüt süresinin öğrenilmesi.</t>
+          <t>1. Taahhüdün tanımı açıklanır
+2. Taahhütlü ve taahhütsüz farkı açıklanır
+3. Taahhüt süresi dolmadan çıkışta ne olduğu açıklanır
+4. Taahhüt süresinin öğrenilmesi adım adım anlatılır</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
@@ -6097,7 +6097,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="115" customHeight="1">
+    <row r="17" ht="128.5" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Konum Paylaşma ve Numaradan Konum Bulma</t>
@@ -6158,9 +6158,9 @@
       <c r="L17" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -6186,10 +6186,10 @@
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>• WhatsApp, Google Haritalar ve iMessage üzerinden konum paylaşma; 
-  • canlı konum paylaşımı süresi; 
-  • numaradan konum bulmanın gerçekte mümkün olup olmadığı; 
-  • konum servislerinin pil etkisi.</t>
+          <t>1. WhatsApp, Google Haritalar ve iMessage üzerinden konum paylaşma adım adım anlatılır
+2. Canlı konum paylaşımı süresi açıklanır
+3. Numaradan konum bulmanın gerçekte mümkün olup olmadığı açıklanır
+4. Konum servislerinin pil etkisi açıklanır</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -6221,7 +6221,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="115" customHeight="1">
+    <row r="18" ht="128.5" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Telefondan Telefona Veri Aktarma: Android, iPhone ve Numara Taşıma</t>
@@ -6282,9 +6282,9 @@
       <c r="L18" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -6310,11 +6310,11 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>• Android'den iPhone'a aktarma; 
-  • iPhone'dan iPhone'a hızlı başlangıç; 
-  • Android'den Android'e aktarma; 
-  • WhatsApp geçmişinin taşınması; 
-  • aktarma sırasında sık karşılaşılan durumlar.</t>
+          <t>1. Android'den iPhone'a aktarma adım adım anlatılır
+2. IPhone'dan iPhone'a hızlı başlangıç açıklanır
+3. Android'den Android'e aktarma adım adım anlatılır
+4. WhatsApp geçmişinin taşınması adım adım anlatılır
+5. Aktarma sırasında sık karşılaşılan durumlar açıklanır</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
@@ -6346,7 +6346,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="115" customHeight="1">
+    <row r="19" ht="128.5" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Chrome Eklentisi Nasıl Eklenir ve Kaldırılır?</t>
@@ -6405,9 +6405,9 @@
       <c r="L19" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
@@ -6433,10 +6433,10 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>• Eklentinin Chrome Web Mağazası üzerinden eklenmesi; 
-  • eklentinin kaldırılması ve devre dışı bırakılması; 
-  • eklenti izinlerinin görülmesi; 
-  • güvenilir eklentinin nasıl ayırt edildiği.</t>
+          <t>1. Eklentinin Chrome Web Mağazası üzerinden eklenmesi adım adım anlatılır
+2. Eklentinin kaldırılması ve devre dışı bırakılması adım adım anlatılır
+3. Eklenti izinlerinin görülmesi adım adım anlatılır
+4. Güvenilir eklentinin nasıl ayırt edildiği açıklanır</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -6468,7 +6468,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="115" customHeight="1">
+    <row r="20" ht="142" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>E-Posta Kurulumu ve Yönetimi: Hesap Açma, Aktarma, Güvenlik</t>
@@ -6525,10 +6525,10 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
-2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+          <t>1. bulut bilişim teknolojisinin sunduğu avantajlardan : https://www.turkcell.com.tr/blog/bulut-teknolojisinin-sagladigi-guvenlik-avantajlari
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
@@ -6554,10 +6554,10 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>• E-posta adresi oluşturma adımları; 
-  • telefonda hesap kurulumu; 
-  • e-posta yazarken dikkat edilecekler; 
-  • iki adımlı doğrulama.</t>
+          <t>1. E-posta adresi oluşturma adımları adım adım anlatılır
+2. Telefonda hesap kurulumu adım adım anlatılır
+3. E-posta yazarken dikkat edilecekler açıklanır
+4. Iki adımlı doğrulama adım adım anlatılır</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
@@ -6589,7 +6589,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="115" customHeight="1">
+    <row r="21" ht="128.5" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Telefon Güncellemesi Nasıl Yapılır?</t>
@@ -6647,9 +6647,9 @@
       <c r="L21" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
@@ -6675,10 +6675,10 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>• Android ve iOS için güncelleme adımları; 
-  • güncelleme görünmüyorsa yapılabilecekler; 
-  • güncelleme öncesi yedekleme; 
-  • depolama alanı yetmediğinde izlenecek yol.</t>
+          <t>1. Android ve iOS için güncelleme adımları adım adım anlatılır
+2. Güncelleme görünmüyorsa yapılabilecekler açıklanır
+3. Güncelleme öncesi yedekleme adım adım anlatılır
+4. Depolama alanı yetmediğinde izlenecek yol açıklanır</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -6710,7 +6710,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="115" customHeight="1">
+    <row r="22" ht="128.5" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Ekran Görüntüsü Alma: Bilgisayar, Telefon ve Kısayollar</t>
@@ -6772,9 +6772,9 @@
       <c r="L22" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
-2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. kuantum bilgisayar : https://www.turkcell.com.tr/blog/kuantum-bilgisayar-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
@@ -6817,11 +6817,11 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>• Windows'ta üç yöntem: PrtScn, Windows+Shift+S, Ekran Alıntısı Aracı; 
-  • Mac kısayolları; 
-  • telefonda ekran görüntüsü alma; 
-  • kısayol tablosu; 
-  • görüntünün kaydedildiği klasör.</t>
+          <t>1. Windows'ta üç yöntem: PrtScn, Windows+Shift+S, Ekran Alıntısı Aracı açıklanır
+2. Mac kısayolları adım adım anlatılır
+3. Telefonda ekran görüntüsü alma adım adım anlatılır
+4. Kısayol tablosu verilir
+5. Görüntünün kaydedildiği klasör açıklanır</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -6910,9 +6910,9 @@
       <c r="L23" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
@@ -6938,10 +6938,10 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>• eSIM ile fiziksel SIM farkı; 
-  • eSIM destekleyen telefon listesi; 
-  • mevcut hattı eSIM'e taşıma adımları; 
-  • yurt dışında eSIM kullanımı.</t>
+          <t>1. ESIM ile fiziksel SIM farkı açıklanır
+2. ESIM destekleyen telefon listesi verilir
+3. Mevcut hattı eSIM'e taşıma adımları adım adım anlatılır
+4. Yurt dışında eSIM kullanımı açıklanır</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
@@ -6973,7 +6973,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="115" customHeight="1">
+    <row r="24" ht="128.5" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Telefon Nasıl Sıfırlanır?</t>
@@ -7030,9 +7030,9 @@
       <c r="L24" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -7042,10 +7042,10 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>• Sıfırlama öncesi yedekleme; 
-  • Android'de fabrika ayarlarına dönüş adımları; 
-  • iPhone'da sıfırlama adımları; 
-  • sıfırlama sonrası hesap doğrulama.</t>
+          <t>1. Sıfırlama öncesi yedekleme adım adım anlatılır
+2. Android'de fabrika ayarlarına dönüş adımları adım adım anlatılır
+3. IPhone'da sıfırlama adımları adım adım anlatılır
+4. Sıfırlama sonrası hesap doğrulama adım adım anlatılır</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
@@ -7077,7 +7077,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="115" customHeight="1">
+    <row r="25" ht="128.5" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Deepfake Nedir ve Nasıl Anlaşılır?</t>
@@ -7132,9 +7132,9 @@
       <c r="L25" s="4" t="inlineStr">
         <is>
           <t>1. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
-3. ai agent nedir : https://www.turkcell.com.tr/blog/yapay-zeka-ajani-ai-agent-nedir-nasil-calisir
-4. yapay zeka : https://www.turkcell.com.tr/blog/yapay-zeka-cagi-nasil-calisir-hayati-nasil-donusturur</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -7160,9 +7160,9 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>• Deepfake tanımı; 
-  • sahte içeriğin anlaşılma yolları; 
-  • dolandırıcılık senaryoları.</t>
+          <t>1. Deepfake tanımı açıklanır
+2. Sahte içeriğin anlaşılma yolları adım adım anlatılır
+3. Dolandırıcılık senaryoları açıklanır</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -7194,7 +7194,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="115" customHeight="1">
+    <row r="26" ht="128.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Yenilenmiş Telefon: Garanti, Kalite Sınıfları ve Satın Alma</t>
@@ -7252,9 +7252,9 @@
       <c r="L26" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
@@ -7280,10 +7280,10 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>• Yenilenmiş telefon tanımı ve yasal çerçeve; 
-  • kalite sınıfları; 
-  • garanti süresi ve kapsamı; 
-  • satın almadan önce kontrol listesi.</t>
+          <t>1. Yenilenmiş telefon tanımı ve yasal çerçeve açıklanır
+2. Kalite sınıfları açıklanır
+3. Garanti süresi ve kapsamı açıklanır
+4. Satın almadan önce kontrol listesi verilir</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
@@ -7315,7 +7315,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="115" customHeight="1">
+    <row r="27" ht="128.5" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>AirTag Nedir ve Nasıl Kullanılır?</t>
@@ -7370,10 +7370,10 @@
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>1. kotlin nedir kotlin : https://www.turkcell.com.tr/blog/kotlin-nedir-kotlin-ne-ise-yarar
-2. turkcell hosting : https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. iss : https://www.turkcell.com.tr/blog/iss-internet-servis-saglayicisi-nedir-ne-ise-yarar</t>
+          <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
@@ -7399,9 +7399,9 @@
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>• AirTag tanımı ve çalışma mantığı; 
-  • kurulum adımları; 
-  • takip edilme uyarısı ve gizlilik.</t>
+          <t>1. AirTag tanımı ve çalışma mantığı açıklanır
+2. Kurulum adımları adım adım anlatılır
+3. Takip edilme uyarısı ve gizlilik açıklanır</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="115" customHeight="1">
+    <row r="28" ht="128.5" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>OEM Ne Demek?</t>
@@ -7488,9 +7488,9 @@
       <c r="L28" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
@@ -7516,9 +7516,9 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>• OEM tanımı; 
-  • OEM ürün ile orijinal ürün farkı; 
-  • telefon ve donanımda OEM kullanımı.</t>
+          <t>1. OEM tanımı açıklanır
+2. OEM ürün ile orijinal ürün farkı açıklanır
+3. Telefon ve donanımda OEM kullanımı açıklanır</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
@@ -7550,7 +7550,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="115" customHeight="1">
+    <row r="29" ht="128.5" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>KVKK Nedir? Kişisel Verilerin Korunması Kanunu</t>
@@ -7605,9 +7605,9 @@
       <c r="L29" s="4" t="inlineStr">
         <is>
           <t>1. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-3. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir
-4. wlan nedir : https://www.turkcell.com.tr/blog/wlan-nedir-kablosuz-aglarin-calisma-mantigi-ve-guvenlik-rehberi</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -7633,9 +7633,9 @@
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>• KVKK tanımı; 
-  • kişisel veri türleri; 
-  • veri sahibinin hakları.</t>
+          <t>1. KVKK tanımı açıklanır
+2. Kişisel veri türleri açıklanır
+3. Veri sahibinin hakları açıklanır</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
@@ -7667,7 +7667,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="115" customHeight="1">
+    <row r="30" ht="128.5" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Telefon Neden Isınır?</t>
@@ -7727,9 +7727,9 @@
       <c r="L30" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
-2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. turkcell b2b : https://www.turkcell.com.tr/blog/b2b-telco-sektorunde-urun-oneri-sistemleri-cok-katmanli-bir-yaklasim
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
@@ -7772,10 +7772,10 @@
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>• Isınmanın yaygın nedenleri; 
-  • şarj sırasında ısınma; 
-  • ısınmayı azaltan ayarlar; 
-  • servise götürmeyi gerektiren durumlar.</t>
+          <t>1. Isınmanın yaygın nedenleri açıklanır
+2. Şarj sırasında ısınma adım adım anlatılır
+3. Isınmayı azaltan ayarlar açıklanır
+4. Servise götürmeyi gerektiren durumlar açıklanır</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
@@ -7862,9 +7862,9 @@
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
@@ -7874,9 +7874,9 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>• Müşteri numarasının tanımı; 
-  • faturada ve uygulamada nereden görüldüğü; 
-  • abone numarası ile farkı.</t>
+          <t>1. Müşteri numarasının tanımı açıklanır
+2. Faturada ve uygulamada nereden görüldüğü açıklanır
+3. Abone numarası ile farkı açıklanır</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
@@ -7908,7 +7908,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="115" customHeight="1">
+    <row r="32" ht="128.5" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>OTP Ne Demek?</t>
@@ -7964,9 +7964,9 @@
       <c r="L32" s="4" t="inlineStr">
         <is>
           <t>1. claude ai : https://www.turkcell.com.tr/blog/claude-ai-anthropicin-guvenlik-merkezli-yapay-zeka-modeli
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-3. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir
-4. wlan nedir : https://www.turkcell.com.tr/blog/wlan-nedir-kablosuz-aglarin-calisma-mantigi-ve-guvenlik-rehberi</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
@@ -7976,10 +7976,10 @@
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>• OTP tanımı; 
-  • SMS ile gelen tek kullanımlık şifrenin nasıl çalıştığı; 
-  • OTP paylaşımının riskleri; 
-  • OTP gelmediğinde yapılabilecekler.</t>
+          <t>1. OTP tanımı açıklanır
+2. SMS ile gelen tek kullanımlık şifrenin nasıl çalıştığı açıklanır
+3. OTP paylaşımının riskleri açıklanır
+4. OTP gelmediğinde yapılabilecekler açıklanır</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
@@ -8011,7 +8011,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="115" customHeight="1">
+    <row r="33" ht="128.5" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>QLED Nedir? QLED ve OLED Farkı</t>
@@ -8067,9 +8067,9 @@
       <c r="L33" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
@@ -8079,10 +8079,10 @@
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>• QLED tanımı; 
-  • QLED ve OLED farkı tablo hâlinde; 
-  • hangi kullanım için hangisi; 
-  • parlaklık ve ömür karşılaştırması.</t>
+          <t>1. QLED tanımı açıklanır
+2. QLED ve OLED farkı tablo hâlinde açıklanır
+3. Hangi kullanım için hangisi açıklanır
+4. Parlaklık ve ömür karşılaştırması verilir</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
@@ -8114,7 +8114,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="128.5" customHeight="1">
+    <row r="34" ht="142" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Medya Okuryazarlığı Nedir?</t>
@@ -8170,9 +8170,9 @@
       <c r="L34" s="4" t="inlineStr">
         <is>
           <t>1. güneş enerjisi : https://www.turkcell.com.tr/blog/gunes-enerjisi-nedir-surdurulebilir-gelecegin-enerji-modeli-ve-uygulama-alanlari
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. sürdürülebilirlik nedir : https://www.turkcell.com.tr/blog/bugunu-yasarken-yarini-korumak-surdurulebilirlik-nedir
-3. karbon ayak izi : https://www.turkcell.com.tr/blog/dunyaya-biraktigimiz-iz-karbon-ayak-izi-nedir
-4. yeşil enerji nedir : https://www.turkcell.com.tr/blog/enerjinin-yeni-kodu-yesil-enerji-ile-gelecegi-yeniden-yazmak</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
@@ -8182,10 +8182,10 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>• Medya okuryazarlığının tanımı; 
-  • yanlış bilgiyi ayırt etme adımları; 
-  • kaynak doğrulama yöntemleri; 
-  • çocuklar için ipuçları.</t>
+          <t>1. Medya okuryazarlığının tanımı açıklanır
+2. Yanlış bilgiyi ayırt etme adımları adım adım anlatılır
+3. Kaynak doğrulama yöntemleri açıklanır
+4. Çocuklar için ipuçları açıklanır</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
@@ -8217,7 +8217,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="115" customHeight="1">
+    <row r="35" ht="128.5" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>TAG Nedir?</t>
@@ -8269,9 +8269,9 @@
       <c r="L35" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -8281,10 +8281,10 @@
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>• TAG teriminin anlamı; 
-  • sosyal medyada etiketleme; 
-  • NFC etiketi anlamı; 
-  • hangi bağlamda hangi anlamın kullanıldığı.</t>
+          <t>1. TAG teriminin anlamı açıklanır
+2. Sosyal medyada etiketleme adım adım anlatılır
+3. NFC etiketi anlamı açıklanır
+4. Hangi bağlamda hangi anlamın kullanıldığı açıklanır</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
@@ -8316,7 +8316,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="115" customHeight="1">
+    <row r="36" ht="128.5" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Karekod Nasıl Okutulur?</t>
@@ -8367,9 +8367,9 @@
       <c r="L36" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
@@ -8395,9 +8395,9 @@
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>• Kamerayla karekod okutma adımları; 
-  • kamera okutmadığında yapılabilecekler; 
-  • sahte karekodların ayırt edilmesi.</t>
+          <t>1. Kamerayla karekod okutma adımları adım adım anlatılır
+2. Kamera okutmadığında yapılabilecekler açıklanır
+3. Sahte karekodların ayırt edilmesi adım adım anlatılır</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
@@ -8429,7 +8429,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="115" customHeight="1">
+    <row r="37" ht="128.5" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Apple Arcade Nedir?</t>
@@ -8485,9 +8485,9 @@
       <c r="L37" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -8497,10 +8497,10 @@
       </c>
       <c r="N37" s="4" t="inlineStr">
         <is>
-          <t>• Apple Arcade tanımı; 
-  • abonelik ücreti ve deneme süresi; 
-  • hangi cihazlarda çalıştığı; 
-  • oyunların çevrimdışı oynanabilirliği.</t>
+          <t>1. Apple Arcade tanımı açıklanır
+2. Abonelik ücreti ve deneme süresi açıklanır
+3. Hangi cihazlarda çalıştığı açıklanır
+4. Oyunların çevrimdışı oynanabilirliği açıklanır</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
@@ -8587,10 +8587,10 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-2. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
-3. turkcell 5g : https://www.turkcell.com.tr/blog/5g-ile-hayatimiza-yeni-neler-giriyor-etkilesim-cagi-ve-fwa
-4. turkcell rahat paket nedir : https://www.turkcell.com.tr/blog/turkcell-rahat-paketleri-hem-faturali-hem-faturasiz-taahhutsuz-ozgurluk</t>
+          <t>1. hat resetleme nedir : https://www.turkcell.com.tr/blog/hat-resetleme-nedir-ne-zaman-ve-nasil-yapilir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
@@ -8600,10 +8600,10 @@
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>• Hat devrinin tanımı; 
-  • devir için gereken belgeler; 
-  • devir ücreti; 
-  • devir sonrası fatura ve taahhüt durumu.</t>
+          <t>1. Hat devrinin tanımı açıklanır
+2. Devir için gereken belgeler açıklanır
+3. Devir ücreti açıklanır
+4. Devir sonrası fatura ve taahhüt durumu açıklanır</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
@@ -8635,7 +8635,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="115" customHeight="1">
+    <row r="39" ht="128.5" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>URL Nedir?</t>
@@ -8686,9 +8686,9 @@
       <c r="L39" s="4" t="inlineStr">
         <is>
           <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
 2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-3. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir
-4. bulut depolama : https://www.turkcell.com.tr/blog/dijital-hafizanin-yeni-evi-bulut-depolama</t>
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
@@ -8698,9 +8698,9 @@
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>• URL tanımı; 
-  • URL bölümleri: protokol, alan adı, yol; 
-  • güvenli URL'nin nasıl anlaşıldığı.</t>
+          <t>1. URL tanımı açıklanır
+2. URL bölümleri: protokol, alan adı, yol açıklanır
+3. Güvenli URL'nin nasıl anlaşıldığı açıklanır</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -8732,7 +8732,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="115" customHeight="1">
+    <row r="40" ht="128.5" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>FreeDOS Nedir? İşletim Sistemi Yüklü Olmayan Bilgisayar</t>
@@ -8782,10 +8782,10 @@
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
-2. telefon kendi kendine kapanıyor : https://www.turkcell.com.tr/blog/telefonun-kendi-kendine-acilip-kapanmasi-neden-olur
-3. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
-4. virüs temizleme : https://www.turkcell.com.tr/blog/akilli-cihazlarda-virus-nasil-temizlenir</t>
+          <t>1. kuantum bilgisayar : https://www.turkcell.com.tr/blog/kuantum-bilgisayar-nedir
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.
+2. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Yazı planında karşılığı bulunmamaktadır; konuya değinen bir cümle eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -8811,9 +8811,9 @@
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>• FreeDOS tanımı; 
-  • işletim sistemi yüklü olmayan bilgisayarın anlamı; 
-  • sonrasında yapılabilecekler.</t>
+          <t>1. FreeDOS tanımı açıklanır
+2. Işletim sistemi yüklü olmayan bilgisayarın anlamı açıklanır
+3. Sonrasında yapılabilecekler açıklanır</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
@@ -9353,7 +9353,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="128.5" customHeight="1">
+    <row r="4" ht="142" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/isletim-sistemi-nedir-ve-cesitleri-nelerdir</t>
@@ -9458,10 +9458,10 @@
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>1. inovasyon örnekleri : https://www.turkcell.com.tr/blog/inovasyon-nedir-inovasyon-cesitleri-ve-ornekleri-nelerdir
-2. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
-3. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
-4. cloud gaming : https://www.turkcell.com.tr/blog/oyunlar-artik-bulutta-cloud-gaming-nedir-nasil-calisir</t>
+          <t>1. gemini : https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V4" s="4" t="inlineStr">
@@ -9487,9 +9487,9 @@
       </c>
       <c r="W4" s="4" t="inlineStr">
         <is>
-          <t>• Mobil işletim sistemleri bölümü genişletilebilir; 
-  • Windows, macOS ve Linux karşılaştırması tablo hâlinde verilebilir; 
-  • FreeDOS ve işletim sistemsiz cihaz bölümü eklenebilir.</t>
+          <t>1. Mobil işletim sistemleri bölümü genişletilebilir
+2. Windows, macOS ve Linux karşılaştırması tablo hâlinde verilebilir
+3. FreeDOS ve işletim sistemsiz cihaz bölümü eklenebilir</t>
         </is>
       </c>
       <c r="X4" s="4" t="inlineStr">
@@ -9514,7 +9514,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="115" customHeight="1">
+    <row r="5" ht="128.5" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar</t>
@@ -9624,10 +9624,10 @@
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>1. kotlin nedir kotlin : https://www.turkcell.com.tr/blog/kotlin-nedir-kotlin-ne-ise-yarar
-2. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-3. iss : https://www.turkcell.com.tr/blog/iss-internet-servis-saglayicisi-nedir-ne-ise-yarar
-4. turkcell hotspot : https://www.turkcell.com.tr/blog/hotspot-ile-internet-paylasimi-ne-ise-yarar-nasil-acilir</t>
+          <t>1. domain nedir : https://www.turkcell.com.tr/blog/dijital-varligin-ilk-adimi-domain-alan-adi-nedir
+   Anchor metni gövdede 8 kez geçmektedir; mevcut cümlelerden birine bağlantı verilebilir.
+2. chatgpt atlas : https://www.turkcell.com.tr/blog/ai-destekli-web-tarayici-donemi-chatgpt-atlas-nedir
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
@@ -9653,9 +9653,9 @@
       </c>
       <c r="W5" s="4" t="inlineStr">
         <is>
-          <t>• Hosting türleri karşılaştırması eklenebilir; 
-  • domain ile ilişkisi açıklanabilir; 
-  • küçük işletme için seçim kriterleri bölümü eklenebilir.</t>
+          <t>1. Hosting türleri karşılaştırması eklenebilir
+2. Domain ile ilişkisi açıklanabilir
+3. Küçük işletme için seçim kriterleri bölümü eklenebilir</t>
         </is>
       </c>
       <c r="X5" s="4" t="inlineStr">
@@ -9801,10 +9801,10 @@
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>1. kotlin nedir kotlin : https://www.turkcell.com.tr/blog/kotlin-nedir-kotlin-ne-ise-yarar
-2. turkcell hotspot : https://www.turkcell.com.tr/blog/hotspot-ile-internet-paylasimi-ne-ise-yarar-nasil-acilir
-3. turkcell hosting : https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar
-4. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi</t>
+          <t>1. turkcell hotspot : https://www.turkcell.com.tr/blog/hotspot-ile-internet-paylasimi-ne-ise-yarar-nasil-acilir
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
@@ -9864,11 +9864,11 @@
       </c>
       <c r="W6" s="4" t="inlineStr">
         <is>
-          <t>• NFC özelliğinin telefonda nasıl açıldığı marka bazında eklenebilir; 
-  • iPhone ve Android ayrımı ara başlığa çıkarılabilir; 
-  • NFC destekleyen telefon listesi eklenebilir; 
-  • temassız ödeme bölümü genişletilebilir; 
-  • NFC etiketi kullanımı eklenebilir.</t>
+          <t>1. NFC özelliğinin telefonda nasıl açıldığı marka bazında eklenebilir
+2. IPhone ve Android ayrımı ara başlığa çıkarılabilir
+3. NFC destekleyen telefon listesi eklenebilir
+4. Temassız ödeme bölümü genişletilebilir
+5. NFC etiketi kullanımı eklenebilir</t>
         </is>
       </c>
       <c r="X6" s="4" t="inlineStr">
@@ -9893,7 +9893,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="209.5" customHeight="1">
+    <row r="7" ht="263.5" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis</t>
@@ -9993,9 +9993,13 @@
       <c r="U7" s="4" t="inlineStr">
         <is>
           <t>1. yapay zeka mühendisliği : https://www.turkcell.com.tr/blog/yapay-zeka-muhendisligi-nedir
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
 2. creen ai : https://www.turkcell.com.tr/blog/yesil-yapay-zeka-green-ai
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
 3. yapay zeka sanatçısı ne demek : https://www.turkcell.com.tr/blog/yapay-zeka-sanat-yapabilir-mi
-4. yapay zeka kullanirken : https://www.turkcell.com.tr/blog/yapay-zeka-kullanirken-ne-kadarini-paylasmaliyiz</t>
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+4. ai agent nedir : https://www.turkcell.com.tr/blog/yapay-zeka-ajani-ai-agent-nedir-nasil-calisir
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V7" s="4" t="inlineStr">
@@ -10005,11 +10009,11 @@
       </c>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t>• Yazının hedefi çıplak marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek'; 
-  • kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma; 
-  • ChatGPT ile karşılaştırma tablosu eklenebilir; 
-  • ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir; 
-  • sık sorulanlar bölümü, sonuç sayfasında görünen soru bloğuyla eşleştirilebilir.</t>
+          <t>1. Yazının hedefi çıplak marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek' açıklanır
+2. Kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma adım adım anlatılır
+3. ChatGPT ile karşılaştırma tablosu eklenebilir
+4. Ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir
+5. Sık sorulanlar bölümü, sonuç sayfasında görünen soru bloğuyla eşleştirilebilir</t>
         </is>
       </c>
       <c r="X7" s="4" t="inlineStr">
@@ -10034,7 +10038,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="128.5" customHeight="1">
+    <row r="8" ht="142" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/ping-internette-gecikmenin-gercek-nedeni</t>
@@ -10133,10 +10137,10 @@
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-2. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu</t>
+          <t>1. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. superbox ping düşürme : https://www.turkcell.com.tr/blog/5g-ve-ping-5g-ile-oyunlarda-ping-dusurme-yollari-ve-cozumler
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V8" s="4" t="inlineStr">
@@ -10179,9 +10183,9 @@
       </c>
       <c r="W8" s="4" t="inlineStr">
         <is>
-          <t>• Ping değerinin ne olduğu ve ideal aralık tablo hâlinde verilebilir; 
-  • ping düşürme adımları eklenebilir; 
-  • oyun senaryosu ayrı ara başlığa alınabilir.</t>
+          <t>1. Ping değerinin ne olduğu ve ideal aralık tablo hâlinde verilebilir
+2. Ping düşürme adımları eklenebilir
+3. Oyun senaryosu ayrı ara başlığa alınabilir</t>
         </is>
       </c>
       <c r="X8" s="4" t="inlineStr">
@@ -10336,10 +10340,10 @@
       </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>1. kotlin nedir kotlin : https://www.turkcell.com.tr/blog/kotlin-nedir-kotlin-ne-ise-yarar
-2. turkcell hosting : https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. iss : https://www.turkcell.com.tr/blog/iss-internet-servis-saglayicisi-nedir-ne-ise-yarar</t>
+          <t>1. tethering nedir : https://www.turkcell.com.tr/blog/tethering-nedir-usb-wi-fi-ve-bluetooth-ile-internet-paylasimi-rehberi
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V9" s="4" t="inlineStr">
@@ -10365,9 +10369,9 @@
       </c>
       <c r="W9" s="4" t="inlineStr">
         <is>
-          <t>• Kablo ve şarj aleti seçimi bölümü eklenebilir; 
-  • USB-C standartları ve hız sınıfları tablo hâlinde verilebilir; 
-  • hangi cihazlarda bulunduğu listelenebilir.</t>
+          <t>1. Kablo ve şarj aleti seçimi bölümü eklenebilir
+2. USB-C standartları ve hız sınıfları tablo hâlinde verilebilir
+3. Hangi cihazlarda bulunduğu listelenebilir</t>
         </is>
       </c>
       <c r="X9" s="4" t="inlineStr">
@@ -10500,9 +10504,9 @@
       <c r="U10" s="4" t="inlineStr">
         <is>
           <t>1. sabit internet nedir : https://www.turkcell.com.tr/blog/sabit-internet-nedir-turleri-avantajlari-ve-kullanim-alanlari
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
 2. internet üzerinden erisim : https://www.turkcell.com.tr/blog/uzaktan-baglanti-nedir-turleri-calisma-mantigi-ve-guvenli-kullanim-rehberi
-3. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-4. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi</t>
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr">
@@ -10579,10 +10583,10 @@
       </c>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t>• Hangi bağlantının hangi kullanım için uygun olduğu tablo hâlinde verilebilir; 
-  • hız beklentisi mesafeye göre açıklanabilir; 
-  • altyapı sorgulamaya bağlantı eklenebilir; 
-  • fiber karşılaştırması genişletilebilir.</t>
+          <t>1. Hangi bağlantının hangi kullanım için uygun olduğu tablo hâlinde verilebilir
+2. Hız beklentisi mesafeye göre açıklanabilir
+3. Altyapı sorgulamaya bağlantı eklenebilir
+4. Fiber karşılaştırması genişletilebilir</t>
         </is>
       </c>
       <c r="X10" s="4" t="inlineStr">
@@ -10720,9 +10724,9 @@
       <c r="U11" s="4" t="inlineStr">
         <is>
           <t>1. ping : https://www.turkcell.com.tr/blog/ping-internette-gecikmenin-gercek-nedeni
-2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-3. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-4. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi</t>
+   Anchor metni gövdede 1 kez geçmektedir; mevcut cümlelerden birine bağlantı verilebilir.
+2. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V11" s="4" t="inlineStr">
@@ -10748,9 +10752,9 @@
       </c>
       <c r="W11" s="4" t="inlineStr">
         <is>
-          <t>• İdeal jitter değeri tablo hâlinde verilebilir; 
-  • ölçüm yöntemi eklenebilir; 
-  • paket kaybı ile ilişkisi açıklanabilir.</t>
+          <t>1. İdeal jitter değeri tablo hâlinde verilebilir
+2. Ölçüm yöntemi eklenebilir
+3. Paket kaybı ile ilişkisi açıklanabilir</t>
         </is>
       </c>
       <c r="X11" s="4" t="inlineStr">
@@ -10775,7 +10779,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="128.5" customHeight="1">
+    <row r="12" ht="142" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/wi-fi-6-nedir-wi-fi-5-ile-arasindaki-temel-farklar</t>
@@ -10881,10 +10885,10 @@
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>1. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-2. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-3. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi
-4. proxy : https://www.turkcell.com.tr/blog/proxy-nedir-internette-gizlilik-erisim-ve-guvenlik-uzerindeki-rolu</t>
+          <t>1. 4.5 g ile 5g arasındaki : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. vdsl internet : https://www.turkcell.com.tr/blog/vdsl-ve-adsl-nedir-internet-baglanti-turleri-arasindaki-farklar
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V12" s="4" t="inlineStr">
@@ -10918,9 +10922,9 @@
       </c>
       <c r="W12" s="4" t="inlineStr">
         <is>
-          <t>• Wi-Fi 6 destekleyen modem listesi eklenebilir; 
-  • mesh sistemlerle ilişkisi açıklanabilir; 
-  • yükseltmenin ne zaman anlamlı olduğu bölümü eklenebilir.</t>
+          <t>1. Wi-Fi 6 destekleyen modem listesi eklenebilir
+2. Mesh sistemlerle ilişkisi açıklanabilir
+3. Yükseltmenin ne zaman anlamlı olduğu bölümü eklenebilir</t>
         </is>
       </c>
       <c r="X12" s="4" t="inlineStr">
@@ -10945,7 +10949,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="142" customHeight="1">
+    <row r="13" ht="155.5" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/mac-adresi-her-cihazin-kendine-ozgu-dijital-imzasi</t>
@@ -11056,9 +11060,9 @@
       <c r="U13" s="4" t="inlineStr">
         <is>
           <t>1. kaybolan telefon nasıl bulunur : https://www.turkcell.com.tr/blog/telefonum-nerede-kayip-ve-kapali-telefon-nasil-bulunur
-2. hotspot nedir : https://www.turkcell.com.tr/blog/hotspot-internet-paketi-nedir
-3. 4.5 g ile 5g arasındaki hız farkı : https://www.turkcell.com.tr/blog/5g-ve-4g-arasindaki-farklar-sadece-hiz-mi-yoksa-yeni-bir-donem-mi
-4. vowifi nedir : https://www.turkcell.com.tr/blog/vowifi-nedir-ve-ne-ise-yarar-calisma-mantigi-ve-kullanimi</t>
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.
+2. internet yavaşladı : https://www.turkcell.com.tr/blog/internet-neden-yavasladi-sorunun-kaynagini-adim-adim-bulma-rehberi
+   Anchor metni gövdede geçmemektedir; konuya değinen bir cümle ya da alt başlık eklenirse bağlantı verilebilir.</t>
         </is>
       </c>
       <c r="V13" s="4" t="inlineStr">
@@ -11084,9 +11088,9 @@
       </c>
       <c r="W13" s="4" t="inlineStr">
         <is>
-          <t>• MAC adresinin cihazdan öğrenilmesi işletim sistemi bazında eklenebilir; 
-  • MAC filtreleme bölümü eklenebilir; 
-  • IP adresiyle farkı açıklanabilir.</t>
+          <t>1. MAC adresinin cihazdan öğrenilmesi işletim sistemi bazında eklenebilir
+2. MAC filtreleme bölümü eklenebilir
+3. IP adresiyle farkı açıklanabilir</t>
         </is>
       </c>
       <c r="X13" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Tablo görüntüleyici, sezonsallık renklendirmesi ve terim düzeltmesi
- Fikir-hacim tablosunda sütun genişliği içerikten hesaplanıyor, başlık
  kenarından sürüklenerek değiştirilebiliyor; kaydırma alanı yükseltildi
- Sezonsallık: öneri sütunu genişletildi, renklendirme satır içi kırmızı-sarı-
  yeşil skalaya çevrildi, hücreye ortalamaya göre fark eklendi, peak ayı
  çerçeveli; Excel'de aynı skala ve Peak İndeksi sütunu
- 'çıplak' terimi jenerik / yalın karşılıklarıyla değiştirildi
- Durum rozetinin hücreden taşması ve uzun sayaç rozeti giderildi

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,11 +87,23 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0010332F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="0010332F"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="195">
     <fill>
       <patternFill/>
     </fill>
@@ -120,22 +132,947 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
+        <fgColor rgb="00EA885F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00EC8E53"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
+        <fgColor rgb="00E88367"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEBEE"/>
+        <fgColor rgb="00EA875F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E88269"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98661"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E77F6E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E67C73"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0057BB8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2A132"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0097BB56"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC8D55"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9645"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8BC2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98464"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E77E6F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA8760"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98563"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E88466"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E88368"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8C57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7806D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE934B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE944A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98564"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D7BC21"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC8E54"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E77F6D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA885E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED914F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED9050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE9547"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A0BB4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0073BB74"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2A034"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8816A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E77E70"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9843"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98662"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA895D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC8E55"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F19C3B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9941"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2BC0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9744"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A924"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ABBC46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5AA23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1BC0D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBBC04"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F29F36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3A42D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09A3F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B5BC3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBBB06"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAB80B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAB80A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAB909"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2A134"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8B59"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FABA07"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B3BC3F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09A40"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE9646"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8816B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFBC28"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7B117"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B313"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9B50F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1BC19"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4A827"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9B60E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F19E38"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE9449"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4A62A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC8F51"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09B3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5AB22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8BC20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BABC39"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0076BB71"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8A5B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6AB21"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B314"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7806C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAB80C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B215"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B0BC41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F19E39"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8BC06"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8BC2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDBC1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9B510"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B411"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009CBB52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6AC20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6AE1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FABC05"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005BBB87"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0079BB6F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007DBB6B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBBC1E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFBC1B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BEBC36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3A330"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ABBC45"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCBC1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0086BB63"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0089BB61"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09C3C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EC8F52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EE9548"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A5BB4B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0BC1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BCBC38"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B412"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0069BB7C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4A729"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BEBC35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0BC27"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F19F37"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D2BC26"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A826"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09B3E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E67D71"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED914E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AFBC42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CBBC2B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6BC2F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1BC0C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007FBB6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7AF1B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3BC0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED924D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA895C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4A62B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8B216"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9646"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A2BB4D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0069BB7B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCBC2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEBC1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDBC0F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0094BB58"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6BC08"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A3BB4C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9BC12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4A52B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8C58"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0066BB7E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0072BB74"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008CBB5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7BC08"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7BC14"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2A133"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09A3E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7AF1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5BC09"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDBC10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBBB05"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3BC18"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0BC34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A1BB4D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF9842"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0080BB69"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0065BB7F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3BC0A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4BC16"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005CBB86"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0071BB75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0077BB70"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F09940"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006FBB76"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E98465"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006FBB77"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4BC09"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2A035"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8B58"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7816B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFBC0E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFBC35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0085BB64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0074BB72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F19F36"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4BC3E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8BC07"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0082BB67"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0063BB80"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EB8D56"/>
       </patternFill>
     </fill>
   </fills>
@@ -173,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -217,25 +1154,580 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="30" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="31" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="32" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="33" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="34" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="35" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="36" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="37" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="38" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="39" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="40" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="41" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="42" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="43" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="44" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="45" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="46" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="47" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="48" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="49" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="50" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="51" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="52" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="53" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="54" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="55" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="56" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="57" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="58" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="59" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="60" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="61" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="62" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="63" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="64" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="65" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="66" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="67" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="68" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="69" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="70" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="71" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="72" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="73" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="74" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="75" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="76" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="77" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="78" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="79" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="80" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="81" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="82" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="83" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="84" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="85" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="86" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="87" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="88" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="89" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="90" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="91" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="92" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="93" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="94" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="95" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="96" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="97" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="98" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="99" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="100" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="101" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="102" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="103" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="104" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="105" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="106" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="107" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="108" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="109" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="110" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="111" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="112" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="113" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="114" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="115" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="116" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="117" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="118" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="119" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="120" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="121" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="122" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="123" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="124" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="125" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="126" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="127" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="128" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="129" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="130" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="131" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="132" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="133" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="134" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="135" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="136" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="137" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="138" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="139" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="140" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="141" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="142" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="143" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="144" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="145" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="146" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="147" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="148" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="149" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="150" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="151" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="152" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="153" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="154" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="155" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="156" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="157" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="158" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="159" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="160" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="161" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="162" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="163" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="164" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="165" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="166" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="167" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="168" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="169" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="170" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="171" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="172" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="173" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="174" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="175" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="176" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="177" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="178" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="179" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="180" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="181" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="10" fillId="182" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="183" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="184" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="185" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="186" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="187" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="188" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="189" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="190" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="191" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="192" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="193" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="194" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1499,7 +2991,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Çıplak genel ad; tek bir arama niyeti taşımıyor.</t>
+          <t>Jenerik ad; tek bir arama niyeti taşımıyor.</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1521,7 +3013,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Çıplak genel ad; tek bir arama niyeti taşımıyor.</t>
+          <t>Jenerik ad; tek bir arama niyeti taşımıyor.</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1873,7 +3365,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Çıplak kısaltma; tek başına arama niyetini taşımıyor.</t>
+          <t>Jenerik kısaltma; tek başına arama niyetini taşımıyor.</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2137,7 +3629,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Çıplak kısaltma; tek başına arama niyetini taşımıyor.</t>
+          <t>Jenerik kısaltma; tek başına arama niyetini taşımıyor.</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2465,7 +3957,7 @@
       <c r="F68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="20" t="inlineStr">
+      <c r="A69" s="205" t="inlineStr">
         <is>
           <t>Öneri kümelerindeki değişim</t>
         </is>
@@ -2973,7 +4465,7 @@
       <c r="F88" s="2" t="n"/>
     </row>
     <row r="89" ht="34" customHeight="1">
-      <c r="A89" s="21" t="inlineStr">
+      <c r="A89" s="206" t="inlineStr">
         <is>
           <t>Çakışma ve cannibalization kontrolü</t>
         </is>
@@ -10072,7 +11564,7 @@
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>1. Yazının hedefi çıplak marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek'
+          <t>1. Yazının hedefi jenerik marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek'
 2. Kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma
 3. ChatGPT ile karşılaştırma tablosu eklenebilir
 4. Ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir
@@ -10099,7 +11591,7 @@
       </c>
       <c r="X7" s="4" t="inlineStr">
         <is>
-          <t>1. Yazının hedefi çıplak marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek' açıklanır
+          <t>1. Yazının hedefi jenerik marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek' açıklanır
 2. Kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma adım adım anlatılır
 3. ChatGPT ile karşılaştırma tablosu eklenebilir
 4. Ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir
@@ -10108,7 +11600,7 @@
       </c>
       <c r="Y7" s="4" t="inlineStr">
         <is>
-          <t>Yazının impression'ı çıplak marka aramasından gelmektedir ve bu aramada sonuç sayfasının üst sıraları Google'ın kendi mülkleridir; CTR'ın bu aramada yükselmesi beklenmemelidir. Kazanım uzun kuyruk sorularındadır.</t>
+          <t>Yazının impression'ı jenerik marka aramasından gelmektedir ve bu aramada sonuç sayfasının üst sıraları Google'ın kendi mülkleridir; CTR'ın bu aramada yükselmesi beklenmemelidir. Kazanım uzun kuyruk sorularındadır.</t>
         </is>
       </c>
       <c r="Z7" s="7" t="n">
@@ -10124,7 +11616,7 @@
       </c>
       <c r="AC7" s="4" t="inlineStr">
         <is>
-          <t>Yazı altı ayda 16.3 milyon impression alıp 2.125 click getirmiştir. Sorun içerikte değil, çıplak marka aramasının sonuç sayfasında: üst sıralar Google'ın kendi adreslerinde. Kazanım, kullanım ve karşılaştırma sorularında.</t>
+          <t>Yazı altı ayda 16.3 milyon impression alıp 2.125 click getirmiştir. Sorun içerikte değil, jenerik marka aramasının sonuç sayfasında: üst sıralar Google'ın kendi adreslerinde. Kazanım, kullanım ve karşılaştırma sorularında.</t>
         </is>
       </c>
     </row>
@@ -26883,10 +28375,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -26902,7 +28394,8 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -26927,6 +28420,7 @@
       <c r="O1" s="2" t="n"/>
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -26946,6 +28440,7 @@
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -27030,6 +28525,11 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Peak İndeksi</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>Önerilen Yayın Ayı</t>
         </is>
       </c>
@@ -27048,37 +28548,37 @@
       <c r="C4" s="15" t="n">
         <v>2490</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>3400</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="17" t="n">
         <v>1880</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="18" t="n">
         <v>2480</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="19" t="n">
         <v>1720</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="20" t="n">
         <v>2320</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="21" t="n">
         <v>1270</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="22" t="n">
         <v>910</v>
       </c>
-      <c r="K4" s="16" t="n">
+      <c r="K4" s="23" t="n">
         <v>18400</v>
       </c>
-      <c r="L4" s="17" t="n">
+      <c r="L4" s="24" t="n">
         <v>6000</v>
       </c>
-      <c r="M4" s="16" t="n">
+      <c r="M4" s="25" t="n">
         <v>15000</v>
       </c>
-      <c r="N4" s="15" t="n">
+      <c r="N4" s="26" t="n">
         <v>3280</v>
       </c>
       <c r="O4" s="8" t="inlineStr">
@@ -27089,13 +28589,16 @@
       <c r="P4" s="7" t="n">
         <v>18400</v>
       </c>
-      <c r="Q4" s="8" t="inlineStr">
+      <c r="Q4" s="8" t="n">
+        <v>373</v>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
         <is>
           <t>Temmuz</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Google Güvenli Arama: Açma, Kapatma ve Aile Filtresi</t>
@@ -27106,40 +28609,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="27" t="n">
         <v>121800</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="28" t="n">
         <v>283600</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="26" t="n">
         <v>96200</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="23" t="n">
         <v>408000</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="29" t="n">
         <v>71580</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="30" t="n">
         <v>53700</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="22" t="n">
         <v>47970</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="31" t="n">
         <v>78500</v>
       </c>
-      <c r="K5" s="15" t="n">
+      <c r="K5" s="32" t="n">
         <v>73800</v>
       </c>
-      <c r="L5" s="15" t="n">
+      <c r="L5" s="33" t="n">
         <v>69400</v>
       </c>
-      <c r="M5" s="15" t="n">
+      <c r="M5" s="34" t="n">
         <v>66600</v>
       </c>
-      <c r="N5" s="15" t="n">
+      <c r="N5" s="22" t="n">
         <v>48200</v>
       </c>
       <c r="O5" s="8" t="inlineStr">
@@ -27150,7 +28653,10 @@
       <c r="P5" s="7" t="n">
         <v>408000</v>
       </c>
-      <c r="Q5" s="8" t="inlineStr">
+      <c r="Q5" s="8" t="n">
+        <v>345</v>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
         <is>
           <t>Şubat</t>
         </is>
@@ -27167,40 +28673,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="35" t="n">
         <v>17100</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="36" t="n">
         <v>11900</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="37" t="n">
         <v>20100</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="38" t="n">
         <v>20400</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="39" t="n">
         <v>14100</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="23" t="n">
         <v>64400</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="40" t="n">
         <v>43280</v>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="J6" s="41" t="n">
         <v>18000</v>
       </c>
-      <c r="K6" s="15" t="n">
+      <c r="K6" s="26" t="n">
         <v>17700</v>
       </c>
-      <c r="L6" s="15" t="n">
+      <c r="L6" s="42" t="n">
         <v>11780</v>
       </c>
-      <c r="M6" s="15" t="n">
+      <c r="M6" s="22" t="n">
         <v>10400</v>
       </c>
-      <c r="N6" s="15" t="n">
+      <c r="N6" s="22" t="n">
         <v>10420</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
@@ -27211,7 +28717,10 @@
       <c r="P6" s="7" t="n">
         <v>64400</v>
       </c>
-      <c r="Q6" s="8" t="inlineStr">
+      <c r="Q6" s="8" t="n">
+        <v>298</v>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
         <is>
           <t>Nisan</t>
         </is>
@@ -27228,40 +28737,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="43" t="n">
         <v>4390</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="31" t="n">
         <v>4290</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="44" t="n">
         <v>5200</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="45" t="n">
         <v>5110</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="46" t="n">
         <v>5600</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="47" t="n">
         <v>12280</v>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I7" s="23" t="n">
         <v>14870</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="J7" s="48" t="n">
         <v>13900</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K7" s="49" t="n">
         <v>6570</v>
       </c>
-      <c r="L7" s="15" t="n">
+      <c r="L7" s="22" t="n">
         <v>3310</v>
       </c>
-      <c r="M7" s="15" t="n">
+      <c r="M7" s="50" t="n">
         <v>3780</v>
       </c>
-      <c r="N7" s="15" t="n">
+      <c r="N7" s="51" t="n">
         <v>3490</v>
       </c>
       <c r="O7" s="8" t="inlineStr">
@@ -27272,7 +28781,10 @@
       <c r="P7" s="7" t="n">
         <v>14870</v>
       </c>
-      <c r="Q7" s="8" t="inlineStr">
+      <c r="Q7" s="8" t="n">
+        <v>216</v>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
         <is>
           <t>Mayıs</t>
         </is>
@@ -27289,40 +28801,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="52" t="n">
         <v>25400</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="53" t="n">
         <v>20400</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="27" t="n">
         <v>25100</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="54" t="n">
         <v>21300</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="31" t="n">
         <v>20700</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>21000</v>
       </c>
-      <c r="I8" s="15" t="n">
+      <c r="I8" s="22" t="n">
         <v>17700</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="55" t="n">
         <v>22600</v>
       </c>
-      <c r="K8" s="7" t="n">
+      <c r="K8" s="56" t="n">
         <v>26700</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="L8" s="57" t="n">
         <v>25700</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="M8" s="57" t="n">
         <v>25700</v>
       </c>
-      <c r="N8" s="16" t="n">
+      <c r="N8" s="23" t="n">
         <v>53500</v>
       </c>
       <c r="O8" s="8" t="inlineStr">
@@ -27333,7 +28845,10 @@
       <c r="P8" s="7" t="n">
         <v>53500</v>
       </c>
-      <c r="Q8" s="8" t="inlineStr">
+      <c r="Q8" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
         <is>
           <t>Ekim</t>
         </is>
@@ -27350,40 +28865,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="58" t="n">
         <v>12100</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="59" t="n">
         <v>8100</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="43" t="n">
         <v>6600</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="43" t="n">
         <v>6600</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="22" t="n">
         <v>5400</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="43" t="n">
         <v>6600</v>
       </c>
-      <c r="I9" s="15" t="n">
+      <c r="I9" s="43" t="n">
         <v>6600</v>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="43" t="n">
         <v>6600</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="K9" s="60" t="n">
         <v>9900</v>
       </c>
-      <c r="L9" s="16" t="n">
+      <c r="L9" s="23" t="n">
         <v>18100</v>
       </c>
-      <c r="M9" s="16" t="n">
+      <c r="M9" s="58" t="n">
         <v>12100</v>
       </c>
-      <c r="N9" s="16" t="n">
+      <c r="N9" s="58" t="n">
         <v>12100</v>
       </c>
       <c r="O9" s="8" t="inlineStr">
@@ -27394,7 +28909,10 @@
       <c r="P9" s="7" t="n">
         <v>18100</v>
       </c>
-      <c r="Q9" s="8" t="inlineStr">
+      <c r="Q9" s="8" t="n">
+        <v>196</v>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
         <is>
           <t>Ağustos</t>
         </is>
@@ -27411,40 +28929,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="59" t="n">
         <v>2900</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="59" t="n">
         <v>2900</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="23" t="n">
         <v>6600</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="61" t="n">
         <v>5400</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="62" t="n">
         <v>3600</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="63" t="n">
         <v>4400</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I10" s="22" t="n">
         <v>1900</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="62" t="n">
         <v>3600</v>
       </c>
-      <c r="K10" s="15" t="n">
+      <c r="K10" s="59" t="n">
         <v>2900</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="L10" s="62" t="n">
         <v>3600</v>
       </c>
-      <c r="M10" s="7" t="n">
+      <c r="M10" s="62" t="n">
         <v>3600</v>
       </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="62" t="n">
         <v>3600</v>
       </c>
       <c r="O10" s="8" t="inlineStr">
@@ -27455,7 +28973,10 @@
       <c r="P10" s="7" t="n">
         <v>6600</v>
       </c>
-      <c r="Q10" s="8" t="inlineStr">
+      <c r="Q10" s="8" t="n">
+        <v>176</v>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
         <is>
           <t>Ocak</t>
         </is>
@@ -27472,40 +28993,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="64" t="n">
         <v>109080</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="65" t="n">
         <v>88700</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="66" t="n">
         <v>92300</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="67" t="n">
         <v>85100</v>
       </c>
-      <c r="G11" s="15" t="n">
+      <c r="G11" s="53" t="n">
         <v>70480</v>
       </c>
-      <c r="H11" s="15" t="n">
+      <c r="H11" s="27" t="n">
         <v>82460</v>
       </c>
-      <c r="I11" s="15" t="n">
+      <c r="I11" s="22" t="n">
         <v>63690</v>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="68" t="n">
         <v>128600</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="K11" s="23" t="n">
         <v>154600</v>
       </c>
-      <c r="L11" s="7" t="n">
+      <c r="L11" s="69" t="n">
         <v>108300</v>
       </c>
-      <c r="M11" s="7" t="n">
+      <c r="M11" s="70" t="n">
         <v>106200</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="71" t="n">
         <v>106600</v>
       </c>
       <c r="O11" s="8" t="inlineStr">
@@ -27516,7 +29037,10 @@
       <c r="P11" s="7" t="n">
         <v>154600</v>
       </c>
-      <c r="Q11" s="8" t="inlineStr">
+      <c r="Q11" s="8" t="n">
+        <v>155</v>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
         <is>
           <t>Temmuz</t>
         </is>
@@ -27533,40 +29057,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="72" t="n">
         <v>4400</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="72" t="n">
         <v>4400</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="72" t="n">
         <v>4400</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="73" t="n">
         <v>3600</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="73" t="n">
         <v>3600</v>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H12" s="74" t="n">
         <v>2900</v>
       </c>
-      <c r="I12" s="15" t="n">
+      <c r="I12" s="74" t="n">
         <v>2900</v>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J12" s="22" t="n">
         <v>2400</v>
       </c>
-      <c r="K12" s="16" t="n">
+      <c r="K12" s="68" t="n">
         <v>5400</v>
       </c>
-      <c r="L12" s="16" t="n">
+      <c r="L12" s="23" t="n">
         <v>6600</v>
       </c>
-      <c r="M12" s="16" t="n">
+      <c r="M12" s="68" t="n">
         <v>5400</v>
       </c>
-      <c r="N12" s="16" t="n">
+      <c r="N12" s="68" t="n">
         <v>5400</v>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -27577,7 +29101,10 @@
       <c r="P12" s="7" t="n">
         <v>6600</v>
       </c>
-      <c r="Q12" s="8" t="inlineStr">
+      <c r="Q12" s="8" t="n">
+        <v>154</v>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
         <is>
           <t>Ağustos</t>
         </is>
@@ -27594,40 +29121,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="75" t="n">
         <v>3600</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="75" t="n">
         <v>3600</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="73" t="n">
         <v>2900</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="16" t="n">
         <v>2400</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="22" t="n">
         <v>1900</v>
       </c>
-      <c r="H13" s="15" t="n">
+      <c r="H13" s="22" t="n">
         <v>1900</v>
       </c>
-      <c r="I13" s="15" t="n">
+      <c r="I13" s="22" t="n">
         <v>1900</v>
       </c>
-      <c r="J13" s="17" t="n">
+      <c r="J13" s="68" t="n">
         <v>4400</v>
       </c>
-      <c r="K13" s="16" t="n">
+      <c r="K13" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="L13" s="16" t="n">
+      <c r="L13" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="M13" s="16" t="n">
+      <c r="M13" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="N13" s="17" t="n">
+      <c r="N13" s="68" t="n">
         <v>4400</v>
       </c>
       <c r="O13" s="8" t="inlineStr">
@@ -27638,7 +29165,10 @@
       <c r="P13" s="7" t="n">
         <v>5400</v>
       </c>
-      <c r="Q13" s="8" t="inlineStr">
+      <c r="Q13" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
         <is>
           <t>Eylül</t>
         </is>
@@ -27655,40 +29185,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="76" t="n">
         <v>13180</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="77" t="n">
         <v>9300</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="46" t="n">
         <v>9020</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="78" t="n">
         <v>9060</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="79" t="n">
         <v>7760</v>
       </c>
-      <c r="H14" s="15" t="n">
+      <c r="H14" s="37" t="n">
         <v>8880</v>
       </c>
-      <c r="I14" s="15" t="n">
+      <c r="I14" s="22" t="n">
         <v>7460</v>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J14" s="23" t="n">
         <v>15400</v>
       </c>
-      <c r="K14" s="17" t="n">
+      <c r="K14" s="80" t="n">
         <v>12500</v>
       </c>
-      <c r="L14" s="7" t="n">
+      <c r="L14" s="81" t="n">
         <v>10760</v>
       </c>
-      <c r="M14" s="7" t="n">
+      <c r="M14" s="82" t="n">
         <v>10880</v>
       </c>
-      <c r="N14" s="7" t="n">
+      <c r="N14" s="83" t="n">
         <v>11020</v>
       </c>
       <c r="O14" s="8" t="inlineStr">
@@ -27699,7 +29229,10 @@
       <c r="P14" s="7" t="n">
         <v>15400</v>
       </c>
-      <c r="Q14" s="8" t="inlineStr">
+      <c r="Q14" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
@@ -27716,40 +29249,40 @@
           <t>Yapay Zeka</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="23" t="n">
         <v>13700</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="41" t="n">
         <v>8200</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="84" t="n">
         <v>11000</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="85" t="n">
         <v>9500</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="84" t="n">
         <v>11000</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="86" t="n">
         <v>10200</v>
       </c>
-      <c r="I15" s="15" t="n">
+      <c r="I15" s="22" t="n">
         <v>7300</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" s="85" t="n">
         <v>9500</v>
       </c>
-      <c r="K15" s="15" t="n">
+      <c r="K15" s="22" t="n">
         <v>7300</v>
       </c>
-      <c r="L15" s="18" t="n">
+      <c r="L15" s="87" t="n">
         <v>9000</v>
       </c>
-      <c r="M15" s="18" t="n">
+      <c r="M15" s="88" t="n">
         <v>8500</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="89" t="n">
         <v>9400</v>
       </c>
       <c r="O15" s="8" t="inlineStr">
@@ -27760,7 +29293,10 @@
       <c r="P15" s="7" t="n">
         <v>13700</v>
       </c>
-      <c r="Q15" s="8" t="inlineStr">
+      <c r="Q15" s="8" t="n">
+        <v>143</v>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
         <is>
           <t>Kasım</t>
         </is>
@@ -27777,40 +29313,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="86" t="n">
         <v>4900</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="89" t="n">
         <v>4480</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="86" t="n">
         <v>4900</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="90" t="n">
         <v>3900</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="91" t="n">
         <v>4200</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>3700</v>
       </c>
-      <c r="I16" s="15" t="n">
+      <c r="I16" s="22" t="n">
         <v>3400</v>
       </c>
-      <c r="J16" s="7" t="n">
+      <c r="J16" s="86" t="n">
         <v>4900</v>
       </c>
-      <c r="K16" s="7" t="n">
+      <c r="K16" s="92" t="n">
         <v>4600</v>
       </c>
-      <c r="L16" s="17" t="n">
+      <c r="L16" s="93" t="n">
         <v>5400</v>
       </c>
-      <c r="M16" s="16" t="n">
+      <c r="M16" s="23" t="n">
         <v>6700</v>
       </c>
-      <c r="N16" s="17" t="n">
+      <c r="N16" s="94" t="n">
         <v>5700</v>
       </c>
       <c r="O16" s="8" t="inlineStr">
@@ -27821,7 +29357,10 @@
       <c r="P16" s="7" t="n">
         <v>6700</v>
       </c>
-      <c r="Q16" s="8" t="inlineStr">
+      <c r="Q16" s="8" t="n">
+        <v>142</v>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
         <is>
           <t>Eylül</t>
         </is>
@@ -27838,40 +29377,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C17" s="16" t="n">
+      <c r="C17" s="95" t="n">
         <v>158600</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="36" t="n">
         <v>89780</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="96" t="n">
         <v>96010</v>
       </c>
-      <c r="F17" s="7" t="n">
+      <c r="F17" s="97" t="n">
         <v>116530</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="98" t="n">
         <v>121110</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="22" t="n">
         <v>87480</v>
       </c>
-      <c r="I17" s="15" t="n">
+      <c r="I17" s="99" t="n">
         <v>89790</v>
       </c>
-      <c r="J17" s="7" t="n">
+      <c r="J17" s="62" t="n">
         <v>115960</v>
       </c>
-      <c r="K17" s="16" t="n">
+      <c r="K17" s="23" t="n">
         <v>166060</v>
       </c>
-      <c r="L17" s="7" t="n">
+      <c r="L17" s="100" t="n">
         <v>124010</v>
       </c>
-      <c r="M17" s="7" t="n">
+      <c r="M17" s="101" t="n">
         <v>120920</v>
       </c>
-      <c r="N17" s="17" t="n">
+      <c r="N17" s="102" t="n">
         <v>144660</v>
       </c>
       <c r="O17" s="8" t="inlineStr">
@@ -27882,7 +29421,10 @@
       <c r="P17" s="7" t="n">
         <v>166060</v>
       </c>
-      <c r="Q17" s="8" t="inlineStr">
+      <c r="Q17" s="8" t="n">
+        <v>139</v>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
         <is>
           <t>Temmuz</t>
         </is>
@@ -27899,40 +29441,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="103" t="n">
         <v>40600</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="22" t="n">
         <v>32760</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="91" t="n">
         <v>40100</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="57" t="n">
         <v>39520</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="104" t="n">
         <v>47980</v>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H18" s="75" t="n">
         <v>47280</v>
       </c>
-      <c r="I18" s="17" t="n">
+      <c r="I18" s="105" t="n">
         <v>52400</v>
       </c>
-      <c r="J18" s="16" t="n">
+      <c r="J18" s="23" t="n">
         <v>62700</v>
       </c>
-      <c r="K18" s="7" t="n">
+      <c r="K18" s="106" t="n">
         <v>50500</v>
       </c>
-      <c r="L18" s="7" t="n">
+      <c r="L18" s="107" t="n">
         <v>46120</v>
       </c>
-      <c r="M18" s="7" t="n">
+      <c r="M18" s="108" t="n">
         <v>45920</v>
       </c>
-      <c r="N18" s="18" t="n">
+      <c r="N18" s="27" t="n">
         <v>38920</v>
       </c>
       <c r="O18" s="8" t="inlineStr">
@@ -27943,13 +29485,16 @@
       <c r="P18" s="7" t="n">
         <v>62700</v>
       </c>
-      <c r="Q18" s="8" t="inlineStr">
+      <c r="Q18" s="8" t="n">
+        <v>138</v>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="21" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>SSD, RAM ve Ekran Kartı: Bilgisayar Donanımı Rehberi</t>
@@ -27960,40 +29505,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="109" t="n">
         <v>30080</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="110" t="n">
         <v>22320</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="103" t="n">
         <v>20270</v>
       </c>
-      <c r="F19" s="18" t="n">
+      <c r="F19" s="111" t="n">
         <v>22600</v>
       </c>
-      <c r="G19" s="15" t="n">
+      <c r="G19" s="53" t="n">
         <v>16860</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="43" t="n">
         <v>17150</v>
       </c>
-      <c r="I19" s="15" t="n">
+      <c r="I19" s="22" t="n">
         <v>15400</v>
       </c>
-      <c r="J19" s="7" t="n">
+      <c r="J19" s="112" t="n">
         <v>24760</v>
       </c>
-      <c r="K19" s="16" t="n">
+      <c r="K19" s="113" t="n">
         <v>33800</v>
       </c>
-      <c r="L19" s="16" t="n">
+      <c r="L19" s="113" t="n">
         <v>33800</v>
       </c>
-      <c r="M19" s="16" t="n">
+      <c r="M19" s="114" t="n">
         <v>32100</v>
       </c>
-      <c r="N19" s="16" t="n">
+      <c r="N19" s="23" t="n">
         <v>34000</v>
       </c>
       <c r="O19" s="8" t="inlineStr">
@@ -28004,13 +29549,16 @@
       <c r="P19" s="7" t="n">
         <v>34000</v>
       </c>
-      <c r="Q19" s="8" t="inlineStr">
+      <c r="Q19" s="8" t="n">
+        <v>135</v>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
         <is>
           <t>Ekim</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="34" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Ekran Yansıtma: Telefondan Televizyona Görüntü Aktarma</t>
@@ -28021,40 +29569,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="115" t="n">
         <v>48000</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="116" t="n">
         <v>39200</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="E20" s="117" t="n">
         <v>38900</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="118" t="n">
         <v>41900</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="119" t="n">
         <v>30200</v>
       </c>
-      <c r="H20" s="15" t="n">
+      <c r="H20" s="22" t="n">
         <v>21020</v>
       </c>
-      <c r="I20" s="15" t="n">
+      <c r="I20" s="21" t="n">
         <v>21660</v>
       </c>
-      <c r="J20" s="17" t="n">
+      <c r="J20" s="120" t="n">
         <v>43700</v>
       </c>
-      <c r="K20" s="7" t="n">
+      <c r="K20" s="121" t="n">
         <v>39100</v>
       </c>
-      <c r="L20" s="7" t="n">
+      <c r="L20" s="118" t="n">
         <v>41900</v>
       </c>
-      <c r="M20" s="17" t="n">
+      <c r="M20" s="122" t="n">
         <v>47100</v>
       </c>
-      <c r="N20" s="16" t="n">
+      <c r="N20" s="23" t="n">
         <v>51500</v>
       </c>
       <c r="O20" s="8" t="inlineStr">
@@ -28065,7 +29613,10 @@
       <c r="P20" s="7" t="n">
         <v>51500</v>
       </c>
-      <c r="Q20" s="8" t="inlineStr">
+      <c r="Q20" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
         <is>
           <t>Ekim</t>
         </is>
@@ -28082,40 +29633,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C21" s="123" t="n">
         <v>13300</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="64" t="n">
         <v>10800</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="124" t="n">
         <v>9000</v>
       </c>
-      <c r="F21" s="15" t="n">
+      <c r="F21" s="125" t="n">
         <v>8300</v>
       </c>
-      <c r="G21" s="15" t="n">
+      <c r="G21" s="126" t="n">
         <v>8600</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="67" t="n">
         <v>8900</v>
       </c>
-      <c r="I21" s="15" t="n">
+      <c r="I21" s="22" t="n">
         <v>7220</v>
       </c>
-      <c r="J21" s="16" t="n">
+      <c r="J21" s="23" t="n">
         <v>14400</v>
       </c>
-      <c r="K21" s="17" t="n">
+      <c r="K21" s="127" t="n">
         <v>12700</v>
       </c>
-      <c r="L21" s="7" t="n">
+      <c r="L21" s="128" t="n">
         <v>11400</v>
       </c>
-      <c r="M21" s="17" t="n">
+      <c r="M21" s="129" t="n">
         <v>12200</v>
       </c>
-      <c r="N21" s="17" t="n">
+      <c r="N21" s="109" t="n">
         <v>12900</v>
       </c>
       <c r="O21" s="8" t="inlineStr">
@@ -28126,13 +29677,16 @@
       <c r="P21" s="7" t="n">
         <v>14400</v>
       </c>
-      <c r="Q21" s="8" t="inlineStr">
+      <c r="Q21" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="34" customHeight="1">
+    <row r="22" ht="21" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>KVKK Nedir? Kişisel Verilerin Korunması Kanunu</t>
@@ -28143,40 +29697,40 @@
           <t>Güvenlik &amp; Gizlilik</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="72" t="n">
         <v>16400</v>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="121" t="n">
         <v>17200</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="E22" s="72" t="n">
         <v>16400</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F22" s="72" t="n">
         <v>16400</v>
       </c>
-      <c r="G22" s="18" t="n">
+      <c r="G22" s="31" t="n">
         <v>13700</v>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H22" s="72" t="n">
         <v>16400</v>
       </c>
-      <c r="I22" s="18" t="n">
+      <c r="I22" s="19" t="n">
         <v>13400</v>
       </c>
-      <c r="J22" s="15" t="n">
+      <c r="J22" s="22" t="n">
         <v>13100</v>
       </c>
-      <c r="K22" s="18" t="n">
+      <c r="K22" s="19" t="n">
         <v>13400</v>
       </c>
-      <c r="L22" s="15" t="n">
+      <c r="L22" s="22" t="n">
         <v>13100</v>
       </c>
-      <c r="M22" s="7" t="n">
+      <c r="M22" s="130" t="n">
         <v>16100</v>
       </c>
-      <c r="N22" s="16" t="n">
+      <c r="N22" s="23" t="n">
         <v>20000</v>
       </c>
       <c r="O22" s="8" t="inlineStr">
@@ -28187,7 +29741,10 @@
       <c r="P22" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="Q22" s="8" t="inlineStr">
+      <c r="Q22" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="R22" s="8" t="inlineStr">
         <is>
           <t>Ekim</t>
         </is>
@@ -28204,40 +29761,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="C23" s="131" t="n">
         <v>4480</v>
       </c>
-      <c r="D23" s="15" t="n">
+      <c r="D23" s="65" t="n">
         <v>2990</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="132" t="n">
         <v>3120</v>
       </c>
-      <c r="F23" s="15" t="n">
+      <c r="F23" s="65" t="n">
         <v>2990</v>
       </c>
-      <c r="G23" s="15" t="n">
+      <c r="G23" s="22" t="n">
         <v>2380</v>
       </c>
-      <c r="H23" s="15" t="n">
+      <c r="H23" s="65" t="n">
         <v>2990</v>
       </c>
-      <c r="I23" s="18" t="n">
+      <c r="I23" s="132" t="n">
         <v>3120</v>
       </c>
-      <c r="J23" s="7" t="n">
+      <c r="J23" s="133" t="n">
         <v>3900</v>
       </c>
-      <c r="K23" s="7" t="n">
+      <c r="K23" s="134" t="n">
         <v>3780</v>
       </c>
-      <c r="L23" s="16" t="n">
+      <c r="L23" s="23" t="n">
         <v>4600</v>
       </c>
-      <c r="M23" s="16" t="n">
+      <c r="M23" s="23" t="n">
         <v>4600</v>
       </c>
-      <c r="N23" s="7" t="n">
+      <c r="N23" s="134" t="n">
         <v>3780</v>
       </c>
       <c r="O23" s="8" t="inlineStr">
@@ -28248,7 +29805,10 @@
       <c r="P23" s="7" t="n">
         <v>4600</v>
       </c>
-      <c r="Q23" s="8" t="inlineStr">
+      <c r="Q23" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="R23" s="8" t="inlineStr">
         <is>
           <t>Eylül</t>
         </is>
@@ -28265,40 +29825,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C24" s="23" t="n">
         <v>8100</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="135" t="n">
         <v>5400</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="E24" s="121" t="n">
         <v>6600</v>
       </c>
-      <c r="F24" s="15" t="n">
+      <c r="F24" s="22" t="n">
         <v>4400</v>
       </c>
-      <c r="G24" s="15" t="n">
+      <c r="G24" s="22" t="n">
         <v>4400</v>
       </c>
-      <c r="H24" s="15" t="n">
+      <c r="H24" s="22" t="n">
         <v>4400</v>
       </c>
-      <c r="I24" s="15" t="n">
+      <c r="I24" s="22" t="n">
         <v>4400</v>
       </c>
-      <c r="J24" s="16" t="n">
+      <c r="J24" s="23" t="n">
         <v>8100</v>
       </c>
-      <c r="K24" s="16" t="n">
+      <c r="K24" s="23" t="n">
         <v>8100</v>
       </c>
-      <c r="L24" s="7" t="n">
+      <c r="L24" s="121" t="n">
         <v>6600</v>
       </c>
-      <c r="M24" s="16" t="n">
+      <c r="M24" s="23" t="n">
         <v>8100</v>
       </c>
-      <c r="N24" s="7" t="n">
+      <c r="N24" s="121" t="n">
         <v>6600</v>
       </c>
       <c r="O24" s="8" t="inlineStr">
@@ -28309,13 +29869,16 @@
       <c r="P24" s="7" t="n">
         <v>8100</v>
       </c>
-      <c r="Q24" s="8" t="inlineStr">
+      <c r="Q24" s="8" t="n">
+        <v>129</v>
+      </c>
+      <c r="R24" s="8" t="inlineStr">
         <is>
           <t>Kasım</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1">
+    <row r="25" ht="21" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>PUK, PIN ve SIM Kilidi: Kod Öğrenme ve Kilit Açma</t>
@@ -28326,40 +29889,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="136" t="n">
         <v>64200</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="45" t="n">
         <v>51880</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="E25" s="137" t="n">
         <v>56900</v>
       </c>
-      <c r="F25" s="15" t="n">
+      <c r="F25" s="22" t="n">
         <v>47800</v>
       </c>
-      <c r="G25" s="18" t="n">
+      <c r="G25" s="138" t="n">
         <v>54100</v>
       </c>
-      <c r="H25" s="15" t="n">
+      <c r="H25" s="139" t="n">
         <v>47980</v>
       </c>
-      <c r="I25" s="18" t="n">
+      <c r="I25" s="140" t="n">
         <v>52200</v>
       </c>
-      <c r="J25" s="16" t="n">
+      <c r="J25" s="23" t="n">
         <v>74000</v>
       </c>
-      <c r="K25" s="17" t="n">
+      <c r="K25" s="141" t="n">
         <v>67000</v>
       </c>
-      <c r="L25" s="7" t="n">
+      <c r="L25" s="142" t="n">
         <v>64700</v>
       </c>
-      <c r="M25" s="7" t="n">
+      <c r="M25" s="143" t="n">
         <v>65100</v>
       </c>
-      <c r="N25" s="7" t="n">
+      <c r="N25" s="144" t="n">
         <v>61700</v>
       </c>
       <c r="O25" s="8" t="inlineStr">
@@ -28370,7 +29933,10 @@
       <c r="P25" s="7" t="n">
         <v>74000</v>
       </c>
-      <c r="Q25" s="8" t="inlineStr">
+      <c r="Q25" s="8" t="n">
+        <v>126</v>
+      </c>
+      <c r="R25" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
@@ -28387,40 +29953,40 @@
           <t>Güvenlik &amp; Gizlilik</t>
         </is>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C26" s="145" t="n">
         <v>30700</v>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="86" t="n">
         <v>25800</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="E26" s="146" t="n">
         <v>25100</v>
       </c>
-      <c r="F26" s="7" t="n">
+      <c r="F26" s="146" t="n">
         <v>25100</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G26" s="22" t="n">
         <v>20500</v>
       </c>
-      <c r="H26" s="7" t="n">
+      <c r="H26" s="86" t="n">
         <v>25800</v>
       </c>
-      <c r="I26" s="15" t="n">
+      <c r="I26" s="19" t="n">
         <v>21000</v>
       </c>
-      <c r="J26" s="16" t="n">
+      <c r="J26" s="23" t="n">
         <v>32100</v>
       </c>
-      <c r="K26" s="7" t="n">
+      <c r="K26" s="147" t="n">
         <v>26600</v>
       </c>
-      <c r="L26" s="18" t="n">
+      <c r="L26" s="148" t="n">
         <v>22500</v>
       </c>
-      <c r="M26" s="15" t="n">
+      <c r="M26" s="149" t="n">
         <v>21700</v>
       </c>
-      <c r="N26" s="17" t="n">
+      <c r="N26" s="145" t="n">
         <v>30700</v>
       </c>
       <c r="O26" s="8" t="inlineStr">
@@ -28431,7 +29997,10 @@
       <c r="P26" s="7" t="n">
         <v>32100</v>
       </c>
-      <c r="Q26" s="8" t="inlineStr">
+      <c r="Q26" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="R26" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
@@ -28448,40 +30017,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="69" t="n">
         <v>15280</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="150" t="n">
         <v>14120</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="E27" s="151" t="n">
         <v>14780</v>
       </c>
-      <c r="F27" s="18" t="n">
+      <c r="F27" s="92" t="n">
         <v>14390</v>
       </c>
-      <c r="G27" s="18" t="n">
+      <c r="G27" s="57" t="n">
         <v>13420</v>
       </c>
-      <c r="H27" s="18" t="n">
+      <c r="H27" s="152" t="n">
         <v>13290</v>
       </c>
-      <c r="I27" s="15" t="n">
+      <c r="I27" s="22" t="n">
         <v>11880</v>
       </c>
-      <c r="J27" s="17" t="n">
+      <c r="J27" s="153" t="n">
         <v>17200</v>
       </c>
-      <c r="K27" s="7" t="n">
+      <c r="K27" s="128" t="n">
         <v>15900</v>
       </c>
-      <c r="L27" s="17" t="n">
+      <c r="L27" s="154" t="n">
         <v>18400</v>
       </c>
-      <c r="M27" s="17" t="n">
+      <c r="M27" s="23" t="n">
         <v>18780</v>
       </c>
-      <c r="N27" s="7" t="n">
+      <c r="N27" s="155" t="n">
         <v>16320</v>
       </c>
       <c r="O27" s="8" t="inlineStr">
@@ -28492,7 +30061,10 @@
       <c r="P27" s="7" t="n">
         <v>18780</v>
       </c>
-      <c r="Q27" s="8" t="inlineStr">
+      <c r="Q27" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="R27" s="8" t="inlineStr">
         <is>
           <t>Eylül</t>
         </is>
@@ -28509,40 +30081,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="156" t="n">
         <v>28200</v>
       </c>
-      <c r="D28" s="15" t="n">
+      <c r="D28" s="22" t="n">
         <v>21900</v>
       </c>
-      <c r="E28" s="15" t="n">
+      <c r="E28" s="22" t="n">
         <v>21900</v>
       </c>
-      <c r="F28" s="15" t="n">
+      <c r="F28" s="30" t="n">
         <v>22100</v>
       </c>
-      <c r="G28" s="7" t="n">
+      <c r="G28" s="157" t="n">
         <v>27700</v>
       </c>
-      <c r="H28" s="15" t="n">
+      <c r="H28" s="30" t="n">
         <v>22100</v>
       </c>
-      <c r="I28" s="18" t="n">
+      <c r="I28" s="41" t="n">
         <v>23400</v>
       </c>
-      <c r="J28" s="17" t="n">
+      <c r="J28" s="23" t="n">
         <v>32600</v>
       </c>
-      <c r="K28" s="17" t="n">
+      <c r="K28" s="23" t="n">
         <v>32600</v>
       </c>
-      <c r="L28" s="17" t="n">
+      <c r="L28" s="158" t="n">
         <v>30600</v>
       </c>
-      <c r="M28" s="7" t="n">
+      <c r="M28" s="157" t="n">
         <v>27700</v>
       </c>
-      <c r="N28" s="7" t="n">
+      <c r="N28" s="159" t="n">
         <v>27400</v>
       </c>
       <c r="O28" s="8" t="inlineStr">
@@ -28553,7 +30125,10 @@
       <c r="P28" s="7" t="n">
         <v>32600</v>
       </c>
-      <c r="Q28" s="8" t="inlineStr">
+      <c r="Q28" s="8" t="n">
+        <v>123</v>
+      </c>
+      <c r="R28" s="8" t="inlineStr">
         <is>
           <t>Temmuz</t>
         </is>
@@ -28570,40 +30145,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="160" t="n">
         <v>17000</v>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D29" s="161" t="n">
         <v>15600</v>
       </c>
-      <c r="E29" s="18" t="n">
+      <c r="E29" s="162" t="n">
         <v>14100</v>
       </c>
-      <c r="F29" s="18" t="n">
+      <c r="F29" s="162" t="n">
         <v>14100</v>
       </c>
-      <c r="G29" s="15" t="n">
+      <c r="G29" s="163" t="n">
         <v>12800</v>
       </c>
-      <c r="H29" s="18" t="n">
+      <c r="H29" s="60" t="n">
         <v>14300</v>
       </c>
-      <c r="I29" s="15" t="n">
+      <c r="I29" s="22" t="n">
         <v>12000</v>
       </c>
-      <c r="J29" s="18" t="n">
+      <c r="J29" s="60" t="n">
         <v>14300</v>
       </c>
-      <c r="K29" s="17" t="n">
+      <c r="K29" s="23" t="n">
         <v>18500</v>
       </c>
-      <c r="L29" s="17" t="n">
+      <c r="L29" s="123" t="n">
         <v>17500</v>
       </c>
-      <c r="M29" s="17" t="n">
+      <c r="M29" s="164" t="n">
         <v>18200</v>
       </c>
-      <c r="N29" s="17" t="n">
+      <c r="N29" s="164" t="n">
         <v>18200</v>
       </c>
       <c r="O29" s="8" t="inlineStr">
@@ -28614,7 +30189,10 @@
       <c r="P29" s="7" t="n">
         <v>18500</v>
       </c>
-      <c r="Q29" s="8" t="inlineStr">
+      <c r="Q29" s="8" t="n">
+        <v>119</v>
+      </c>
+      <c r="R29" s="8" t="inlineStr">
         <is>
           <t>Temmuz</t>
         </is>
@@ -28631,40 +30209,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C30" s="165" t="n">
         <v>9700</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="166" t="n">
         <v>9400</v>
       </c>
-      <c r="E30" s="17" t="n">
+      <c r="E30" s="165" t="n">
         <v>9700</v>
       </c>
-      <c r="F30" s="7" t="n">
+      <c r="F30" s="167" t="n">
         <v>8200</v>
       </c>
-      <c r="G30" s="18" t="n">
+      <c r="G30" s="82" t="n">
         <v>7900</v>
       </c>
-      <c r="H30" s="18" t="n">
+      <c r="H30" s="82" t="n">
         <v>7900</v>
       </c>
-      <c r="I30" s="18" t="n">
+      <c r="I30" s="82" t="n">
         <v>7900</v>
       </c>
-      <c r="J30" s="15" t="n">
+      <c r="J30" s="22" t="n">
         <v>6300</v>
       </c>
-      <c r="K30" s="15" t="n">
+      <c r="K30" s="88" t="n">
         <v>7000</v>
       </c>
-      <c r="L30" s="15" t="n">
+      <c r="L30" s="88" t="n">
         <v>7000</v>
       </c>
-      <c r="M30" s="17" t="n">
+      <c r="M30" s="23" t="n">
         <v>10000</v>
       </c>
-      <c r="N30" s="17" t="n">
+      <c r="N30" s="165" t="n">
         <v>9700</v>
       </c>
       <c r="O30" s="8" t="inlineStr">
@@ -28675,7 +30253,10 @@
       <c r="P30" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="Q30" s="8" t="inlineStr">
+      <c r="Q30" s="8" t="n">
+        <v>119</v>
+      </c>
+      <c r="R30" s="8" t="inlineStr">
         <is>
           <t>Eylül</t>
         </is>
@@ -28692,40 +30273,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="168" t="n">
         <v>226000</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="22" t="n">
         <v>187300</v>
       </c>
-      <c r="E31" s="7" t="n">
+      <c r="E31" s="169" t="n">
         <v>207100</v>
       </c>
-      <c r="F31" s="18" t="n">
+      <c r="F31" s="170" t="n">
         <v>203700</v>
       </c>
-      <c r="G31" s="18" t="n">
+      <c r="G31" s="124" t="n">
         <v>204500</v>
       </c>
-      <c r="H31" s="7" t="n">
+      <c r="H31" s="171" t="n">
         <v>214900</v>
       </c>
-      <c r="I31" s="7" t="n">
+      <c r="I31" s="98" t="n">
         <v>216900</v>
       </c>
-      <c r="J31" s="17" t="n">
+      <c r="J31" s="23" t="n">
         <v>256400</v>
       </c>
-      <c r="K31" s="7" t="n">
+      <c r="K31" s="172" t="n">
         <v>223100</v>
       </c>
-      <c r="L31" s="7" t="n">
+      <c r="L31" s="173" t="n">
         <v>224900</v>
       </c>
-      <c r="M31" s="7" t="n">
+      <c r="M31" s="116" t="n">
         <v>228500</v>
       </c>
-      <c r="N31" s="7" t="n">
+      <c r="N31" s="174" t="n">
         <v>221400</v>
       </c>
       <c r="O31" s="8" t="inlineStr">
@@ -28736,13 +30317,16 @@
       <c r="P31" s="7" t="n">
         <v>256400</v>
       </c>
-      <c r="Q31" s="8" t="inlineStr">
+      <c r="Q31" s="8" t="n">
+        <v>118</v>
+      </c>
+      <c r="R31" s="8" t="inlineStr">
         <is>
           <t>Haziran</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="21" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Telefondan Telefona Veri Aktarma: Android ve iPhone</t>
@@ -28753,40 +30337,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C32" s="23" t="n">
         <v>22100</v>
       </c>
-      <c r="D32" s="7" t="n">
+      <c r="D32" s="175" t="n">
         <v>19080</v>
       </c>
-      <c r="E32" s="7" t="n">
+      <c r="E32" s="175" t="n">
         <v>19080</v>
       </c>
-      <c r="F32" s="18" t="n">
+      <c r="F32" s="138" t="n">
         <v>16700</v>
       </c>
-      <c r="G32" s="18" t="n">
+      <c r="G32" s="56" t="n">
         <v>16800</v>
       </c>
-      <c r="H32" s="15" t="n">
+      <c r="H32" s="22" t="n">
         <v>15000</v>
       </c>
-      <c r="I32" s="15" t="n">
+      <c r="I32" s="20" t="n">
         <v>15580</v>
       </c>
-      <c r="J32" s="7" t="n">
+      <c r="J32" s="176" t="n">
         <v>19820</v>
       </c>
-      <c r="K32" s="7" t="n">
+      <c r="K32" s="177" t="n">
         <v>20490</v>
       </c>
-      <c r="L32" s="18" t="n">
+      <c r="L32" s="178" t="n">
         <v>16580</v>
       </c>
-      <c r="M32" s="17" t="n">
+      <c r="M32" s="179" t="n">
         <v>21220</v>
       </c>
-      <c r="N32" s="17" t="n">
+      <c r="N32" s="180" t="n">
         <v>21800</v>
       </c>
       <c r="O32" s="8" t="inlineStr">
@@ -28797,7 +30381,10 @@
       <c r="P32" s="7" t="n">
         <v>22100</v>
       </c>
-      <c r="Q32" s="8" t="inlineStr">
+      <c r="Q32" s="8" t="n">
+        <v>118</v>
+      </c>
+      <c r="R32" s="8" t="inlineStr">
         <is>
           <t>Kasım</t>
         </is>
@@ -28814,40 +30401,40 @@
           <t>Cihaz &amp; Donanım</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n">
+      <c r="C33" s="93" t="n">
         <v>31380</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="119" t="n">
         <v>28090</v>
       </c>
-      <c r="E33" s="7" t="n">
+      <c r="E33" s="181" t="n">
         <v>30480</v>
       </c>
-      <c r="F33" s="7" t="n">
+      <c r="F33" s="143" t="n">
         <v>31980</v>
       </c>
-      <c r="G33" s="15" t="n">
+      <c r="G33" s="149" t="n">
         <v>25890</v>
       </c>
-      <c r="H33" s="7" t="n">
+      <c r="H33" s="182" t="n">
         <v>30980</v>
       </c>
-      <c r="I33" s="15" t="n">
+      <c r="I33" s="31" t="n">
         <v>25690</v>
       </c>
-      <c r="J33" s="15" t="n">
+      <c r="J33" s="22" t="n">
         <v>24780</v>
       </c>
-      <c r="K33" s="7" t="n">
+      <c r="K33" s="116" t="n">
         <v>31290</v>
       </c>
-      <c r="L33" s="17" t="n">
+      <c r="L33" s="183" t="n">
         <v>35520</v>
       </c>
-      <c r="M33" s="17" t="n">
+      <c r="M33" s="184" t="n">
         <v>34820</v>
       </c>
-      <c r="N33" s="17" t="n">
+      <c r="N33" s="23" t="n">
         <v>35680</v>
       </c>
       <c r="O33" s="8" t="inlineStr">
@@ -28858,7 +30445,10 @@
       <c r="P33" s="7" t="n">
         <v>35680</v>
       </c>
-      <c r="Q33" s="8" t="inlineStr">
+      <c r="Q33" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="R33" s="8" t="inlineStr">
         <is>
           <t>Ekim</t>
         </is>
@@ -28875,40 +30465,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C34" s="185" t="n">
         <v>133600</v>
       </c>
-      <c r="D34" s="7" t="n">
+      <c r="D34" s="186" t="n">
         <v>112180</v>
       </c>
-      <c r="E34" s="17" t="n">
+      <c r="E34" s="187" t="n">
         <v>134380</v>
       </c>
-      <c r="F34" s="18" t="n">
+      <c r="F34" s="37" t="n">
         <v>110680</v>
       </c>
-      <c r="G34" s="18" t="n">
+      <c r="G34" s="53" t="n">
         <v>107320</v>
       </c>
-      <c r="H34" s="18" t="n">
+      <c r="H34" s="188" t="n">
         <v>106880</v>
       </c>
-      <c r="I34" s="18" t="n">
+      <c r="I34" s="22" t="n">
         <v>104920</v>
       </c>
-      <c r="J34" s="18" t="n">
+      <c r="J34" s="57" t="n">
         <v>112100</v>
       </c>
-      <c r="K34" s="7" t="n">
+      <c r="K34" s="169" t="n">
         <v>114100</v>
       </c>
-      <c r="L34" s="17" t="n">
+      <c r="L34" s="23" t="n">
         <v>136700</v>
       </c>
-      <c r="M34" s="7" t="n">
+      <c r="M34" s="92" t="n">
         <v>116500</v>
       </c>
-      <c r="N34" s="17" t="n">
+      <c r="N34" s="189" t="n">
         <v>134400</v>
       </c>
       <c r="O34" s="8" t="inlineStr">
@@ -28919,7 +30509,10 @@
       <c r="P34" s="7" t="n">
         <v>136700</v>
       </c>
-      <c r="Q34" s="8" t="inlineStr">
+      <c r="Q34" s="8" t="n">
+        <v>115</v>
+      </c>
+      <c r="R34" s="8" t="inlineStr">
         <is>
           <t>Ağustos</t>
         </is>
@@ -28936,40 +30529,40 @@
           <t>Abone İşlemleri &amp; Hat</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C35" s="190" t="n">
         <v>7000</v>
       </c>
-      <c r="D35" s="18" t="n">
+      <c r="D35" s="171" t="n">
         <v>6700</v>
       </c>
-      <c r="E35" s="17" t="n">
+      <c r="E35" s="23" t="n">
         <v>8200</v>
       </c>
-      <c r="F35" s="18" t="n">
+      <c r="F35" s="171" t="n">
         <v>6700</v>
       </c>
-      <c r="G35" s="18" t="n">
+      <c r="G35" s="171" t="n">
         <v>6700</v>
       </c>
-      <c r="H35" s="15" t="n">
+      <c r="H35" s="22" t="n">
         <v>5700</v>
       </c>
-      <c r="I35" s="15" t="n">
+      <c r="I35" s="22" t="n">
         <v>5700</v>
       </c>
-      <c r="J35" s="7" t="n">
+      <c r="J35" s="190" t="n">
         <v>7000</v>
       </c>
-      <c r="K35" s="17" t="n">
+      <c r="K35" s="23" t="n">
         <v>8200</v>
       </c>
-      <c r="L35" s="17" t="n">
+      <c r="L35" s="23" t="n">
         <v>8200</v>
       </c>
-      <c r="M35" s="17" t="n">
+      <c r="M35" s="23" t="n">
         <v>8200</v>
       </c>
-      <c r="N35" s="17" t="n">
+      <c r="N35" s="23" t="n">
         <v>8200</v>
       </c>
       <c r="O35" s="8" t="inlineStr">
@@ -28980,7 +30573,10 @@
       <c r="P35" s="7" t="n">
         <v>8200</v>
       </c>
-      <c r="Q35" s="19" t="inlineStr">
+      <c r="Q35" s="8" t="n">
+        <v>114</v>
+      </c>
+      <c r="R35" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
@@ -28997,40 +30593,40 @@
           <t>Altyapı &amp; Bağlantı</t>
         </is>
       </c>
-      <c r="C36" s="17" t="n">
+      <c r="C36" s="23" t="n">
         <v>135900</v>
       </c>
-      <c r="D36" s="7" t="n">
+      <c r="D36" s="188" t="n">
         <v>114800</v>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="192" t="n">
         <v>119700</v>
       </c>
-      <c r="F36" s="7" t="n">
+      <c r="F36" s="83" t="n">
         <v>123500</v>
       </c>
-      <c r="G36" s="18" t="n">
+      <c r="G36" s="99" t="n">
         <v>114100</v>
       </c>
-      <c r="H36" s="7" t="n">
+      <c r="H36" s="193" t="n">
         <v>116100</v>
       </c>
-      <c r="I36" s="18" t="n">
+      <c r="I36" s="22" t="n">
         <v>113400</v>
       </c>
-      <c r="J36" s="18" t="n">
+      <c r="J36" s="194" t="n">
         <v>114200</v>
       </c>
-      <c r="K36" s="7" t="n">
+      <c r="K36" s="149" t="n">
         <v>115700</v>
       </c>
-      <c r="L36" s="7" t="n">
+      <c r="L36" s="184" t="n">
         <v>134100</v>
       </c>
-      <c r="M36" s="7" t="n">
+      <c r="M36" s="195" t="n">
         <v>125500</v>
       </c>
-      <c r="N36" s="7" t="n">
+      <c r="N36" s="196" t="n">
         <v>128800</v>
       </c>
       <c r="O36" s="8" t="inlineStr">
@@ -29041,13 +30637,16 @@
       <c r="P36" s="7" t="n">
         <v>135900</v>
       </c>
-      <c r="Q36" s="19" t="inlineStr">
+      <c r="Q36" s="8" t="n">
+        <v>112</v>
+      </c>
+      <c r="R36" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="36" customHeight="1">
+    <row r="37" ht="34" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
           <t>En İyi Chrome Eklentileri: Hangisi Ne İşe Yarar?</t>
@@ -29058,40 +30657,40 @@
           <t>Dijital Araç &amp; Uygulama</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n">
+      <c r="C37" s="197" t="n">
         <v>18900</v>
       </c>
-      <c r="D37" s="7" t="n">
+      <c r="D37" s="104" t="n">
         <v>16900</v>
       </c>
-      <c r="E37" s="7" t="n">
+      <c r="E37" s="153" t="n">
         <v>18400</v>
       </c>
-      <c r="F37" s="7" t="n">
+      <c r="F37" s="84" t="n">
         <v>17300</v>
       </c>
-      <c r="G37" s="7" t="n">
+      <c r="G37" s="76" t="n">
         <v>18100</v>
       </c>
-      <c r="H37" s="7" t="n">
+      <c r="H37" s="84" t="n">
         <v>17300</v>
       </c>
-      <c r="I37" s="15" t="n">
+      <c r="I37" s="22" t="n">
         <v>14000</v>
       </c>
-      <c r="J37" s="18" t="n">
+      <c r="J37" s="130" t="n">
         <v>16500</v>
       </c>
-      <c r="K37" s="7" t="n">
+      <c r="K37" s="153" t="n">
         <v>18400</v>
       </c>
-      <c r="L37" s="7" t="n">
+      <c r="L37" s="153" t="n">
         <v>18400</v>
       </c>
-      <c r="M37" s="7" t="n">
+      <c r="M37" s="23" t="n">
         <v>19700</v>
       </c>
-      <c r="N37" s="7" t="n">
+      <c r="N37" s="198" t="n">
         <v>19200</v>
       </c>
       <c r="O37" s="8" t="inlineStr">
@@ -29102,13 +30701,16 @@
       <c r="P37" s="7" t="n">
         <v>19700</v>
       </c>
-      <c r="Q37" s="19" t="inlineStr">
+      <c r="Q37" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="R37" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="36" customHeight="1">
+    <row r="38" ht="34" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>192.168.1.1 Modem Arayüzü: Giriş ve Şifre Değiştirme</t>
@@ -29119,40 +30721,40 @@
           <t>Altyapı &amp; Bağlantı</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
+      <c r="C38" s="23" t="n">
         <v>304040</v>
       </c>
-      <c r="D38" s="7" t="n">
+      <c r="D38" s="151" t="n">
         <v>280130</v>
       </c>
-      <c r="E38" s="7" t="n">
+      <c r="E38" s="130" t="n">
         <v>280860</v>
       </c>
-      <c r="F38" s="7" t="n">
+      <c r="F38" s="78" t="n">
         <v>271210</v>
       </c>
-      <c r="G38" s="7" t="n">
+      <c r="G38" s="20" t="n">
         <v>266260</v>
       </c>
-      <c r="H38" s="7" t="n">
+      <c r="H38" s="55" t="n">
         <v>268560</v>
       </c>
-      <c r="I38" s="7" t="n">
+      <c r="I38" s="117" t="n">
         <v>287020</v>
       </c>
-      <c r="J38" s="7" t="n">
+      <c r="J38" s="89" t="n">
         <v>276370</v>
       </c>
-      <c r="K38" s="7" t="n">
+      <c r="K38" s="199" t="n">
         <v>274170</v>
       </c>
-      <c r="L38" s="7" t="n">
+      <c r="L38" s="26" t="n">
         <v>268510</v>
       </c>
-      <c r="M38" s="7" t="n">
+      <c r="M38" s="22" t="n">
         <v>262910</v>
       </c>
-      <c r="N38" s="7" t="n">
+      <c r="N38" s="123" t="n">
         <v>297710</v>
       </c>
       <c r="O38" s="8" t="inlineStr">
@@ -29163,13 +30765,16 @@
       <c r="P38" s="7" t="n">
         <v>304040</v>
       </c>
-      <c r="Q38" s="19" t="inlineStr">
+      <c r="Q38" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="R38" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="36" customHeight="1">
+    <row r="39" ht="34" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Spam Ne Demek? Spam Mesaj ve Aramaları Engelleme</t>
@@ -29180,40 +30785,40 @@
           <t>Güvenlik &amp; Gizlilik</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n">
+      <c r="C39" s="177" t="n">
         <v>27000</v>
       </c>
-      <c r="D39" s="7" t="n">
+      <c r="D39" s="200" t="n">
         <v>26700</v>
       </c>
-      <c r="E39" s="7" t="n">
+      <c r="E39" s="71" t="n">
         <v>25400</v>
       </c>
-      <c r="F39" s="7" t="n">
+      <c r="F39" s="71" t="n">
         <v>25400</v>
       </c>
-      <c r="G39" s="7" t="n">
+      <c r="G39" s="71" t="n">
         <v>25400</v>
       </c>
-      <c r="H39" s="7" t="n">
+      <c r="H39" s="71" t="n">
         <v>25400</v>
       </c>
-      <c r="I39" s="7" t="n">
+      <c r="I39" s="201" t="n">
         <v>25600</v>
       </c>
-      <c r="J39" s="7" t="n">
+      <c r="J39" s="23" t="n">
         <v>28200</v>
       </c>
-      <c r="K39" s="7" t="n">
+      <c r="K39" s="202" t="n">
         <v>27500</v>
       </c>
-      <c r="L39" s="18" t="n">
+      <c r="L39" s="22" t="n">
         <v>22900</v>
       </c>
-      <c r="M39" s="7" t="n">
+      <c r="M39" s="95" t="n">
         <v>27700</v>
       </c>
-      <c r="N39" s="7" t="n">
+      <c r="N39" s="203" t="n">
         <v>28000</v>
       </c>
       <c r="O39" s="8" t="inlineStr">
@@ -29224,7 +30829,10 @@
       <c r="P39" s="7" t="n">
         <v>28000</v>
       </c>
-      <c r="Q39" s="19" t="inlineStr">
+      <c r="Q39" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="R39" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
@@ -29241,40 +30849,40 @@
           <t>Güvenlik &amp; Gizlilik</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C40" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="D40" s="7" t="n">
+      <c r="D40" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="E40" s="7" t="n">
+      <c r="E40" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="F40" s="18" t="n">
+      <c r="F40" s="204" t="n">
         <v>4600</v>
       </c>
-      <c r="G40" s="18" t="n">
+      <c r="G40" s="22" t="n">
         <v>4480</v>
       </c>
-      <c r="H40" s="18" t="n">
+      <c r="H40" s="204" t="n">
         <v>4600</v>
       </c>
-      <c r="I40" s="18" t="n">
+      <c r="I40" s="22" t="n">
         <v>4480</v>
       </c>
-      <c r="J40" s="7" t="n">
+      <c r="J40" s="23" t="n">
         <v>5400</v>
       </c>
-      <c r="K40" s="7" t="n">
+      <c r="K40" s="202" t="n">
         <v>5280</v>
       </c>
-      <c r="L40" s="7" t="n">
+      <c r="L40" s="202" t="n">
         <v>5280</v>
       </c>
-      <c r="M40" s="7" t="n">
+      <c r="M40" s="202" t="n">
         <v>5280</v>
       </c>
-      <c r="N40" s="7" t="n">
+      <c r="N40" s="202" t="n">
         <v>5280</v>
       </c>
       <c r="O40" s="8" t="inlineStr">
@@ -29285,7 +30893,10 @@
       <c r="P40" s="7" t="n">
         <v>5400</v>
       </c>
-      <c r="Q40" s="19" t="inlineStr">
+      <c r="Q40" s="8" t="n">
+        <v>106</v>
+      </c>
+      <c r="R40" s="191" t="inlineStr">
         <is>
           <t>sezon etkisi sınırlı</t>
         </is>
@@ -29309,6 +30920,7 @@
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="n"/>
       <c r="Q41" s="2" t="n"/>
+      <c r="R41" s="2" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -29318,7 +30930,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Hücrelerde kümedeki kelimelerin o aydaki toplam araması yazılıdır. Renk, ayın yıl ortalamasına oranını gösterir: ortalamanın %25 ve üzerinde olan aylar koyu yeşil, %12-24 üzeri açık yeşil, ortalama bandı nötr, %6-14 altı açık kırmızı, %15 ve fazlası altı kırmızıdır. Peak indeksi 115 altında kalan önerilerde sezon etkisi sınırlı sayılmış, yayın ayı puana göre belirlenmiştir.</t>
+          <t>Hücrelerde kümedeki kelimelerin o aydaki toplam araması yazılıdır. Renk satır içi konumu gösterir: satırın en düşük ayı kırmızı, orta bant sarı, en yüksek ayı yeşildir. Peak indeksi sütunu, peak ayının yıl ortalamasına oranıdır (100 = yıl ortalaması). Peak indeksi 115 altında kalan önerilerde sezon etkisi sınırlı sayılmış, yayın ayı puana göre belirlenmiştir.</t>
         </is>
       </c>
       <c r="C42" s="12" t="n"/>
@@ -29336,6 +30948,7 @@
       <c r="O42" s="12" t="n"/>
       <c r="P42" s="12" t="n"/>
       <c r="Q42" s="12" t="n"/>
+      <c r="R42" s="12" t="n"/>
     </row>
     <row r="43" ht="21" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -29363,12 +30976,13 @@
       <c r="O43" s="12" t="n"/>
       <c r="P43" s="12" t="n"/>
       <c r="Q43" s="12" t="n"/>
+      <c r="R43" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B43:Q43"/>
-    <mergeCell ref="B42:Q42"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="B43:R43"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="B42:R42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Kelime denetimi bölümü çıkarıldı, eleme ölçütü yöntem notuna indirgendi
İç çalışma katmanı olan bölüm hem rapordan hem Excel'den kaldırıldı:
öneri kümelerindeki değişim tablosu, 64 satırlık elenen kelime listesi ve
çakışma kontrolü. Yerine Yöntem bölümüne dört cümlelik eleme ölçütü notu
eklendi; markanın kendi hizmet sayfasına ait aramalar bu notta korundu.

Rapor 12 bölümden 11'e, Excel 13 sekmeden 12'ye indi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -17,9 +17,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Sezonsallık" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Mevcut Blog Performansı" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Planlanan İçerikler" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Kelime Denetimi" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Yöntem ve Kaynaklar" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Terim Sözlüğü" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Yöntem ve Kaynaklar" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Terim Sözlüğü" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,12 +94,6 @@
       <b val="1"/>
       <color rgb="0010332F"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0010332F"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="195">
@@ -1110,7 +1103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="207">
+  <cellXfs count="205">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1724,12 +1717,6 @@
     <xf numFmtId="3" fontId="9" fillId="194" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2461,2779 +2448,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="64" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Öneri kümelerinden çıkarılan kelimeler | Konu, arama niyeti ve tek anlam denetimi</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="21" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Elenen Kelime</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Aylık Arama</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Gerekçe</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Dayanak</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="61" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>13600000</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfasının ilk beş sırası Google'ın kendi Gemini adresleri; yönlendirme amaçlı marka araması.</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="61" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>imei sorgu</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>550000</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>'imei sorgula' ile aynı sonuç sayfası; araç ve hizmet sayfası araması.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-    </row>
-    <row r="6" ht="61" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>imei sorgula</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>550000</v>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası e-Devlet ve BTK sorgulama araçları ile operatörlerin hizmet sayfaları; blog içeriğinin karşılığı değil.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="61" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>konum</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>368000</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası Google Haritalar ve konum aracı; bilgi amaçlı içerik ilk sırada yer almıyor.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>google gemini</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>368000</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Aynı marka adresleri; yönlendirme amaçlı arama.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="61" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>beyaz ekran</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>İlk altı sıra beyaz ekran aracı ve uygulaması; sorun giderme içeriği ancak yedinci sıradan itibaren görünüyor.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-    </row>
-    <row r="10" ht="61" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>e posta</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>135000</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası Gmail ve Outlook giriş adresleri; yönlendirme amaçlı arama.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="74.5" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>90500</v>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">İlk on sıranın tamamı operatörlerin altyapı sorgulama hizmet sayfaları; Turkcell </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Superonline</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> sayfası da bu sırada yer alıyor.</t>
-          </r>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-    </row>
-    <row r="12" ht="61" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>alt yapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>90500</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>'altyapı sorgulama' ile aynı hizmet sayfası kümesi; yazım varyantı.</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="61" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>ekran kartı</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>60500</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası fiyat listeleri ve mağaza kategorileri; ürün arama.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14" ht="61" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>ram</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>49500</v>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası bilgisayar bileşeni satan mağazalar; ürün arama.</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-    </row>
-    <row r="15" ht="61" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>ssd</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>49500</v>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Bileşen satan mağaza sayfaları; 'ram' ve 'ekran kartı' ile aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-    </row>
-    <row r="16" ht="61" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>perplexity</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>49500</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası perplexity.ai ve site bağlantıları; yönlendirme amaçlı marka araması.</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-    </row>
-    <row r="17" ht="61" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>anakart</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Bileşen satan mağaza sayfaları; 'ram' ve 'ekran kartı' ile aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-    </row>
-    <row r="18" ht="61" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>güncellemeler</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası dağınık: uygulama mağazası yardımı, forum ve oyun videosu bir arada; tek bir arama niyeti yok.</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="61" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>internet altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Aynı hizmet sayfası kümesi.</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-    </row>
-    <row r="20" ht="61" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>fiber altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Aynı hizmet sayfası kümesi.</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="61" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>qr kod</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası QR okuyucu ve oluşturucu araçları; bilgi amaçlı içerik altıncı sıradan sonra.</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-    </row>
-    <row r="22" ht="61" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>uzantılar</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n">
-        <v>27100</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası Chrome Web Mağazası ve alan adı uzantısı içerikleri; iki ayrı anlam bir arada.</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-    </row>
-    <row r="23" ht="61" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>taşınabilir internet</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>27100</v>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>İlk iki sıra operatörlerin ev interneti ürün sayfaları; Turkcell Superbox sayfası da bu sırada.</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Ahrefs sonuç sayfası görüntüsü · Eylül 2026</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-    </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>wi-fi</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>22200</v>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Jenerik ad; tek bir arama niyeti taşımıyor.</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>wifi</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>22200</v>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Jenerik ad; tek bir arama niyeti taşımıyor.</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>bard</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>18100</v>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Farklı bir ürünün marka adı; önerinin konusuyla eşleşmiyor.</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-    </row>
-    <row r="27" ht="47.5" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>type c şarj aleti</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>18100</v>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfasının tamamı şarj cihazı satan mağazalar; ürün araması.</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>türkiye posta kodu</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Posta kodu sorgulaması e-posta konusuyla ilgili değil.</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-    </row>
-    <row r="29" ht="61" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>eklentiler</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>'uzantılar' ile aynı sınıf; mağaza yönlendirmesi.</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-    </row>
-    <row r="30" ht="61" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>eklenti</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>'uzantılar' ile aynı sınıf; mağaza yönlendirmesi.</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-    </row>
-    <row r="31" ht="34" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>sistemi</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Anlam taşımayan kelime parçası.</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-    </row>
-    <row r="32" ht="47.5" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>hosting</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası barındırma hizmeti satan sağlayıcılar; ticari arama.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-    </row>
-    <row r="33" ht="47.5" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>type c kablo</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Kablo satan mağaza sayfaları; 'type c şarj aleti' ile aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-    </row>
-    <row r="34" ht="61" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>192168.1.1</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>9900</v>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Ana kelimenin yazım varyantı; aynı sayfaya gidiyor, toplama iki kez girmemesi için çıkarıldı.</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Yazım varyantı</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-    </row>
-    <row r="35" ht="61" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>qr kodu</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>9900</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>'qr kod' ile aynı araç kümesi.</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-    </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>192.168</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n">
-        <v>8100</v>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Eksik yazılmış adres; ana kelimenin varyantı.</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Yazım varyantı</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-    </row>
-    <row r="37" ht="61" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>oem ne demek</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>6600</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Kendi kısa içerik önerisinde hedefleniyor; iki sayfanın aynı kelimede yarışmaması için güncelleme kümesinden çıkarıldı.</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Başka öneriyle çakışma</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-    </row>
-    <row r="38" ht="61" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>192.168.01</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Ana kelimenin yazım varyantı; aynı sayfaya gidiyor, toplama iki kez girmemesi için çıkarıldı.</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Yazım varyantı</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-    </row>
-    <row r="39" ht="61" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>altyapısız internet</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası operatörlerin ev interneti ürün sayfaları; blog içeriği değil.</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-    </row>
-    <row r="40" ht="61" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>taşınabilir internet fiyatları</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Fiyat araması; ürün sayfası karşılığı.</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-    </row>
-    <row r="41" ht="34" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Jenerik kısaltma; tek başına arama niyetini taşımıyor.</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-    </row>
-    <row r="42" ht="34" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>ping testi</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="n">
-        <v>4400</v>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası hız testi araçları; bilgi amaçlı içerik değil.</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-    </row>
-    <row r="43" ht="61" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>usb type c</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="n">
-        <v>4400</v>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Ürün araması; aynı sınıf. Yazının bilgi amaçlı hedefi 'type c nedir' ve 'usb-c nedir' kelimeleridir.</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-    </row>
-    <row r="44" ht="34" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>freedos nedir</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="n">
-        <v>3600</v>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Kendi kısa içerik önerisinde hedefleniyor.</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Başka öneriyle çakışma</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-    </row>
-    <row r="45" ht="34" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>type c şarj kablosu</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="n">
-        <v>3600</v>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Ürün araması; aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-    </row>
-    <row r="46" ht="34" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>type c adaptör</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="n">
-        <v>3600</v>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Ürün araması; aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-    </row>
-    <row r="47" ht="61" customHeight="1">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>otomatik güncellemeler</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="n">
-        <v>2900</v>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>'güncellemeler' ile aynı dağınık sonuç sayfası.</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-    </row>
-    <row r="48" ht="47.5" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>mac ne demek</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="n">
-        <v>2900</v>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Mac bilgisayar ve MAC adresi anlamları bir arada; tek anlam koşulunu sağlamıyor.</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-    </row>
-    <row r="49" ht="74.5" customHeight="1">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>apple arcade</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası Apple'ın kendi hizmet adresi; yönlendirme amaçlı marka araması. Yazının hedefi 'apple arcade nedir' kelimesidir.</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-    </row>
-    <row r="50" ht="61" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>fiber internet altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Aynı hizmet sayfası kümesi.</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-    </row>
-    <row r="51" ht="34" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>mesh wifi</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası mesh cihaz satışı; ticari arama.</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-    </row>
-    <row r="52" ht="34" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>usb c kablo</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Ürün araması; aynı sınıf.</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
-    </row>
-    <row r="53" ht="34" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>puk</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="n">
-        <v>1900</v>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Jenerik kısaltma; tek başına arama niyetini taşımıyor.</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
-    </row>
-    <row r="54" ht="61" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>ttnet fiber altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="n">
-        <v>1600</v>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Aynı hizmet sayfası kümesi; ayrıca rakip marka adı taşıyor.</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-    </row>
-    <row r="55" ht="34" customHeight="1">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>oem nedir</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="n">
-        <v>1600</v>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>Kendi kısa içerik önerisinde hedefleniyor.</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Başka öneriyle çakışma</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-    </row>
-    <row r="56" ht="47.5" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>gizli dns sunucusuna erişilemiyor</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="n">
-        <v>1300</v>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>DNS hata giderme ayrı bir konu; barındırma içeriğiyle eşleşmiyor.</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-    </row>
-    <row r="57" ht="34" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>dns sunucusu yanıt vermiyor</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="n">
-        <v>1300</v>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>DNS hata giderme ayrı bir konu.</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
-    </row>
-    <row r="58" ht="34" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>adsl modem</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="n">
-        <v>1300</v>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Cihaz araması.</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
-    </row>
-    <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>vdsl internet</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="n">
-        <v>1300</v>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>Hizmet ve tarife araması; bilgilendirici yazı hedefi değil.</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
-    </row>
-    <row r="60" ht="34" customHeight="1">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>mesh modem</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>Cihaz araması.</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
-    </row>
-    <row r="61" ht="61" customHeight="1">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>eposta</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="n">
-        <v>880</v>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>Yönlendirme amaçlı arama; 'e posta' ile aynı sonuç sayfası.</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>Aynı sınıftaki kelimeyle örtüşen sonuç sayfası</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-    </row>
-    <row r="62" ht="47.5" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t>airtag kedi tasması</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="n">
-        <v>880</v>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Ürün aksesuarı araması; AirTag tanımı sorusundan ayrı bir niyet.</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
-    </row>
-    <row r="63" ht="47.5" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>işletim sistemleri hakkında aşağıdakilerden hangisi doğru değildir</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="n">
-        <v>390</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Sınav sorusu araması; içerikle karşılanmıyor.</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="n"/>
-    </row>
-    <row r="64" ht="34" customHeight="1">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>mac ne</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>320</v>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Anlam taşımayan kelime parçası.</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="n"/>
-    </row>
-    <row r="65" ht="34" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>işletim sistemleri sadece bilgisayarlara özgü müdür</t>
-        </is>
-      </c>
-      <c r="B65" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Sınav sorusu araması; içerikle karşılanmıyor.</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>Konu ve niyet eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
-    </row>
-    <row r="66" ht="34" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>wifi şifresi kırma</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Yetkisiz erişim araması; marka içeriğine uygun değil.</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-    </row>
-    <row r="67" ht="34" customHeight="1">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>instagram mavi tik nasıl alınır</t>
-        </is>
-      </c>
-      <c r="B67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Hesap doğrulama başvurusu ayrı bir konu; küme dışında.</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>Konu eşleşmesi</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="n"/>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="2" t="n"/>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="205" t="inlineStr">
-        <is>
-          <t>Öneri kümelerindeki değişim</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="n"/>
-    </row>
-    <row r="70" ht="36" customHeight="1">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t>Değişim</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>Öneri</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>Başlık</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>Önceki Aylık Arama</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Sonraki Aylık Arama</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>Gerekçe</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="34" customHeight="1">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Modem Arayüzüne Giriş ve Modem Şifresi Değiştirme</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="n">
-        <v>454420</v>
-      </c>
-      <c r="E71" s="7" t="n">
-        <v>483870</v>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı. Havuzdan niteleyici kelime eklendi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="34" customHeight="1">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>Konum Paylaşma ve Numaradan Konum Bulma</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="n">
-        <v>415080</v>
-      </c>
-      <c r="E72" s="7" t="n">
-        <v>47080</v>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="47.5" customHeight="1">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>öneri kaldırıldı</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>İnternet Altyapı Sorgulama: Adrese Göre Hız ve Teknoloji Kontrolü</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="n">
-        <v>256600</v>
-      </c>
-      <c r="E73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Kümenin tamamı operatör hizmet sayfası aramasıdır; blog içeriğiyle karşılanmıyor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="34" customHeight="1">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>P18</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>SSD, RAM ve Ekran Kartı: Bilgisayar Donanımı Rehberi</t>
-        </is>
-      </c>
-      <c r="D74" s="7" t="n">
-        <v>218620</v>
-      </c>
-      <c r="E74" s="7" t="n">
-        <v>26020</v>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="34" customHeight="1">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>öneri kaldırıldı</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Telefonda Beyaz Ekran, Siyah Ekran ve Donma Sorunları</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="n">
-        <v>166000</v>
-      </c>
-      <c r="E75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>Hacmin tamamı beyaz ekran aracı aramasından geliyordu; niteleyici kelime havuzda bulunmuyor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="34" customHeight="1">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Gizli Numara: Arama, Kapatma ve Numara Gizleme Ayarları</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="n">
-        <v>323300</v>
-      </c>
-      <c r="E76" s="7" t="n">
-        <v>327700</v>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı. Havuzdan niteleyici kelime eklendi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="47.5" customHeight="1">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>Yurt Dışından Getirilen Telefonun IMEI Kaydı: Ücret, Süre ve Adımlar</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="n">
-        <v>1264130</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>169430</v>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı. Havuzdan niteleyici kelime eklendi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="34" customHeight="1">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>P16</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>E-Posta Kurulumu ve Yönetimi: Hesap Açma, Aktarma, Güvenlik</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="n">
-        <v>165780</v>
-      </c>
-      <c r="E78" s="7" t="n">
-        <v>15100</v>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="34" customHeight="1">
-      <c r="A79" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>PUK, PIN ve SIM Kilidi: Kod Öğrenme ve Kilit Açma</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="n">
-        <v>67200</v>
-      </c>
-      <c r="E79" s="7" t="n">
-        <v>65300</v>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="34" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
-        <is>
-          <t>öneri bölündü</t>
-        </is>
-      </c>
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>K9</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Tarayıcı Eklentileri ve Güncellemeleri Yönetme</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="n">
-        <v>125880</v>
-      </c>
-      <c r="E80" s="7" t="n">
-        <v>33180</v>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>Küme iki ayrı soruyu bir arada taşıyordu; her soru kendi kısa içeriğine ayrıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="34" customHeight="1">
-      <c r="A81" s="6" t="inlineStr">
-        <is>
-          <t>öneri kaldırıldı</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>QR Kod: Okutma, Oluşturma ve Güvenlik Riskleri</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="n">
-        <v>47400</v>
-      </c>
-      <c r="E81" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>Küme QR okuyucu ve oluşturucu aracı aramasından oluşuyordu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="34" customHeight="1">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>öneri kaldırıldı</t>
-        </is>
-      </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>K10</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>Perplexity Nedir? Yapay Zeka Arama Motoru</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="n">
-        <v>67600</v>
-      </c>
-      <c r="E82" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" s="4" t="inlineStr">
-        <is>
-          <t>İki kelime de marka yönlendirmesi; tanım araması havuzda yer almıyor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="34" customHeight="1">
-      <c r="A83" s="6" t="inlineStr">
-        <is>
-          <t>öneri kaldırıldı</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Taşınabilir İnternet ve Mobil WiFi Cihazları</t>
-        </is>
-      </c>
-      <c r="D83" s="7" t="n">
-        <v>32500</v>
-      </c>
-      <c r="E83" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>İki kelime de ev interneti ürün sayfası aramasıdır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="34" customHeight="1">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>K5</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>AirTag Nedir ve Nasıl Kullanılır?</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="n">
-        <v>21580</v>
-      </c>
-      <c r="E84" s="7" t="n">
-        <v>20700</v>
-      </c>
-      <c r="F84" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="20.5" customHeight="1">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>küme daraltıldı</t>
-        </is>
-      </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>K22</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Apple Arcade Nedir?</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="n">
-        <v>9000</v>
-      </c>
-      <c r="E85" s="7" t="n">
-        <v>6600</v>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="34" customHeight="1">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>güncelleme kümesi daraltıldı</t>
-        </is>
-      </c>
-      <c r="B86" s="4" t="inlineStr">
-        <is>
-          <t>gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="n">
-        <v>14045400</v>
-      </c>
-      <c r="E86" s="7" t="n">
-        <v>77400</v>
-      </c>
-      <c r="F86" s="4" t="inlineStr">
-        <is>
-          <t>Niyeti eşleşmeyen ya da başka öneriyle çakışan kelimeler çıkarıldı.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="2" t="n"/>
-      <c r="D87" s="2" t="n"/>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="n"/>
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="n"/>
-      <c r="D88" s="2" t="n"/>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="n"/>
-    </row>
-    <row r="89" ht="34" customHeight="1">
-      <c r="A89" s="206" t="inlineStr">
-        <is>
-          <t>Çakışma ve cannibalization kontrolü</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="n"/>
-    </row>
-    <row r="90" ht="21" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>Kontrol</t>
-        </is>
-      </c>
-      <c r="B90" s="5" t="inlineStr">
-        <is>
-          <t>Nasıl yapıldı</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>Sonuç</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="n"/>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n"/>
-    </row>
-    <row r="91" ht="47.5" customHeight="1">
-      <c r="A91" s="4" t="inlineStr">
-        <is>
-          <t>Öneri hedef kelimesi mevcut bir yazının arama sorgusuyla örtüşüyor mu?</t>
-        </is>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>37 önerinin hedef kelimeleri blogun 4.917 satırlık sorgu verisiyle karşılaştırıldı</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="inlineStr">
-        <is>
-          <t>Bulgu yok</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
-    </row>
-    <row r="92" ht="47.5" customHeight="1">
-      <c r="A92" s="4" t="inlineStr">
-        <is>
-          <t>Öneri, markanın kendi hizmet ya da ürün sayfasıyla yarışıyor mu?</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>Yüksek hacimli kelimelerin sonuç sayfası tek tek görüntülendi</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>11 kelime havuzdan çıkarıldı</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
-    </row>
-    <row r="93" ht="47.5" customHeight="1">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>Yeni öneri, blogda yayında olan bir yazının konusunu tekrarlıyor mu?</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>Havuzdaki her arama 196 yayındaki yazının konusuyla karşılaştırıldı</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>4 arama yeni yazı yerine güncelleme kapsamına bırakıldı</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="n"/>
-      <c r="E93" s="2" t="n"/>
-      <c r="F93" s="2" t="n"/>
-    </row>
-    <row r="94" ht="47.5" customHeight="1">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t>Önerilen başlık, yayındaki bir başlığın benzeri mi?</t>
-        </is>
-      </c>
-      <c r="B94" s="4" t="inlineStr">
-        <is>
-          <t>Her öneri başlığı 196 yazının başlığıyla karakter benzerliği üzerinden karşılaştırıldı (eşik 0.72)</t>
-        </is>
-      </c>
-      <c r="C94" s="6" t="inlineStr">
-        <is>
-          <t>2 bulgu</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="n"/>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="2" t="n"/>
-    </row>
-    <row r="95" ht="34" customHeight="1">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>İki öneri aynı kelimeyi hedefliyor mu?</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>Kelime sahipliği tüm öneri kümelerinde karşılaştırıldı</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>Bulgu yok</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="n"/>
-      <c r="E95" s="2" t="n"/>
-      <c r="F95" s="2" t="n"/>
-    </row>
-    <row r="96" ht="47.5" customHeight="1">
-      <c r="A96" s="4" t="inlineStr">
-        <is>
-          <t>Bir kelime hem yeni öneride hem güncellemede hedefleniyor mu?</t>
-        </is>
-      </c>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t>Öneri ve güncelleme kümeleri karşılaştırıldı</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>Bulgu yok</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="n"/>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="2" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="n"/>
-      <c r="B97" s="2" t="n"/>
-      <c r="C97" s="2" t="n"/>
-      <c r="D97" s="2" t="n"/>
-      <c r="E97" s="2" t="n"/>
-      <c r="F97" s="2" t="n"/>
-    </row>
-    <row r="98" ht="21" customHeight="1">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>Bulgu Tipi</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>İlgili Öğe</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>Kelime</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>Hacim</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>Karşılık</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>Karar</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20.5" customHeight="1">
-      <c r="A99" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>imei sorgu</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="n">
-        <v>550000</v>
-      </c>
-      <c r="E99" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F99" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="20.5" customHeight="1">
-      <c r="A100" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B100" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C100" s="6" t="inlineStr">
-        <is>
-          <t>imei sorgula</t>
-        </is>
-      </c>
-      <c r="D100" s="7" t="n">
-        <v>550000</v>
-      </c>
-      <c r="E100" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F100" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="20.5" customHeight="1">
-      <c r="A101" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="inlineStr">
-        <is>
-          <t>altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D101" s="7" t="n">
-        <v>90500</v>
-      </c>
-      <c r="E101" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F101" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="20.5" customHeight="1">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B102" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C102" s="6" t="inlineStr">
-        <is>
-          <t>alt yapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D102" s="7" t="n">
-        <v>90500</v>
-      </c>
-      <c r="E102" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F102" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="20.5" customHeight="1">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C103" s="6" t="inlineStr">
-        <is>
-          <t>internet altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D103" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="E103" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F103" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="20.5" customHeight="1">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr">
-        <is>
-          <t>fiber altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D104" s="7" t="n">
-        <v>33100</v>
-      </c>
-      <c r="E104" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F104" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="20.5" customHeight="1">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr">
-        <is>
-          <t>taşınabilir internet</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="n">
-        <v>27100</v>
-      </c>
-      <c r="E105" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F105" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="20.5" customHeight="1">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B106" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr">
-        <is>
-          <t>altyapısız internet</t>
-        </is>
-      </c>
-      <c r="D106" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="E106" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F106" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="20.5" customHeight="1">
-      <c r="A107" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B107" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C107" s="6" t="inlineStr">
-        <is>
-          <t>taşınabilir internet fiyatları</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="n">
-        <v>5400</v>
-      </c>
-      <c r="E107" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F107" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="34" customHeight="1">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>fiber internet altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="n">
-        <v>2400</v>
-      </c>
-      <c r="E108" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F108" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="20.5" customHeight="1">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>Markanın kendi sayfası</t>
-        </is>
-      </c>
-      <c r="B109" s="4" t="inlineStr">
-        <is>
-          <t>öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>ttnet fiber altyapı sorgulama</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="n">
-        <v>1600</v>
-      </c>
-      <c r="E109" s="4" t="inlineStr">
-        <is>
-          <t>Turkcell hizmet ya da ürün sayfası</t>
-        </is>
-      </c>
-      <c r="F109" s="4" t="inlineStr">
-        <is>
-          <t>Kelime blog kümesinden çıkarıldı; hedefi ilgili hizmet sayfasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="34" customHeight="1">
-      <c r="A110" s="6" t="inlineStr">
-        <is>
-          <t>Mevcut yazının kapsamı</t>
-        </is>
-      </c>
-      <c r="B110" s="4" t="inlineStr">
-        <is>
-          <t>yeni öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C110" s="6" t="inlineStr">
-        <is>
-          <t>internet neden yavaş</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="n">
-        <v>6400</v>
-      </c>
-      <c r="E110" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/internet-neden-yavasladi-sorunun-kaynagini-adim-adim-bulma-rehberi</t>
-        </is>
-      </c>
-      <c r="F110" s="4" t="inlineStr">
-        <is>
-          <t>Yeni yazı önerilmedi; kelime mevcut yazının güncelleme kapsamına bırakıldı</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="34" customHeight="1">
-      <c r="A111" s="6" t="inlineStr">
-        <is>
-          <t>Mevcut yazının kapsamı</t>
-        </is>
-      </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>yeni öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>internet neden yok</t>
-        </is>
-      </c>
-      <c r="D111" s="7" t="n">
-        <v>7700</v>
-      </c>
-      <c r="E111" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/internet-neden-yavasladi-sorunun-kaynagini-adim-adim-bulma-rehberi</t>
-        </is>
-      </c>
-      <c r="F111" s="4" t="inlineStr">
-        <is>
-          <t>Yeni yazı önerilmedi; kelime mevcut yazının güncelleme kapsamına bırakıldı</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="34" customHeight="1">
-      <c r="A112" s="6" t="inlineStr">
-        <is>
-          <t>Mevcut yazının kapsamı</t>
-        </is>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>yeni öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C112" s="6" t="inlineStr">
-        <is>
-          <t>vpn nasıl açılır</t>
-        </is>
-      </c>
-      <c r="D112" s="7" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E112" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/dijital-guvenligin-temel-bileseni-vpn-nedir</t>
-        </is>
-      </c>
-      <c r="F112" s="4" t="inlineStr">
-        <is>
-          <t>Yeni yazı önerilmedi; kelime mevcut yazının güncelleme kapsamına bırakıldı</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="34" customHeight="1">
-      <c r="A113" s="6" t="inlineStr">
-        <is>
-          <t>Mevcut yazının kapsamı</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>yeni öneri havuzu</t>
-        </is>
-      </c>
-      <c r="C113" s="6" t="inlineStr">
-        <is>
-          <t>chatgpt ücretli mi</t>
-        </is>
-      </c>
-      <c r="D113" s="7" t="n">
-        <v>3900</v>
-      </c>
-      <c r="E113" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/chatgpt-nedir-adim-adim-chatgpt-kullanma-rehberi</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>Yeni yazı önerilmedi; kelime mevcut yazının güncelleme kapsamına bırakıldı</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="34" customHeight="1">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>Başlık benzerliği</t>
-        </is>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t>K15 · URL Nedir?</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D114" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/crm-nedir</t>
-        </is>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>Yalnız 'X nedir' başlık kalıbı benzeşmektedir; konular farklı olduğu için çakışma bulunmamaktadır</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="34" customHeight="1">
-      <c r="A115" s="6" t="inlineStr">
-        <is>
-          <t>Başlık benzerliği</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>K15 · URL Nedir?</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E115" s="14" t="inlineStr">
-        <is>
-          <t>https://www.turkcell.com.tr/blog/unix-nedir</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>Yalnız 'X nedir' başlık kalıbı benzeşmektedir; konular farklı olduğu için çakışma bulunmamaktadır</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="n"/>
-      <c r="B116" s="2" t="n"/>
-      <c r="C116" s="2" t="n"/>
-      <c r="D116" s="2" t="n"/>
-      <c r="E116" s="2" t="n"/>
-      <c r="F116" s="2" t="n"/>
-    </row>
-    <row r="117" ht="81" customHeight="1">
-      <c r="A117" s="3" t="inlineStr">
-        <is>
-          <t>YÖNTEM</t>
-        </is>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>Bir kelime öneri kümesinde ancak üç koşulu birlikte sağladığında kalmaktadır: kelimenin önerinin konusunu niteleyerek adlandırması, sonuç sayfasının bilgi amaçlı içerikle karşılanması ve kelimenin ikinci bir yaygın anlamının bulunmaması. Alışveriş listesi, giriş sayfası, sorgulama aracı ya da markanın kendi hizmet sayfasıyla karşılanan kelimeler blog kümesine alınmamıştır.</t>
-        </is>
-      </c>
-      <c r="C117" s="12" t="n"/>
-      <c r="D117" s="12" t="n"/>
-      <c r="E117" s="2" t="n"/>
-      <c r="F117" s="2" t="n"/>
-    </row>
-    <row r="118" ht="51" customHeight="1">
-      <c r="A118" s="3" t="inlineStr">
-        <is>
-          <t>DAYANAK</t>
-        </is>
-      </c>
-      <c r="B118" s="4" t="inlineStr">
-        <is>
-          <t>Sonuç sayfası kontrolü Ahrefs görüntüsüyle yapılmıştır (Eylül 2026). Doğrudan görüntülenen kelimeler 'Ahrefs sonuç sayfası görüntüsü', aynı sınıfa giren kelimeler 'Aynı sınıftaki kelimeyle örtüşen sonuç sayfası' olarak işaretlenmiştir.</t>
-        </is>
-      </c>
-      <c r="C118" s="12" t="n"/>
-      <c r="D118" s="12" t="n"/>
-      <c r="E118" s="2" t="n"/>
-      <c r="F118" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B118:D118"/>
-    <mergeCell ref="B117:D117"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId6"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5342,7 +2556,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="51" customHeight="1">
+    <row r="7" ht="81" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>KELİME DENETİMİ</t>
@@ -5350,7 +2564,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Her kelime konu, arama niyeti ve tek anlam koşullarına göre denetlenmiştir. Sonuç sayfası alışveriş listesi, giriş sayfası, sorgulama aracı ya da markanın kendi hizmet sayfasıyla karşılanan kelimeler kümelerden çıkarılmıştır; elenen kelimeler ve gerekçeleri 11 Kelime Denetimi sekmesindedir.</t>
+          <t>Her kelime konu, arama niyeti ve tek anlam koşullarına göre denetlenmiştir. Sonuç sayfası alışveriş listesi, giriş sayfası, sorgulama aracı ya da markanın kendi hizmet sayfasıyla karşılanan kelimeler kümelerden çıkarılmıştır; Bu ölçütle elenen kelimelerin bir bölümünde hedef sayfa blog değil, markanın kendi hizmet ya da ürün sayfasıdır: imei sorgulama, altyapı sorgulama ve taşınabilir internet aramaları bu gruptadır. Önerilerin yayındaki yazılarla ve birbiriyle çakışmadığı ayrıca denetlenmiştir.</t>
         </is>
       </c>
     </row>
@@ -5458,7 +2672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10559,7 +7773,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t xml:space="preserve"> bloglarının sıraladığı, blogun yer almadığı kelimelerden seçilmiştir. Her kelime konu ve arama niyeti denetiminden geçirilmiştir; elenen kelimeler 11 Kelime Denetimi sekmesinde gerekçesiyle listelenmiştir. Bir kelime tek öneriye aittir; varyantlar toplama dahil edilmemiştir.</t>
+            <t xml:space="preserve"> bloglarının sıraladığı, blogun yer almadığı kelimelerden seçilmiştir. Her kelime konu ve arama niyeti denetiminden geçirilmiştir; eleme ölçütü 11 Yöntem ve Kaynaklar sekmesinde açıklanmıştır. Bir kelime tek öneriye aittir; varyantlar toplama dahil edilmemiştir.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Güncelleme yönergeleri veriye bağlanarak yeniden yazıldı
On yazının yönergesi genel geçer maddelerden çıkarılıp her maddesi bir
dayanağa bağlandı: Search Console sorgusu ve sırası, rakip yazının yapısı
ya da gövdede karşılığı bulunmayan kelime. Ne yapılacağı somut yazıldı
(hangi başlık, kaç kırılım, tabloda hangi sütunlar).

Alt başlık önerileri ayrı alandan üretiliyor; rakip başlık farkı
listesinden gezinme blokları süzüldü.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -8129,7 +8129,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="142" customHeight="1">
+    <row r="4" ht="291" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/isletim-sistemi-nedir-ve-cesitleri-nelerdir</t>
@@ -8231,9 +8231,9 @@
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>1. Mobil işletim sistemleri bölümü genişletilebilir
-2. Windows, macOS ve Linux karşılaştırması tablo hâlinde verilebilir
-3. FreeDOS ve işletim sistemsiz cihaz bölümü eklenebilir
+          <t>1. Windows, macOS ve Linux Karşılaştırması
+2. İşletim Sistemi Yalnız Bilgisayarlarda mı Bulunur?
+3. Android ve iOS Arasındaki Farklar
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: İşletim Sistemi Özellikleri Nelerdir?</t>
         </is>
       </c>
@@ -8268,14 +8268,16 @@
       </c>
       <c r="X4" s="4" t="inlineStr">
         <is>
-          <t>1. Mobil işletim sistemleri bölümü genişletilebilir
-2. Windows, macOS ve Linux karşılaştırması tablo hâlinde verilebilir
-3. FreeDOS ve işletim sistemsiz cihaz bölümü eklenebilir</t>
+          <t>1. 'Windows nedir' sorgusu 1.059 Impression alıyor ancak sayfa 9.7 ortalama sırada kalıyor; Windows, macOS ve Linux için üç ayrı H3 açılıp her birine sürüm adı, tipik kullanıcı profili ve donanım gereksinimi yazılabilir
+2. 'işletim sistemleri sadece bilgisayarlara özgü müdür' sorgusu 646 Impression ile 3.2 sırada geliyor, yani soru soruluyor ama yanıt bölümü yok: telefon, akıllı televizyon, akıllı saat ve araç sistemlerini kapsayan 'İşletim Sistemi Yalnız Bilgisayarlarda mı Bulunur?' başlığı eklenebilir
+3. Mobil tarafta Android ve iOS tek cümlede geçiyor; ikisi ayrı H3 olarak açılıp aralarındaki uygulama mağazası, güncelleme ve donanım farkı üç maddeyle verilebilir
+4. 'bilgisayar işletim sistemleri' ve 'işletim sistemleri nelerdir' kelimeleri gövdede hiç geçmiyor; mevcut 'İşletim Sistemi Çeşitleri Nelerdir?' başlığının açılış cümlesi bu iki kalıbı da karşılayacak biçimde yazılabilir
+5. 'işletim sistemleri hakkında aşağıdakilerden hangisi doğru değildir' sorgusu 4.221 Impression alıyor ve ödev kaynaklı; bu sorguya içerik yazılması önerilmez, ölçüm okunurken hesaba katılması yeterlidir açıklanır</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
         <is>
-          <t>Sorgu eğitim amaçlı arama da içermektedir; tanım bölümü kısa ve alıntılanabilir tutulabilir.</t>
+          <t>Sürüm adları ve donanım gereksinimleri yıl içinde değişiyor; güncellenme tarihinin görünür tutulması bu yazıda değer taşıyor.</t>
         </is>
       </c>
       <c r="Z4" s="7" t="n">
@@ -8295,7 +8297,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="128.5" customHeight="1">
+    <row r="5" ht="261" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar</t>
@@ -8402,10 +8404,10 @@
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>1. Hosting türleri karşılaştırması eklenebilir
-2. Domain ile ilişkisi açıklanabilir
-3. Küçük işletme için seçim kriterleri bölümü eklenebilir
-Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Hosting Nedir? Hangi Hizmetleri Sağlar? · İlginizi Çekebilir</t>
+          <t>1. Hosting Türleri Karşılaştırma Tablosu
+2. Domain ve Hosting Ayrı Ayrı mı Alınır?
+3. Küçük İşletme İçin Hangi Hosting Seçilir?
+Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Hosting Nedir? Hangi Hizmetleri Sağlar?</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
@@ -8439,14 +8441,39 @@
       </c>
       <c r="X5" s="4" t="inlineStr">
         <is>
-          <t>1. Hosting türleri karşılaştırması eklenebilir
-2. Domain ile ilişkisi açıklanabilir
-3. Küçük işletme için seçim kriterleri bölümü eklenebilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. Sayfa 'hosting' sorgusunda 31.2 ortalama sırada; bu sorguda ilk sayfaya girebilmek için mevcut 'Hosting Türleri Nelerdir?' başlığı tabloya çevrilebilir: paylaşımlı, VPS, bulut ve adanmış sunucu satırlarında kaynak paylaşımı, tipik trafik kapasitesi ve kimin için uygun olduğu üç sütunda verilir
+2. 'domain ve hosting nedir' sorgusu 4.6 sırada 409 Impression alıyor; mevcut fark bölümü iki cümlede kalıyor, alan adı ile barındırmanın ilişkisi bir örnek üzerinden anlatılıp 'ikisi ayrı ayrı mı alınır' sorusu yanıtlanabilir
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Türk Telekom</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un aynı sorguda 3. sıradaki yazısı 1.239 kelime ve konuyu tek uzun bölümde veriyor; bizim yazımız 12 ara başlıkla daha ayrıntılı, eksik olan derinlik değil seçim kriteri: 'Küçük İşletme İçin Hangi Hosting Seçilir?' başlığı altında aylık ziyaretçi bandına göre üç senaryo eklenebilir
+4. 'turkcell host' sorgusu 399 Impression ile 5.1 sırada geliyor; markanın barındırma hizmetine tek cümlelik bir bağlantı, arama niyetini karşılar açıklanır</t>
+          </r>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
         <is>
-          <t>Sonuç sayfası ticari hizmet sayfalarından oluşmaktadır; açıklama yazısının ilk sıraya çıkması yapısal olarak sınırlıdır.</t>
+          <t>Fiyat bilgisi verilmemesi, kapasite ve kullanım senaryosu üzerinden anlatılması önerilir.</t>
         </is>
       </c>
       <c r="Z5" s="7" t="n">
@@ -8466,7 +8493,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="250" customHeight="1">
+    <row r="6" ht="261" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/nfc-nedir-nfc-ile-neler-yapilabilir</t>
@@ -8582,12 +8609,37 @@
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>1. NFC özelliğinin telefonda nasıl açıldığı marka bazında eklenebilir
-2. IPhone ve Android ayrımı ara başlığa çıkarılabilir
-3. NFC destekleyen telefon listesi eklenebilir
-4. Temassız ödeme bölümü genişletilebilir
-5. NFC etiketi kullanımı eklenebilir
-Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: NFC Nedir, NFC ile Neler Yapılabilir? · İlginizi Çekebilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. NFC Etiketi Nedir, Ne İşe Yarar?
+2. NFC Kart Nedir?
+3. iPhone'da NFC Nasıl Açılır?
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Samsung</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve"> ve Xiaomi Cihazlarda NFC Nasıl Açılır?
+5. NFC Destekleyen Telefon Modelleri
+6. Telefonda NFC Anteni Nerede Bulunur?
+Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: NFC Nedir, NFC ile Neler Yapılabilir?</t>
+          </r>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
@@ -8655,16 +8707,40 @@
       </c>
       <c r="X6" s="4" t="inlineStr">
         <is>
-          <t>1. NFC özelliğinin telefonda nasıl açıldığı marka bazında eklenebilir
-2. IPhone ve Android ayrımı ara başlığa çıkarılabilir
-3. NFC destekleyen telefon listesi eklenebilir
-4. Temassız ödeme bölümü genişletilebilir
-5. NFC etiketi kullanımı eklenebilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. 'nfc etiketi nedir' sorgusu 3.835 Impression alıyor ancak sayfa 8.7 sırada ve tek click getiriyor; yazıda NFC etiketi hiç geçmiyor. 'NFC Etiketi Nedir, Ne İşe Yarar?' başlığı altında etiketin ne olduğu, telefona nasıl okutulduğu ve ev otomasyonu gibi kullanım örnekleri verilebilir
+2. 'nfc kart nedir' 832 Impression alıyor; temassız kartın NFC ile ilişkisi ayrı bir H3 olarak açılabilir
+3. 'nfc açma', 'iphone nfc açma', 'apple nfc açma' ve 'nfc özelliği nasıl açılır redmi' kelimelerinin hiçbiri gövdede geçmiyor; mevcut 'NFC Nasıl Açılır ve Kullanılır?' başlığı cihaz bazında üçe ayrılabilir: iPhone, </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Samsung</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve"> ve Xiaomi/Redmi. Her biri iki-üç adımla anlatılır
+4. 'nfc özelliği olan telefonlar' kelimesi gövdede yok; NFC destekleyen model ailelerini marka bazında listeleyen kısa bir tablo, bu aramayı karşılar açıklanır
+5. 'nfc alanı neresi' aramasının karşılığı da bulunmuyor; NFC anteninin telefonun neresinde olduğu ve nasıl bulunacağı tek paragrafla eklenebilir</t>
+          </r>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
         <is>
-          <t>Bankaların ödeme niyetli sayfaları önde olduğundan, ödeme bölümü tek başına yeterli olmayabilir; cihaz ayarları katmanı ayırt edici olmaktadır.</t>
+          <t>Cihaz arayüzleri sürümle değişiyor; adımların model ailesi düzeyinde verilmesi ve güncellenme tarihinin görünür tutulması önerilir.</t>
         </is>
       </c>
       <c r="Z6" s="7" t="n">
@@ -8684,7 +8760,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="263.5" customHeight="1">
+    <row r="7" ht="276" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis</t>
@@ -8778,11 +8854,9 @@
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>1. Yazının hedefi jenerik marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek'
-2. Kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma
-3. ChatGPT ile karşılaştırma tablosu eklenebilir
-4. Ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir
-5. Sık sorulanlar bölümü, sonuç sayfasında görünen soru bloğuyla eşleştirilebilir
+          <t>1. Gemini Türkçe Destekliyor mu?
+2. Gemini ile ChatGPT Arasındaki Fark
+3. Gemini Ücretsiz mi?
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Google Gemini Nedir? · Peki, Gemini’yi Kim Geliştirdi? · Gemini’ye Nasıl Ulaşılabilir? · Peki Gemini’nin GPT’den Farkı Ne?</t>
         </is>
       </c>
@@ -8805,16 +8879,16 @@
       </c>
       <c r="X7" s="4" t="inlineStr">
         <is>
-          <t>1. Yazının hedefi jenerik marka aramasından uzun kuyruğa taşınabilir: 'gemini nedir', 'gemini yapay zeka', 'gemini ne demek' açıklanır
-2. Kullanım senaryoları bölümü eklenebilir: telefonda kullanım, dosya yükleme, görsel oluşturma adım adım anlatılır
-3. ChatGPT ile karşılaştırma tablosu eklenebilir
-4. Ücretsiz ve ücretli sürüm farkı ayrı ara başlıkta verilebilir
-5. Sık sorulanlar bölümü, sonuç sayfasında görünen soru bloğuyla eşleştirilebilir</t>
+          <t>1. 'gemini yapay zeka' sorgusu 92.496 Impression ile 79 click getiriyor ve kelime gövdede hiç geçmiyor; giriş paragrafında ve bir ara başlıkta bu kalıbın kullanılması, sayfanın hâlihazırda göründüğü aramayı güçlendirir açıklanır
+2. 'gemini türkçe' kelimesi de gövdede yok; 'Gemini Türkçe Destekliyor mu?' başlığı altında dil desteği, Türkçe yanıt kalitesi ve arayüz dili üç maddeyle verilebilir
+3. Mevcut 'Gemini ile Bard Arasındaki Fark' bölümü artık geçerliliğini yitiriyor, Bard adı kullanımdan kalktı; bu bölüm 'Gemini ile ChatGPT Arasındaki Fark' karşılaştırmasına çevrilip yanıt kaynağı, görsel üretimi, dosya yükleme ve ücretsiz sürüm sınırları dört satırlık tabloya alınabilir
+4. Ücretsiz ve ücretli sürüm ayrımı yazıda geçmiyor; 'Gemini Ücretsiz mi?' başlığı, sonuç sayfasındaki soru bloğunda da görünen bir arama adım adım anlatılır
+5. Sayfanın Impression'ı jenerik marka aramasından geliyor ve o aramada sonuç sayfasının ilk beş sırası Google'ın kendi adresleri; kazanım kullanım ve karşılaştırma sorularında olduğu için yeni bölümler bu iki eksende kurgulanmalıdır</t>
         </is>
       </c>
       <c r="Y7" s="4" t="inlineStr">
         <is>
-          <t>Yazının impression'ı jenerik marka aramasından gelmektedir ve bu aramada sonuç sayfasının üst sıraları Google'ın kendi mülkleridir; CTR'ın bu aramada yükselmesi beklenmemelidir. Kazanım uzun kuyruk sorularındadır.</t>
+          <t>Yapay zeka ürünlerinde sürüm ve fiyatlandırma sık değişiyor; tablo değerlerinin tarihiyle birlikte verilmesi önerilir.</t>
         </is>
       </c>
       <c r="Z7" s="7" t="n">
@@ -8834,7 +8908,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="142" customHeight="1">
+    <row r="8" ht="261" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/ping-internette-gecikmenin-gercek-nedeni</t>
@@ -8930,10 +9004,10 @@
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>1. Ping değerinin ne olduğu ve ideal aralık tablo hâlinde verilebilir
-2. Ping düşürme adımları eklenebilir
-3. Oyun senaryosu ayrı ara başlığa alınabilir
-Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Ping Testi Nedir? Nasıl Yapılır? · İlginizi Çekebilir</t>
+          <t>1. Ping Testi Nasıl Yapılır?
+2. İdeal Ping Değerleri Tablosu
+3. Ping Nasıl Düşürülür? Dört Adım
+Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Ping Testi Nedir? Nasıl Yapılır?</t>
         </is>
       </c>
       <c r="V8" s="4" t="inlineStr">
@@ -8984,14 +9058,39 @@
       </c>
       <c r="X8" s="4" t="inlineStr">
         <is>
-          <t>1. Ping değerinin ne olduğu ve ideal aralık tablo hâlinde verilebilir
-2. Ping düşürme adımları eklenebilir
-3. Oyun senaryosu ayrı ara başlığa alınabilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Türk Telekom</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un aynı konudaki yazısının başlığı 'Ping Testi Nedir? Nasıl Yapılır?'; bizim yazımızda ölçüm bölümü var ancak test adımı yok. Komut satırından ping testi, hız testi siteleri ve oyun içi gecikme göstergesi üç adımda anlatılabilir
+2. 'ping nedir' sorgusunda sayfa 3.7 ortalama sırada ancak 3.918 Impression'dan yalnız 1 click geliyor; bu tablo sonuç sayfasının üstünde yanıtın verildiğine işaret ediyor. Giriş paragrafındaki tanımın tek cümleye indirilmesi ve ideal ping aralığının hemen altına tablo olarak konması, alıntılanma ihtimalini artırır açıklanır
+3. Ideal değer aralığı yazıda cümle içinde geçiyor; 'Rekabetçi oyun 0-30 ms, genel oyun 30-60 ms, video görüşme 60-100 ms, üzeri sorunlu' satırlarından oluşan bir tablo hem okuyucuya hem AI yanıtına daha kullanışlı geliyor açıklanır
+4. Mevcut 'Ping Nasıl Düşürülür?' bölümü genel öneriler içeriyor; kablo bağlantısı, 5 GHz bant, arka plan indirmeleri ve sunucu bölgesi seçimi gibi dört somut adıma çevrilebilir</t>
+          </r>
         </is>
       </c>
       <c r="Y8" s="4" t="inlineStr">
         <is>
-          <t>Rakip bir araç sayfasıyla sıralanmaktadır; yazının bir hız testi aracına bağlanması değerlendirilebilir.</t>
+          <t>Ping değerleri bağlantı türüne göre değişiyor; verilen aralıkların hangi bağlantı için geçerli olduğu belirtilmelidir.</t>
         </is>
       </c>
       <c r="Z8" s="7" t="n">
@@ -9011,7 +9110,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="155.5" customHeight="1">
+    <row r="9" ht="223" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/type-c-teknolojisi-ne-ise-yarar-neden-bu-kadar-yaygin</t>
@@ -9120,9 +9219,10 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t xml:space="preserve">1. Kablo ve şarj aleti seçimi bölümü eklenebilir
-2. USB-C standartları ve hız sınıfları tablo hâlinde verilebilir
-3. Hangi cihazlarda bulunduğu listelenebilir
+            <t xml:space="preserve">1. Type-C Nedir, Ne Demek?
+2. USB 3.2, USB4 ve Thunderbolt Arasındaki Fark
+3. Type-C ile Hızlı Şarj Nasıl Çalışır?
+4. Kablo Kalitesi Aktarım Hızını Nasıl Etkiler?
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Type C Nedir? · Type C Girişe Sahip Olan Cihazlar Hangileridir? · USB Type-C’nin diğer USB türlerinden Farkı · USB Type-C’nin Avantajları ve USB Type-C’nin Dezavantajları · Type-C Girişli Telefonlara </t>
           </r>
           <r>
@@ -9175,14 +9275,15 @@
       </c>
       <c r="X9" s="4" t="inlineStr">
         <is>
-          <t>1. Kablo ve şarj aleti seçimi bölümü eklenebilir
-2. USB-C standartları ve hız sınıfları tablo hâlinde verilebilir
-3. Hangi cihazlarda bulunduğu listelenebilir</t>
+          <t>1. Sayfa 'type c' sorgusunda 91.693 Impression alıyor ancak 7.8 sırada ve 23 click getiriyor; bu aramada sonuç sayfasının üst sıraları ürün listeleyen mağazalarda olduğu için bilgi tarafında kazanım 'type c nedir' ve 'type c ne demek' kalıplarında. İkisi de gövdede birer kez geçiyor, ara başlığa taşınabilir
+2. USB-C sürümleri yazıda ayrışmıyor; USB 3.2, USB4 ve Thunderbolt 4 için veri hızı, güç aktarımı ve görüntü desteği sütunlarından oluşan bir tablo, konunun en çok karıştırılan yanını karşılar açıklanır
+3. 'Type-C ile hızlı şarj nasıl çalışır' sorusu yazıda yanıtlanmıyor; Power Delivery kademelerinin watt değerleriyle verildiği bir bölüm eklenebilir
+4. Yazıda kablo kalitesinin aktarım hızını nasıl sınırladığı geçmiyor; aynı görünen iki kablonun farklı hız vermesi somut bir okuyucu sorusu ve tek paragrafla karşılanabilir</t>
         </is>
       </c>
       <c r="Y9" s="4" t="inlineStr">
         <is>
-          <t>Sorgunun büyük bölümü ürün satın alma niyetlidir; açıklama yazısının ilk sıraya çıkması sınırlıdır, Pasaj sayfasına yönlendirme değerlendirilebilir.</t>
+          <t>Ürün önerisi verilmemesi, teknik ayrım katmanında kalınması önerilir; şarj aleti ve kablo aramaları mağaza sayfalarına aittir.</t>
         </is>
       </c>
       <c r="Z9" s="7" t="n">
@@ -9202,7 +9303,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="155.5" customHeight="1">
+    <row r="10" ht="246" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/vdsl-ve-adsl-nedir-internet-baglanti-turleri-arasindaki-farklar</t>
@@ -9306,10 +9407,9 @@
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>1. Hangi bağlantının hangi kullanım için uygun olduğu tablo hâlinde verilebilir
-2. Hız beklentisi mesafeye göre açıklanabilir
-3. Altyapı sorgulamaya bağlantı eklenebilir
-4. Fiber karşılaştırması genişletilebilir</t>
+          <t>1. ADSL, VDSL ve Fiber Karşılaştırma Tablosu
+2. VDSL Modem Nedir, ADSL Modemden Farkı Ne?
+3. Hangi Bağlantı Kimin İçin Uygun?</t>
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr">
@@ -9394,15 +9494,39 @@
       </c>
       <c r="X10" s="4" t="inlineStr">
         <is>
-          <t>1. Hangi bağlantının hangi kullanım için uygun olduğu tablo hâlinde verilebilir
-2. Hız beklentisi mesafeye göre açıklanabilir
-3. Altyapı sorgulamaya bağlantı eklenebilir
-4. Fiber karşılaştırması genişletilebilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. 'adsl vdsl farkı' sorgusu 3.3 ortalama sırada 3.014 Impression alıyor; bu sayfanın en güçlü olduğu alan ve mevcut karşılaştırma metin hâlinde. Hız, mesafe hassasiyeti, upload oranı ve tipik kullanım satırlarından oluşan bir tabloya çevrilmesi ilk üçe girme ihtimalini artırır açıklanır
+2. 'vdsl modem nedir' sorgusu 1.878 Impression ile 4.5 sırada; modem tarafı yazıda tek cümlede geçiyor. 'VDSL Modem Nedir, ADSL Modemden Farkı Ne?' başlığı altında uyumluluk ve değişim gerekliliği anlatılabilir
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Vodafone</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un aynı sorguda 1. sıradaki yazısı 485 kelime; bizim yazımız 1.092 kelimeyle iki katı ve daha kapsamlı. Eksik olan uzunluk değil, tablo ve karar yardımı: 'Hangi Bağlantı Kimin İçin Uygun?' bölümü, ev tipi ve kullanıcı sayısına göre üç senaryo verebilir
+4. Fiber bağlantı yazıda karşılaştırmaya girmiyor; ADSL, VDSL ve fiber üçlüsünün aynı tabloda görülmesi, okuyucunun asıl sorusunu karşılar açıklanır</t>
+          </r>
         </is>
       </c>
       <c r="Y10" s="4" t="inlineStr">
         <is>
-          <t>Rakip sayfalar aynı formatta olduğundan fark içerik derinliğindedir; sayfa türü değişikliği gerekmemektedir.</t>
+          <t>Altyapı ve hız değerleri bölgeye göre değişiyor; sorgulama işleminin ilgili hizmet sayfasından yapılabileceği belirtilebilir.</t>
         </is>
       </c>
       <c r="Z10" s="7" t="n">
@@ -9422,7 +9546,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="128.5" customHeight="1">
+    <row r="11" ht="263.5" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/internette-dalgalanma-neden-olur-jitter-degeri-nedir</t>
@@ -9531,9 +9655,10 @@
       </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>1. İdeal jitter değeri tablo hâlinde verilebilir
-2. Ölçüm yöntemi eklenebilir
-3. Paket kaybı ile ilişkisi açıklanabilir
+          <t>1. İdeal Jitter Değerleri Tablosu
+2. Net Jitter Ne Demek?
+3. Jitter, Ping ve Paket Kaybı Arasındaki Fark
+4. Jitter Nasıl Düşürülür?
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Jitter Nedir? · Jitter Nasıl Anlaşılır?</t>
         </is>
       </c>
@@ -9568,14 +9693,40 @@
       </c>
       <c r="X11" s="4" t="inlineStr">
         <is>
-          <t>1. İdeal jitter değeri tablo hâlinde verilebilir
-2. Ölçüm yöntemi eklenebilir
-3. Paket kaybı ile ilişkisi açıklanabilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. 'jitter kaç olmalı' sorgusu 866 Impression ile 7.8 sırada geliyor ve yazıda ideal aralık tablo hâlinde verilmiyor; 'Video görüşme için 30 ms altı, oyun için 20 ms altı, akış için 50 ms altı' satırlarından oluşan bir tablo bu aramayı karşılar açıklanır
+2. 'net jitter ne demek' ve 'net jitter' sorguları birlikte 1.869 Impression alıyor; terim gövdede geçmiyor. Ağ tarafındaki kullanımın ayrı bir cümleyle açıklanması yeterli açıklanır
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Vodafone</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un 1. sıradaki yazısında ana terim 55 kez geçiyor, bizim yazımızda 23; sayının artırılması değil, jitter kelimesinin ara başlıklarda ve tablo satırlarında da kullanılması öneriliyor açıklanır
+4. Jitter ile ping ve paket kaybı arasındaki fark yazıda net ayrılmıyor; üç kavramı yan yana koyan kısa bir bölüm, konunun en sık karıştırılan yanını kapatıyor açıklanır
+5. Jitter düşürme adımları yazıda genel kalıyor; kablolu bağlantı, QoS ayarı, arka plan trafiği ve modem konumu dört somut maddeye çevrilebilir</t>
+          </r>
         </is>
       </c>
       <c r="Y11" s="4" t="inlineStr">
         <is>
-          <t>Rakip sayfa aynı formattadır; fark ölçüm ve değer tablosundadır.</t>
+          <t>Değerler bağlantı türüne ve uygulamaya göre değişiyor; aralıkların hangi senaryo için geçerli olduğu yazılmalıdır.</t>
         </is>
       </c>
       <c r="Z11" s="7" t="n">
@@ -9595,7 +9746,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="142" customHeight="1">
+    <row r="12" ht="236.5" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/wi-fi-6-nedir-wi-fi-5-ile-arasindaki-temel-farklar</t>
@@ -9698,9 +9849,9 @@
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>1. Wi-Fi 6 destekleyen modem listesi eklenebilir
-2. Mesh sistemlerle ilişkisi açıklanabilir
-3. Yükseltmenin ne zaman anlamlı olduğu bölümü eklenebilir
+          <t>1. Wi-Fi 6 Modem Nedir, Hangi Modemler Destekler?
+2. OFDMA, MU-MIMO ve Target Wake Time Nedir?
+3. Wi-Fi 6E ve Wi-Fi 7 ile Arasındaki Fark
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Wi-Fi 6 Nedir? · Wi-Fi 6 Özellikleri · Wifi 6 Avantajları Nelerdir? · Wi-Fi 6 ve Wi-Fi 5 Arasındaki Farklar · Wi-Fi 6 Uyumlu Cihazlar Nelerdir?</t>
         </is>
       </c>
@@ -9743,14 +9894,39 @@
       </c>
       <c r="X12" s="4" t="inlineStr">
         <is>
-          <t>1. Wi-Fi 6 destekleyen modem listesi eklenebilir
-2. Mesh sistemlerle ilişkisi açıklanabilir
-3. Yükseltmenin ne zaman anlamlı olduğu bölümü eklenebilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. 'wifi 6 modem' ve 'wifi 6 modem nedir' sorguları birlikte 4.132 Impression alıyor, sayfa 7.8 ve 4.1 sıralarda; modem tarafı yazıda tek cümlede geçiyor. 'Wi-Fi 6 Modem Nedir, Hangi Modemler Destekler?' başlığı altında uyumluluk, cihaz tarafı gereksinimi ve mevcut modemin yeterli olup olmadığı anlatılabilir
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Vodafone</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un aynı sorguda 1. sıradaki yazısı 1.639 kelime ve 14 ara başlık taşıyor; bizim yazımız 1.146 kelime ve 11 başlık. Fark, kapsam derinliğinde: OFDMA, MU-MIMO ve Target Wake Time gibi teknik kavramların her biri iki cümlelik alt bölüme çevrilebilir
+3. Wi-Fi 6E ve Wi-Fi 7 yazıda geçmiyor; okuyucu Wi-Fi 6 ile Wi-Fi 6E ayrımını sık soruyor, kısa bir bölüm bu boşluğu kapatır açıklanır
+4. 'wifi 6 nedir' sorgusunda sayfa 3.4 sırada ve 48 click alıyor; giriş paragrafındaki tanımın tek cümleye indirilmesi, ilk üçe yaklaşmak için en düşük maliyetli adım açıklanır</t>
+          </r>
         </is>
       </c>
       <c r="Y12" s="4" t="inlineStr">
         <is>
-          <t>Sorgu ticari niyet taşımaktadır; 1. sıradaki açıklama yazısının düşük trafik alması bunun göstergesidir. Cihaz sayfasına bağlantı kurulması değerlendirilebilir.</t>
+          <t>Cihaz uyumluluğu marka ve model ailesine göre değişiyor; genel ifadeler yerine standart adları kullanılmalıdır.</t>
         </is>
       </c>
       <c r="Z12" s="7" t="n">
@@ -9770,7 +9946,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="155.5" customHeight="1">
+    <row r="13" ht="231" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/mac-adresi-her-cihazin-kendine-ozgu-dijital-imzasi</t>
@@ -9877,9 +10053,11 @@
       </c>
       <c r="U13" s="4" t="inlineStr">
         <is>
-          <t>1. MAC adresinin cihazdan öğrenilmesi işletim sistemi bazında eklenebilir
-2. MAC filtreleme bölümü eklenebilir
-3. IP adresiyle farkı açıklanabilir
+          <t>1. Windows ve macOS'ta MAC Adresi Nasıl Bulunur?
+2. Android ve iPhone'da MAC Adresi Nasıl Öğrenilir?
+3. Modem Arayüzünden Bağlı Cihazların MAC Adresi
+4. MAC Adresinden Cihaz Üreticisi Nasıl Bulunur?
+5. Telefonlarda MAC Adresi Neden Değişiyor?
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: MAC Adresi Değiştirme Nasıl Yapılır?</t>
         </is>
       </c>
@@ -9914,14 +10092,39 @@
       </c>
       <c r="X13" s="4" t="inlineStr">
         <is>
-          <t>1. MAC adresinin cihazdan öğrenilmesi işletim sistemi bazında eklenebilir
-2. MAC filtreleme bölümü eklenebilir
-3. IP adresiyle farkı açıklanabilir</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">1. 'mac adresi sorgulama' ve 'mac adresi nasıl bulunur' sorguları birlikte 1.800 Impression alıyor, sayfa 6.7 ve 9.2 sıralarda; adım anlatımı yazıda cihaz bazında ayrışmıyor. Windows, macOS, Android, iPhone ve modem arayüzü için beş kısa adım listesi eklenebilir
+2. 'mac adresinden cihaz bulma' sorgusu 237 Impression alıyor ve yazıda karşılığı yok; MAC adresinin ilk üç baytının üretici kodunu taşıdığı ve bu bilgiyle cihaz markasının bulunabildiği tek paragrafla açıklanabilir
+3. 'telefon mac adresi nedir' sorgusu 4.3 sırada 283 Impression alıyor; telefonlarda rastgele MAC kullanımının (privacy MAC) neden devreye girdiği, okuyucunun gördüğü değerin neden değiştiğini açıklar açıklanır
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Vodafone</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>'un 3. sıradaki yazısında ana terim 46 kez geçiyor, bizim yazımızda 43; kelime sıklığı yeterli, eksik olan cihaz bazında adım anlatımı açıklanır</t>
+          </r>
         </is>
       </c>
       <c r="Y13" s="4" t="inlineStr">
         <is>
-          <t>Sorgu adım arama niyetlidir; tanım bölümü kısaltılıp adımlar öne alınabilir.</t>
+          <t>Rastgele MAC kullanımı işletim sistemi sürümüne göre değişiyor; adımların sürüm bilgisiyle verilmesi önerilir.</t>
         </is>
       </c>
       <c r="Z13" s="7" t="n">

</xml_diff>

<commit_message>
Alt başlıklar ve FAQ gerçek soru kelimesi verisiyle doğrulandı
- Ahrefs Keywords Explorer soru kelimesi taraması: 47 primary için 189 soru
  kelimesi, 356.790 aylık arama · data/soru_kelimeleri.json
- Türk Telekom blogunun 22 rakip yazısının H2/H3 yapısı çekilip karşılaştırıldı
- Soru kelimesi hacminin karşılanan payı %78'den %92'ye çıktı
- 41 yeni başlık ve 61 yeni FAQ girdisi eklendi (398 başlık, 297 FAQ)
- K20 ve K16 için niyet notu eklendi: jenerik hacmin büyük bölümü marka
  aramasından geliyor (martı tag 6.600 · yapı kredi müşteri numarası 2.400)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -10401,7 +10401,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="304" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Gizli Numara: Arama, Kapatma ve Numara Gizleme Ayarları</t>
@@ -10474,6 +10474,7 @@
 H3: iPhone'da Gizli Numara Kapatma
 H3: Operatör Servisiyle Kalıcı Engelleme
 H2: Gizli Numarayı Öğrenmek Mümkün mü?
+H2: Gizli Numaradan Gelen Aramalar Tehlikeli mi?
 H2: Numara Gizleme ile İlgili Yasal Sınırlar
 H2: Gizli Numara Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -10503,6 +10504,10 @@
 Kullanıcı tarafından öğrenilemez. Rahatsız edici aramalarda numara ancak yasal başvuru sonrasında yetkili makamlarca tespit edilebilir.
 H3: iPhone'da Numara Gizleme Nereden Yapılır?
 Ayarlar bölümündeki telefon menüsünde yer alan arayan kimliğimi göster seçeneği kapatılarak yapılır.
+H3: Gizli Numaradan Gelen Aramalar Tehlikeli mi?
+Her gizli arama zararlı değildir; ancak kişisel bilgi, doğrulama kodu ya da ödeme talep eden aramalar dolandırıcılık girişimi olarak değerlendirilmelidir.
+H3: Gizli Numara Engelleme Kalıcı mı?
+Telefon ayarından yapılan engelleme cihaz sıfırlandığında kalkar; operatör tarafında tanımlanan engelleme ise talep edilene kadar sürer.
 H3: Gizli Numara Engellendiğinde Arayan Ne Duyar?
 Arama karşı tarafa iletilmez; arayan genellikle meşgul ya da ulaşılamıyor uyarısı alır.</t>
         </is>
@@ -10591,7 +10596,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="358" customHeight="1">
+    <row r="6" ht="409" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Yurt Dışından Getirilen Telefonun IMEI Kaydı: Ücret, Süre ve Adımlar</t>
@@ -10670,6 +10675,7 @@
 H2: IMEI Sorgulama Nasıl Yapılır?
 H3: e-Devlet Üzerinden IMEI Sorgulama
 H3: BTK IMEI Sorgulama Ekranı
+H2: IMEI Sorgulama Neden Önemlidir?
 H2: IMEI Kaydı Nasıl Yapılır? Adım Adım
 H2: Kayıtsız Telefon Kaç Gün Kullanılabilir?
 H2: IMEI Kaydı Sonrası Telefon Ne Zaman Açılır?
@@ -10702,6 +10708,10 @@
 Yurt dışından getirilen telefon, yasal kullanım süresi boyunca şebekede çalışır; süre dolduğunda kayıt yapılmadıysa cihaz şebekeye kapatılır.
 H3: IMEI Kaydı Yapıldıktan Sonra Telefon Ne Zaman Açılır?
 Kayıt işlemi tamamlandıktan sonra cihaz genellikle kısa süre içinde şebekeye açılır; açılmazsa cihazın yeniden başlatılması denenebilir.
+H3: IMEI Sorgulama Neden Önemlidir?
+Sorgulama, cihazın kayıtlı olup olmadığını ve şebekeye kapatılma riskini önceden gösterir; ikinci el alımda da ilk kontrol adımıdır.
+H3: Yurt Dışı Telefon Kayıt Ücreti Taksitle Ödenir mi?
+Harç ödemesi tek seferde yapılır; taksit imkânı ödeme yapılan kanalın kart koşullarına bağlıdır.
 H3: Bir Kişi Kaç Telefon Kaydettirebilir?
 Yurt dışından getirilen cihazların kaydı kişi başına ve belirli bir süre aralığında sınırlıdır; güncel sınır kayıt başvurusu sırasında görüntülenir.</t>
         </is>
@@ -10807,7 +10817,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="263.5" customHeight="1">
+    <row r="7" ht="371.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Google Güvenli Arama: Açma, Kapatma ve Aile Filtresi</t>
@@ -10864,6 +10874,8 @@
 H2: Güvenli Arama Nasıl Kapatılır?
 H3: Bilgisayarda Güvenli Arama Filtresi Kapatma
 H3: Telefonda Google Güvenli Arama Kapatma
+H2: iPhone'da Güvenli Arama Nasıl Kapatılır?
+H2: Operatör Ayarlarından Güvenli Arama Nasıl Kapatılır?
 H2: Güvenli Arama Kilidi Nasıl Açılır?
 H2: Çocuk Hesaplarında Güvenli Arama Ayarları
 H2: Operatörün Güvenli İnternet Hizmetiyle Farkı Nedir?
@@ -10893,7 +10905,11 @@
 H3: Güvenli Arama ile Güvenli İnternet Aynı Şey mi?
 Hayır. Güvenli arama Google sonuçlarını süzer, operatörün güvenli internet hizmeti ise bağlantı düzeyinde erişimi sınırlar.
 H3: Çocuk Hesabında Güvenli Arama Nasıl Açılır?
-Aile bağlantısı uygulamasından çocuğun hesabı seçilir ve içerik kısıtlamaları bölümünden güvenli arama etkinleştirilir.</t>
+Aile bağlantısı uygulamasından çocuğun hesabı seçilir ve içerik kısıtlamaları bölümünden güvenli arama etkinleştirilir.
+H3: iPhone'da Güvenli Arama Nasıl Kapatılır?
+Safari ya da Chrome üzerinden Google arama ayarları açılır ve güvenli arama seçeneği kapatılır; ekran süresi kısıtlaması varsa önce o kaldırılır.
+H3: Operatörün Güvenli İnternet Hizmeti Nasıl Kapatılır?
+Operatörün mobil uygulaması ya da çevrimiçi işlem merkezindeki güvenli internet bölümünden profil kapatılır; işlem abone doğrulaması gerektirir.</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -11159,7 +11175,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="263.5" customHeight="1">
+    <row r="9" ht="409" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Ekran Yansıtma: Telefondan Televizyona Görüntü Aktarma</t>
@@ -11211,15 +11227,43 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>H2: Ekran Yansıtma Nedir?
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">H2: Ekran Yansıtma Nedir?
 H2: Ekran Yansıtma Nasıl Yapılır?
 H3: iPhone Ekran Yansıtma Adımları
 H3: Android Telefonu Televizyona Yansıtma
 H2: Kablo ile Telefonu TV'ye Yansıtma
+H2: Televizyonda Ekran Yansıtma Özelliği Nasıl Açılır?
+H3: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Samsung</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve"> ve LG Televizyonlarda Yansıtma
+H3: Vestel, Arçelik ve Beko Televizyonlarda Yansıtma
+H2: Bilgisayardan Televizyona Ekran Yansıtma
 H2: iPhone Ekran Yansıtma TV Bulmuyorsa Ne Yapmalı?
 H2: Yansıtma Sırasında Görüntü Donuyorsa Neye Bakılmalı?
 H2: Yansıtma Yöntemleri Karşılaştırma Tablosu
 H2: Ekran Yansıtma Hakkında Sıkça Sorulan Sorular</t>
+          </r>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -11246,7 +11290,13 @@
 H3: Kablo ile Telefon TV'ye Nasıl Bağlanır?
 Telefonun bağlantı tipine uygun HDMI adaptörü kullanılır ve televizyonun HDMI girişi kaynak olarak seçilir.
 H3: Yansıtmada Görüntü Neden Takılıyor?
-Takılma çoğunlukla ağ yoğunluğundan kaynaklanır; modeme yakın olmak ve 5 GHz bandı kullanmak akıcılığı artırır.</t>
+Takılma çoğunlukla ağ yoğunluğundan kaynaklanır; modeme yakın olmak ve 5 GHz bandı kullanmak akıcılığı artırır.
+H3: Televizyonda Ekran Yansıtma Özelliği Nasıl Açılır?
+Televizyonun kaynak ya da ayarlar menüsünden ekran yansıtma özelliği etkinleştirilir; menü adı markaya göre Screen Mirroring, Smart View veya Miracast olarak geçer.
+H3: Eski Televizyonlarda Ekran Yansıtma Mümkün mü?
+Akıllı olmayan televizyonlarda kablosuz yansıtma çalışmaz; HDMI adaptörü ya da harici bir yayın cihazı kullanılarak görüntü aktarılabilir.
+H3: Bilgisayardan Televizyona Ekran Yansıtma Nasıl Yapılır?
+Windows'ta bağlan menüsünden televizyon seçilir; kablosuz bağlantı desteklenmiyorsa HDMI kablosu kullanılır.</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -11473,7 +11523,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="263.5" customHeight="1">
+    <row r="11" ht="371.5" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>İndirilenler Klasörü: Telefonda ve Bilgisayarda Dosya Bulma</t>
@@ -11532,6 +11582,7 @@
 H3: Safari İndirilenler Klasörü Nasıl Açılır?
 H2: Bilgisayarda İndirilenler Klasörü Nerede?
 H2: Tarayıcıya Göre İndirilenler Nereye Kaydedilir?
+H2: Uygulama İçi İndirilenler Nerede? Telegram, YouTube ve WhatsApp
 H2: İndirilen Dosya Bulunamıyorsa Ne Yapmalı?
 H2: Son İndirilenler Nasıl Görüntülenir?
 H2: İndirilenler Klasörü Nasıl Temizlenir?
@@ -11562,6 +11613,10 @@
 Tarayıcının indirme geçmişinden dosyanın konumu açılabilir; dosya adı dosya yöneticisinde aratılarak da bulunabilir.
 H3: Bilgisayarda İndirilenler Klasörü Nerede?
 Windows ve macOS'ta kullanıcı klasörünün altındaki indirilenler dizininde bulunur ve dosya yöneticisinin hızlı erişim bölümünden açılabilir.
+H3: Telegram'da İndirilenler Nerede?
+Telegram indirdiği dosyaları kendi klasörüne kaydeder; uygulamanın ayarlarından cihazın galerisine kaydetme seçeneği açılabilir.
+H3: YouTube'da İndirilenler Nerede?
+YouTube üzerinden indirilen videolar uygulama içinde saklanır ve yalnızca uygulamadan izlenebilir; cihazın dosya yöneticisinde görünmez.
 H3: İndirilenler Klasörü Temizlenirse Ne Olur?
 Klasördeki dosyalar silinir ve cihazda yer açılır; silinen dosyalar geri dönüşüm kutusu bulunmayan cihazlarda geri getirilemez.</t>
         </is>
@@ -11810,7 +11865,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="209.5" customHeight="1">
+    <row r="13" ht="409" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Spam Ne Demek? Spam Mesaj ve Aramaları Engelleme</t>
@@ -11860,6 +11915,8 @@
         <is>
           <t>H2: Spam Ne Demek?
 H2: Spam Arama Ne Demek?
+H2: Spam Numara Ne Demek?
+H2: Spam Bildir ve Spam Şüphesi Ne Anlama Gelir?
 H2: Spam Mesajlar Nasıl Engellenir?
 H2: Spam Aramalar Nasıl Engellenir?
 H2: Operatör Tarafındaki Engelleme Servisleri
@@ -11886,7 +11943,15 @@
 H3: Spam Mesajlar Nasıl Engellenir?
 Gönderen numara engellenir, mesaj spam olarak bildirilir ve ticari ileti izinleri izin yönetim sistemi üzerinden iptal edilir.
 H3: Gelen Aramanın Spam Olduğu Nasıl Anlaşılır?
-Tanımadık numaradan gelen, kişisel bilgi ya da doğrulama kodu isteyen aramalar spam olarak değerlendirilir; kod hiçbir koşulda paylaşılmamalıdır.</t>
+Tanımadık numaradan gelen, kişisel bilgi ya da doğrulama kodu isteyen aramalar spam olarak değerlendirilir; kod hiçbir koşulda paylaşılmamalıdır.
+H3: Spam Numara Ne Demek?
+Çok sayıda kullanıcı tarafından istenmeyen olarak bildirilen ve bu nedenle telefon uygulamasında uyarı etiketiyle gösterilen numaradır.
+H3: Spam Şüphesi Ne Demek?
+Telefonun arayan numarayı bilinen istenmeyen arama listeleriyle eşleştirdiğini ve bu aramanın büyük olasılıkla tanıtım ya da dolandırıcılık amaçlı olduğunu gösterir.
+H3: Spam Bildir Ne İşe Yarar?
+Bildirim, o numaranın istenmeyen olarak işaretlenmesini sağlar ve benzer aramaların hem kendinizde hem diğer kullanıcılarda uyarı almasına katkıda bulunur.
+H3: Spam Atmak Ne Demek?
+Aynı içeriğin çok sayıda kişiye ya da aynı kişiye tekrar tekrar gönderilmesini ifade eder.</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -11954,7 +12019,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="317.5" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>SSD, RAM ve Ekran Kartı: Bilgisayar Donanımı Rehberi</t>
@@ -12008,9 +12073,14 @@
         <is>
           <t>H2: RAM Nedir, Ne İşe Yarar?
 H2: Kaç GB RAM Yeterlidir?
+H2: RAM Plus ve Sanal RAM Nedir?
 H2: SSD Nedir, Ne İşe Yarar?
+H2: SSD Çeşitleri: SATA, NVMe ve M.2
 H2: SSD ile HDD Arasındaki Fark Nedir?
+H2: RAM Raporu Nedir, Nereden Bakılır?
 H2: Ekran Kartı Nedir, Ne İşe Yarar?
+H3: Dahili ve Harici Ekran Kartı Arasındaki Fark
+H3: Paylaşımlı ve Onboard Ekran Kartı Ne Demek?
 H2: Anakart Nedir?
 H2: Bilgisayar Donanımı Karşılaştırma Tablosu
 H2: Bilgisayar Yavaşladığında Hangi Donanıma Bakılmalı?
@@ -12044,6 +12114,18 @@
 SSD çok daha hızlı, sessiz ve darbeye dayanıklıdır; HDD ise aynı fiyata daha yüksek kapasite sunar.
 H3: Ekran Kartı Ne İşe Yarar?
 Ekran kartı görüntünün işlenmesinden sorumludur; oyun, video düzenleme ve grafik işlerinde performansı doğrudan etkiler.
+H3: RAM Raporu Nedir?
+RAM raporu, telefonun bellek kullanımını ve hangi uygulamaların ne kadar bellek tükettiğini gösteren tanılama ekranıdır.
+H3: Dahili ve Harici Ekran Kartı Arasındaki Fark Nedir?
+Dahili ekran kartı işlemciyle bütünleşik çalışır ve sistem belleğini kullanır; harici ekran kartı ayrı bir bileşendir ve kendi belleğine sahiptir.
+H3: Paylaşımlı Ekran Kartı Ne Demek?
+Ekran kartının ayrı bir belleği olmadığını, sistem RAM'inin bir bölümünü görüntü işleme için kullandığını ifade eder.
+H3: RAM Plus Nedir?
+RAM Plus, telefonun depolama alanının bir bölümünü geçici olarak bellek gibi kullanmasını sağlayan sanal RAM özelliğidir.
+H3: Sanal RAM Gerçek RAM'in Yerini Tutar mı?
+Tutmaz. Depolama birimi bellekten yavaştır; sanal RAM yalnızca yoğun anlarda ek nefes alanı sağlar.
+H3: NVMe ile SATA SSD Arasındaki Fark Nedir?
+NVMe diskler SATA'ya göre çok daha yüksek okuma ve yazma hızı sunar; M.2 ise diskin fiziksel bağlantı biçimini tanımlar.
 H3: Bilgisayar Yavaşladığında Önce Neye Bakılmalı?
 Açılış ve dosya erişimi yavaşsa depolama birimine, aynı anda çok uygulama açıkken takılma yaşanıyorsa RAM kapasitesine bakılır.</t>
         </is>
@@ -12088,7 +12170,8 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>Ürün önerisi verilmemeli; bilgi katmanında kalınmalıdır.</t>
+          <t>Ürün önerisi verilmemeli; bilgi katmanında kalınmalıdır.
+NİYET NOTU: 'ram krizi' (500) bellek fiyatlarına ilişkin haber niyetlidir ve bu yazının kapsamı dışındadır.</t>
         </is>
       </c>
       <c r="R14" s="8" t="n">
@@ -12115,7 +12198,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="263.5" customHeight="1">
+    <row r="15" ht="371.5" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>E-İmza Nasıl Alınır?</t>
@@ -12166,6 +12249,8 @@
 H2: E-İmza Nasıl Alınır? Adım Adım
 H2: E-İmza Başvurusu İçin Gereken Belgeler
 H2: E-İmza ile Mobil İmza Arasındaki Fark Nedir?
+H2: Mobil İmza e-Devlet Üzerinden Nasıl Alınır?
+H2: E-İmza Ücreti Ne Kadar, Ücretsiz Alınabilir mi?
 H2: E-İmza Nerelerde Kullanılır?
 H2: E-İmza Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -12192,7 +12277,11 @@
 H3: E-İmza Başvurusu İçin Hangi Belgeler Gerekir?
 Bireysel başvurularda kimlik belgesi yeterlidir; kurumsal başvurularda ayrıca yetki belgesi ve şirket bilgileri istenir.
 H3: E-İmza Nerelerde Kullanılır?
-e-Devlet işlemlerinde, resmî yazışmalarda, sözleşme onaylarında ve kurumsal imza akışlarında kullanılır.</t>
+e-Devlet işlemlerinde, resmî yazışmalarda, sözleşme onaylarında ve kurumsal imza akışlarında kullanılır.
+H3: Mobil İmza e-Devlet'ten Nasıl Alınır?
+Mobil imza başvurusu operatör üzerinden yapılır; hat sahibi doğrulandıktan sonra imza e-Devlet girişlerinde kullanılabilir hâle gelir.
+H3: E-İmza Ücretsiz Alınabilir mi?
+Sertifika hizmeti ücretlidir; bazı kurumlar çalışanlarına ya da üyelerine kurumsal anlaşma kapsamında sağlayabilir.</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -12260,7 +12349,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="209.5" customHeight="1">
+    <row r="16" ht="371.5" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Taahhüt Ne Demek?</t>
@@ -12310,8 +12399,10 @@
         <is>
           <t>H2: Taahhüt Ne Demek?
 H2: Taahhütlü Ne Demek, Taahhütsüzden Farkı Nedir?
-H2: Taahhüt Süresi Nasıl Öğrenilir?
+H2: Taahhüt Etmek Ne Demek?
+H2: Taahhüt Süresi ve Taahhüt Tarihi Nasıl Öğrenilir?
 H2: Taahhüt Süresi Dolmadan Çıkılırsa Ne Olur?
+H2: Taahhüt Bittiğinde Ne Olur?
 H2: Taahhüt Hakkında Sıkça Sorulan Sorular</t>
         </is>
       </c>
@@ -12335,7 +12426,13 @@
 H3: Taahhüt Süresi Nereden Öğrenilir?
 Taahhüt süresi operatörün mobil uygulaması ya da çevrimiçi işlem merkezindeki abonelik bilgileri bölümünden görüntülenir.
 H3: Taahhüt Bitmeden Çıkılırsa Ne Olur?
-Kalan süreye bağlı olarak sözleşmede belirtilen cayma bedeli uygulanır; tutar kalan ay sayısına göre değişir.</t>
+Kalan süreye bağlı olarak sözleşmede belirtilen cayma bedeli uygulanır; tutar kalan ay sayısına göre değişir.
+H3: Taahhüt Etmek Ne Demek?
+Bir hizmeti belirli bir süre boyunca kullanacağını sözleşmeyle beyan etmek anlamına gelir.
+H3: Taahhüt Tarihi Ne Demek?
+Taahhüdün başladığı ve biteceği tarihleri ifade eder; abonelik bilgileri ekranında görüntülenir.
+H3: Taahhüt Bittiğinde Ne Olur?
+Süre dolduğunda bağlayıcılık sona erer; tarife çoğunlukla taahhütsüz koşullarla devam eder ve dilendiğinde değiştirilebilir.</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
@@ -12388,7 +12485,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="277" customHeight="1">
+    <row r="17" ht="371.5" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Konum Paylaşma ve Numaradan Konum Bulma</t>
@@ -12448,6 +12545,7 @@
 H2: Canlı Konum Nasıl Paylaşılır, Ne Kadar Sürer?
 H2: Neredeyim? Kendi Konumumu Nasıl Bulurum?
 H2: Numaradan Konum Bulma Gerçekten Mümkün mü?
+H2: Operatörler Numaradan Konum Bulma Hizmeti Veriyor mu?
 H2: Konum Paylaşımı Nasıl Durdurulur?
 H2: Konum Servisleri Pili Ne Kadar Tüketir?
 H2: Konum Paylaşma Hakkında Sıkça Sorulan Sorular</t>
@@ -12477,6 +12575,10 @@
 Yalnızca telefon numarasıyla bir kişinin konumunu bulmak kullanıcı tarafından mümkün değildir; konum ancak karşı taraf paylaştığında görülebilir.
 H3: Konum Paylaşımı Nasıl Durdurulur?
 Paylaşımın yapıldığı uygulamadaki konum ekranından durdurma seçeneği kullanılır ya da cihaz ayarlarından uygulamanın konum izni kapatılır.
+H3: Operatörler Numaradan Konum Bulma Hizmeti Veriyor mu?
+Bireysel kullanıcıya açık böyle bir hizmet bulunmamaktadır; konum bilgisi yalnızca yasal talep üzerine yetkili makamlarla paylaşılır.
+H3: Telefondan Konum Nasıl Atılır?
+Mesajlaşma uygulamasının ek menüsünden konum seçilir, harita üzerinde nokta onaylanır ve gönderilir.
 H3: Konum Servisleri Pili Çok mu Tüketir?
 Sürekli açık konum izni pil tüketimini artırır; iznin yalnızca uygulama kullanılırken verilmesi tüketimi azaltır.</t>
         </is>
@@ -13336,7 +13438,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="317.5" customHeight="1">
+    <row r="23" ht="371.5" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>eSIM Nedir, Nasıl Aktive Edilir?</t>
@@ -13422,6 +13524,8 @@
 Son yılların üst ve orta segment modellerinin büyük bölümü eSIM destekler; desteğin olup olmadığı cihaz ayarlarındaki hücresel bağlantı menüsünden kontrol edilebilir.
 H3: Mevcut Hat eSIM'e Taşınabilir mi?
 Evet. Numara değişmeden fiziksel SIM eSIM'e dönüştürülebilir; işlem sırasında hat kısa süre kapalı kalabilir.
+H3: eSIM Kart Nedir?
+eSIM kart, fiziksel bir kart yerine cihaza gömülü çip üzerinde tanımlanan dijital SIM kartı ifade eder.
 H3: eSIM Yurt Dışında Kullanılabilir mi?
 Kullanılabilir. eSIM destekleyen cihazlarda ana hat açık kalırken ikinci hat olarak yerel bir eSIM paketi de tanımlanabilir.</t>
         </is>
@@ -13492,7 +13596,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="263.5" customHeight="1">
+    <row r="24" ht="371.5" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Telefon Nasıl Sıfırlanır?</t>
@@ -13544,6 +13648,7 @@
 H2: Sıfırlama Öncesi Yedekleme Nasıl Yapılır?
 H2: Android Telefon Nasıl Sıfırlanır?
 H2: iPhone Nasıl Sıfırlanır?
+H2: Şifresi Unutulan Telefon Nasıl Sıfırlanır?
 H2: Fabrika Ayarlarına Sıfırlama Sonrası Hesap Doğrulaması
 H2: Telefon Sıfırlama Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -13562,7 +13667,13 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>H3: Telefon Nasıl Sıfırlanır?
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">H3: Telefon Nasıl Sıfırlanır?
 Ayarlar menüsündeki sistem ya da genel bölümünden fabrika ayarlarına sıfırlama seçeneği açılır ve ekrandaki onaylar tamamlanır.
 H3: Telefon Sıfırlanınca Veriler Silinir mi?
 Evet. Cihazdaki fotoğraflar, uygulamalar ve ayarlar tamamen silinir; yalnızca buluta yedeklenmiş veriler geri getirilebilir.
@@ -13570,8 +13681,30 @@
 Bulut yedeği alınmalı ve cihazdan hesap çıkışı yapılmalıdır; aksi hâlde sıfırlama sonrası etkinleştirme kilidi devreye girer.
 H3: Telefon Açılmıyorsa Nasıl Sıfırlanır?
 Cihaz kurtarma moduna alınarak sıfırlama yapılabilir; tuş kombinasyonu markaya göre değişir.
+H3: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Samsung</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve"> Telefon Nasıl Sıfırlanır?
+Ayarlar bölümündeki genel yönetim menüsünden sıfırla seçeneği açılır ve fabrika ayarlarına sıfırla adımı tamamlanır.
+H3: Şifresi Unutulan Telefon Nasıl Sıfırlanır?
+Cihaz kurtarma moduna alınarak sıfırlanabilir; sıfırlama sonrasında cihaza en son giriş yapılan hesabın şifresi istenir.
 H3: Sıfırlama Sonrası Hesap Şifresi Neden İsteniyor?
 Cihaz güvenliği için etkinleştirme kilidi devrededir; kilidin kalkması için cihaza en son giriş yapılan hesabın şifresi gerekir.</t>
+          </r>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -13770,7 +13903,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="263.5" customHeight="1">
+    <row r="26" ht="409" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Yenilenmiş Telefon Ne Demek? Garanti ve Kalite Sınıfları</t>
@@ -13824,6 +13957,7 @@
 H2: Yenilenmiş Telefon Kalite Sınıfları Nelerdir?
 H2: Yenilenmiş Telefonda Garanti Süresi Ne Kadar?
 H2: Yenilenmiş iPhone Alınır mı?
+H2: Yenilenmiş Telefon Nereden Alınır?
 H2: Satın Almadan Önce Kontrol Listesi
 H2: Yenilenmiş Telefon Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -13852,7 +13986,13 @@
 H3: Yenilenmiş iPhone Alınır mı?
 Garanti belgesi, IMEI kaydı ve pil sağlığı kontrol edildiğinde uygun bir seçenek olabilir; bu üç başlık satın alma öncesinde sorgulanmalıdır.
 H3: Yenilenmiş Telefonun Kalite Sınıfı Ne Anlama Gelir?
-Kalite sınıfı cihazın dış görünümündeki kullanım izlerini tanımlar; işlevsel performans tüm sınıflarda kontrol edilmiş olur.</t>
+Kalite sınıfı cihazın dış görünümündeki kullanım izlerini tanımlar; işlevsel performans tüm sınıflarda kontrol edilmiş olur.
+H3: A Kalite Yenilenmiş Telefon Ne Demek?
+Dış yüzeyinde belirgin kullanım izi bulunmayan, yeniye en yakın görünümdeki cihazları tanımlar.
+H3: B ve C Kalite Yenilenmiş Telefon Ne Demek?
+B sınıfında hafif, C sınıfında daha belirgin kullanım izleri bulunur; iki sınıfta da cihazın işlevleri kontrol edilmiştir.
+H3: Yenilenmiş Telefon Nereden Alınır?
+Yetkili yenileme merkezleri ve bu merkezlerle çalışan satış kanalları üzerinden alınır; faturanın ve garanti belgesinin verildiği doğrulanmalıdır.</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -13921,7 +14061,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="263.5" customHeight="1">
+    <row r="27" ht="371.5" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>AirTag Nedir ve Nasıl Çalışır?</t>
@@ -14000,6 +14140,10 @@
 Anahtar, cüzdan, çanta ve bavul gibi sık kaybolan eşyaların yerinin bulunmasında kullanılır.
 H3: Yanımda Bilinmeyen Bir AirTag Varsa Ne Olur?
 Telefon bir süre sonra bilinmeyen bir takip cihazının sizinle hareket ettiği uyarısını verir; cihaz bulunup devre dışı bırakılabilir.
+H3: AirTag Ne İşe Yarar, Nasıl Faydası Olur?
+Eşyanın son görüldüğü konumu haritada gösterir, yakındayken ses çıkararak bulunmasını sağlar ve kaybolduğunda kayıp moduna alınabilir.
+H3: AirTag 2. Nesil Nedir?
+İlk sürümün yerini alan, konum hassasiyeti ve menzili geliştirilmiş modeli tanımlar; kurulum ve kullanım mantığı aynıdır.
 H3: AirTag Android Telefonlarda Çalışır mı?
 AirTag kurulumu ve takibi Apple cihazlarla yapılır; Android kullanıcıları ise bilinmeyen takip cihazlarını tarama uygulamasıyla tespit edebilir.</t>
         </is>
@@ -14069,7 +14213,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="209.5" customHeight="1">
+    <row r="28" ht="263.5" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>OEM Ne Demek?</t>
@@ -14142,7 +14286,9 @@
 H3: OEM ile Orijinal Ürün Arasındaki Fark Nedir?
 Orijinal ürün marka ambalajıyla ve marka garantisiyle satılır; OEM ürün sade ambalajla gelir ve garanti çoğunlukla satıcı tarafından verilir.
 H3: OEM Yazılım Ne Demek?
-Cihazla birlikte önceden kurulu gelen ve o cihaza bağlı olan yazılım lisansıdır; başka bir cihaza aktarılamaz.</t>
+Cihazla birlikte önceden kurulu gelen ve o cihaza bağlı olan yazılım lisansıdır; başka bir cihaza aktarılamaz.
+H3: OEM Paket Ne Demek?
+Ürünün perakende kutusu ve aksesuarları olmadan, sade ambalajda satılan hâlidir; içerik aynı, sunum farklıdır.</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
@@ -14210,7 +14356,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="263.5" customHeight="1">
+    <row r="29" ht="371.5" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>KVKK Nedir? Kişisel Verilerin Korunması Kanunu</t>
@@ -14261,6 +14407,8 @@
 H2: Kişisel Veri Nedir, Hangi Bilgiler Kişisel Veri Sayılır?
 H2: Özel Nitelikli Kişisel Veri Ne Demek?
 H2: KVKK Kapsamında Veri Sahibinin Hakları Nelerdir?
+H2: KVKK İzni ve Aydınlatma Metni Nedir?
+H2: KVKK Onayı Geri Alınabilir mi?
 H2: Kişisel Verilerin Korunması İçin Ne Yapılabilir?
 H2: KVKK Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -14287,6 +14435,10 @@
 Ad, soyad, telefon numarası, e-posta adresi, konum bilgisi ve IP adresi gibi kişiyi belirli ya da belirlenebilir kılan her türlü bilgi kişisel veridir.
 H3: KVKK Kapsamında Hangi Haklara Sahibim?
 Verilerinizin işlenip işlenmediğini öğrenme, düzeltilmesini veya silinmesini isteme, aktarıldığı tarafları öğrenme ve işleme faaliyetine itiraz etme haklarınız bulunur.
+H3: KVKK İzni Nedir?
+Kişisel verilerin belirli bir amaçla işlenebilmesi için kişiden alınan açık rızadır; hangi verinin ne amaçla işleneceği aydınlatma metninde belirtilir.
+H3: KVKK Onayı Geri Alınabilir mi?
+Alınabilir. Açık rıza istenildiği zaman geri çekilebilir ve bu durumda ilgili veri işleme faaliyeti durdurulur.
 H3: Kişisel Verilerimin Silinmesini Nasıl İsterim?
 Verinin işlendiği kuruma başvurularak silme talebi iletilir; kurum yasal süre içinde talebi sonuçlandırmakla yükümlüdür.</t>
         </is>
@@ -14356,7 +14508,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="263.5" customHeight="1">
+    <row r="30" ht="371.5" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Telefon Neden Isınır?</t>
@@ -14436,6 +14588,10 @@
 Kılıf çıkarılabilir, arka plan uygulamaları kapatılabilir, ekran parlaklığı düşürülebilir ve cihaz şarjdayken kullanılmayabilir.
 H3: Telefon Isınması Pile Zarar Verir mi?
 Sürekli yüksek sıcaklık pil ömrünü kısaltır; bu nedenle cihazın uzun süre sıcak kalmasından kaçınılmalıdır.
+H3: Telefon Neden Çok Isınır?
+Aynı anda çalışan yoğun uygulamalar, uzun süreli video ve oyun kullanımı, zayıf şebeke sinyali ve yüksek ortam sıcaklığı bir araya geldiğinde ısınma belirginleşir.
+H3: Telefon Şarj Olurken Neden Isınır?
+Şarj sırasında pile aktarılan enerjinin bir bölümü ısıya dönüşür; hızlı şarjda bu ısı daha yüksek olur ve belirli bir düzeye kadar normaldir.
 H3: Telefon Kullanılmazken Isınıyorsa Ne Yapmalı?
 Arka planda çalışan uygulamalar kontrol edilmeli; sorun sürüyorsa ve pilde şişme varsa cihaz kullanılmadan yetkili servise başvurulmalıdır.</t>
         </is>
@@ -14523,7 +14679,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="209.5" customHeight="1">
+    <row r="31" ht="317.5" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Müşteri Numarası Nedir, Nereden Öğrenilir?</t>
@@ -14574,6 +14730,8 @@
 H2: Müşteri Numarası Nereden Öğrenilir?
 H3: Faturada Müşteri Numarası Nerede Yazar?
 H3: Mobil Uygulamadan Müşteri Numarası Öğrenme
+H2: Bankacılıkta Müşteri Numarası Nedir?
+H2: Telekom Hizmetlerinde Müşteri Numarası Nedir?
 H2: Müşteri Numarası ile Abone Numarası Arasındaki Fark Nedir?
 H2: Müşteri Numarası Hangi İşlemlerde Kullanılır?
 H2: Müşteri Numarası Hakkında Sıkça Sorulan Sorular</t>
@@ -14582,7 +14740,10 @@
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>TON: Tanım ve konum gösterme. Okuyucu bir işlem sırasında numarayı arıyor; ilk paragraf tanımı verir, ikinci bölüm doğrudan nereden bulunacağını söyler.
-H2 · Müşteri Numarası Nedir: Aboneye özel, hattan bağımsız kimlik numarası olduğu iki cümlede.
+NİYET NOTU: Soru kelimesi taramasında bu terimin aramalarının büyük bölümü bankacılık kaynaklıdır (yapı kredi 2.400, kurumsal 700, bireysel 700, banka 600, firma 500, halkbank 450). Telekom niyeti azınlıktadır. Aynı ayrımı rakip blog da yapmakta ve konuyu bankacılık ile telekom başlıkları altında ikiye bölmektedir. Yazı bu nedenle terimi önce genel olarak tanımlar, sonra iki alanı ayrı bölümlerde ele alır; jenerik hacmin tamamının bu yazıyla karşılanamayacağı hesaba katılmalıdır.
+H2 · Müşteri Numarası Nedir: Kuruma kayıtlı kişiyi tanımlayan, ürün ve hat sayısından bağımsız kimlik numarası olduğu iki cümlede.
+H2 · Bankacılıkta Müşteri Numarası: Bankaların internet ve mobil şubeye girişte istediği numara; kartın arkasında, sözleşmede ve mobil uygulamada nerede göründüğü. Bireysel, kurumsal ve firma müşteri numarası ayrımı tek paragrafta.
+H2 · Telekom Hizmetlerinde Müşteri Numarası: Operatör tarafındaki karşılığı ve hangi işlemlerde istendiği.
 H2 · Nereden Öğrenilir: İki H3. Faturada hangi bölümde yer aldığı ve uygulamada hangi ekranda göründüğü. Ekran yolları ürün ekibiyle doğrulanır.
 H2 · Abone Numarası Farkı: İki satırlık tablo: neyi tanımlar, kaç tane olur. Bir müşterinin birden çok hattı olabileceği ama tek müşteri numarası bulunduğu net yazılır.
 H2 · Hangi İşlemlerde Kullanılır: Fatura ödeme, başvuru takibi, çağrı merkezi doğrulaması üç madde.
@@ -14598,7 +14759,11 @@
 H3: Müşteri Numarası ile Abone Numarası Aynı mı?
 Değildir. Abone numarası hatta özeldir; müşteri numarası ise kişiye özeldir ve birden çok hat aynı müşteri numarasına bağlı olabilir.
 H3: Müşteri Numarası Nerelerde Kullanılır?
-Fatura ödemelerinde, başvuru takibinde ve çağrı merkezi görüşmelerinde kimlik doğrulaması amacıyla kullanılır.</t>
+Fatura ödemelerinde, başvuru takibinde ve çağrı merkezi görüşmelerinde kimlik doğrulaması amacıyla kullanılır.
+H3: Bankacılıkta Müşteri Numarası Nedir?
+Bankanın her müşterisine verdiği ve internet ile mobil şube girişlerinde kullanılan numaradır; kart arkasında, sözleşmede ve mobil uygulamada görüntülenir.
+H3: Bireysel ve Kurumsal Müşteri Numarası Farkı Nedir?
+Bireysel numara kişiye, kurumsal numara ise firmaya tanımlanır; kurumsal işlemlerde ayrıca yetkili kullanıcı bilgisi istenir.</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -14623,7 +14788,8 @@
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>Tanım sorgusudur; hesap ekranına yönlendirme ürün ekibiyle doğrulanmalıdır.</t>
+          <t>Tanım sorgusudur; hesap ekranına yönlendirme ürün ekibiyle doğrulanmalıdır.
+NİYET NOTU: Jenerik 'müşteri numarası' hacminin büyük bölümü bankacılık aramalarından gelmektedir (yapı kredi 2.400, banka 600, firma 500, halkbank 450, ziraat ve akbank 250'şer). Banka markası içeren aramalar bu yazıyla karşılanamaz. Yazı bankacılık ve telekom kullanımını ayrı bölümlerde ele almakta, aynı ayrımı rakip blog da yapmaktadır.</t>
         </is>
       </c>
       <c r="R31" s="8" t="n">
@@ -14650,7 +14816,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="250" customHeight="1">
+    <row r="32" ht="304" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>OTP Ne Demek?</t>
@@ -14702,6 +14868,7 @@
 H2: OTP Kodu Nerelerde Kullanılır?
 H2: OTP Kodu Neden Kimseyle Paylaşılmamalı?
 H2: OTP Kodu Gelmiyorsa Ne Yapılmalı?
+H2: OTP Hatalı Uyarısı Ne Anlama Gelir?
 H2: OTP Hakkında Sıkça Sorulan Sorular</t>
         </is>
       </c>
@@ -14728,7 +14895,9 @@
 H3: Bankalar Telefonda OTP Kodu İster mi?
 İstemez. Kod talep eden aramalar dolandırıcılık girişimidir ve derhal sonlandırılmalıdır.
 H3: OTP Kodu Gelmiyorsa Ne Yapmalıyım?
-Şebeke bağlantısı, kayıtlı telefon numarasının güncelliği ve mesaj engelleme filtreleri kontrol edilir, ardından kod yeniden istenir.</t>
+Şebeke bağlantısı, kayıtlı telefon numarasının güncelliği ve mesaj engelleme filtreleri kontrol edilir, ardından kod yeniden istenir.
+H3: OTP Hatalı Ne Demek?
+Girilen kodun süresi dolmuş ya da yanlış girilmiş demektir; yeni kod istenip süresi içinde girilmelidir.</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -14781,7 +14950,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="263.5" customHeight="1">
+    <row r="33" ht="317.5" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>QLED Nedir? QLED ve OLED Farkı</t>
@@ -14831,6 +15000,7 @@
           <t>H2: QLED Nedir?
 H2: OLED Nedir?
 H2: QLED ve OLED Farkı Nedir?
+H2: Neo QLED Nedir, QLED'den Farkı Nedir?
 H2: Parlaklık ve Kontrast Karşılaştırması
 H2: Panel Ömrü ve Görüntü Kalıcılığı
 H2: Hangi Kullanım İçin Hangisi Daha Uygun?
@@ -14860,6 +15030,8 @@
 Yüksek tepe parlaklığı nedeniyle QLED paneller aydınlık ortamlarda daha okunaklı bir görüntü sunar.
 H3: OLED'de Görüntü Kalıcılığı Sorun mu?
 Uzun süre sabit kalan görüntülerde risk vardır; güncel panellerde bu riski azaltan koruma özellikleri bulunur.
+H3: Neo QLED Nedir?
+Neo QLED, arkadan aydınlatmada mini LED kullanan ve bu sayede daha hassas parlaklık kontrolü ile daha derin siyah sunabilen QLED sürümüdür.
 H3: Oyun İçin QLED mi OLED mi?
 Tepki süresi ve siyah derinliği nedeniyle OLED öne çıkar; ancak sabit arayüz öğeleri uzun süre ekranda kalıyorsa QLED daha güvenli bir tercih olabilir.</t>
         </is>
@@ -15045,7 +15217,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="209.5" customHeight="1">
+    <row r="35" ht="371.5" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>TAG Nedir?</t>
@@ -15088,9 +15260,11 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>H2: TAG Nedir?
+          <t>H2: TAG Nedir, TAG Açılımı Nedir?
+H2: Martı TAG Nedir, Nasıl Kullanılır?
+H2: AirTag ve Smart Tag Nedir?
+H2: NFC Tag Nedir?
 H2: Sosyal Medyada Etiketleme Ne Anlama Gelir?
-H2: NFC Etiketi (Tag) Nedir?
 H2: Web ve Ölçümlemede Tag Ne Demek?
 H2: Hangi Bağlamda Hangi Anlam Kullanılır?
 H2: TAG Hakkında Sıkça Sorulan Sorular</t>
@@ -15098,8 +15272,11 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>TON: Çok anlamlı terim açıklaması. Açılış paragrafı kelimenin birden çok anlamı olduğunu duyurur ve yazıda hangi üç anlamın ele alındığını sayar; okuyucu doğru bölüme hemen gidebilmeli.
-H2 · TAG Nedir: Genel anlamıyla etiket; içeriği sınıflandıran işaret.
+          <t>TON: Çok anlamlı terim açıklaması. Açılış paragrafı kelimenin birden çok anlamı olduğunu duyurur ve yazıda hangi anlamların ele alındığını sayar; okuyucu doğru bölüme hemen gidebilmeli.
+NİYET NOTU: Soru kelimesi taramasında bu terimin baskın anlamı ulaşım uygulaması (martı tag 6.600, tag taksi 450, tag sürücü 450, tag premium 250) ve takip cihazı (air tag 2.600, smart tag 200) olarak çıkmaktadır. Sosyal medya etiketi ve ölçümleme etiketi anlamları arama tarafında çok daha küçük paya sahiptir. Bu nedenle bölüm sırası arama hacmine göre kurulmuş, jenerik "tag nedir" hacminin tamamının bu yazıyla karşılanamayacağı not edilmiştir.
+H2 · TAG Nedir: Genel anlamıyla etiket; içeriği sınıflandıran işaret. Açılımı ve kelimenin hangi alanlarda karşımıza çıktığı tek paragrafta.
+H2 · Martı TAG: Ulaşım uygulamasındaki kullanım nötr biçimde, bilgilendirme düzeyinde anlatılır; yönlendirme ya da karşılaştırma yapılmaz.
+H2 · AirTag ve Smart Tag: İki takip cihazının ne olduğu ve hangi ekosistemde çalıştığı; ayrıntı için AirTag yazısına iç bağlantı verilir.
 H2 · Sosyal Medyada Etiketleme: Kişi etiketleme ve konu etiketi (hashtag) ayrımı; ikisi karıştırılıyor.
 H2 · NFC Etiketi: Küçük bir çipin okutulmasıyla işlem başlatılması; ev otomasyonu ve kartvizit iki örnekle.
 H2 · Web ve Ölçümlemede Tag: Sayfaya eklenen ölçümleme kodu anlamı ve HTML etiketi anlamı iki cümlede ayrı ayrı.
@@ -15109,14 +15286,44 @@
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>H3: TAG Nedir?
-TAG, Türkçede etiket anlamına gelir ve bağlama göre sosyal medyada kişi etiketlemeyi, NFC çipini ya da web sayfasına eklenen ölçümleme kodunu ifade eder.
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">H3: TAG Nedir?
+TAG, Türkçede etiket anlamına gelir; bağlama göre bir ulaşım uygulamasını, takip cihazını, sosyal medyada kişi etiketlemeyi, NFC çipini ya da web sayfasına eklenen ölçümleme kodunu ifade eder.
+H3: TAG Açılımı Nedir?
+İngilizce etiket anlamındaki tag kelimesinden gelir; kısaltma değil, doğrudan bir sözcüktür.
+H3: Martı TAG Nedir?
+Martı TAG, uygulama üzerinden sürücü ile yolcuyu eşleştiren bir ulaşım hizmetidir.
+H3: AirTag ile Smart Tag Arasındaki Fark Nedir?
+İkisi de eşya takip cihazıdır; AirTag Apple ekosisteminde, Smart Tag ise </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Samsung</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve"> ekosisteminde çalışır.
 H3: Sosyal Medyada Tag Ne Demek?
 Bir gönderide kişinin hesabının bağlanmasıdır; konu etiketi anlamındaki hashtag ise içeriğin konusunu sınıflandırır.
 H3: NFC Tag Ne İşe Yarar?
 Telefonun yaklaştırılmasıyla önceden tanımlanmış bir işlemi başlatan küçük bir çiptir; ev otomasyonu ve dijital kartvizit gibi kullanımları vardır.
 H3: HTML'de Tag Ne Anlama Gelir?
 Sayfanın yapısını tanımlayan işaretleme öğesidir; başlık, paragraf ve bağlantı gibi öğeler tag'lerle belirtilir.</t>
+          </r>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
@@ -15142,7 +15349,8 @@
       </c>
       <c r="Q35" s="4" t="inlineStr">
         <is>
-          <t>Kelimenin birden çok anlamı bulunmaktadır; açılışta hangi anlamların ele alındığı belirtilmelidir.</t>
+          <t>Kelimenin birden çok anlamı bulunmaktadır; açılışta hangi anlamların ele alındığı belirtilmelidir.
+NİYET NOTU: Jenerik 'tag' hacminin büyük bölümü ulaşım uygulaması (martı tag 6.600, tag taksi 450, tag sürücü 450, tag premium 250) ve takip cihazı (air tag 2.600) aramalarından gelmektedir; skin tag ve Google Tag Manager gibi alan dışı anlamlar da bu hacme dahildir. Yazı, arama hacmine göre sıralanmış anlam bölümleriyle kurgulanmıştır; kümeye atanan hacmin tamamının karşılanması beklenmemelidir.</t>
         </is>
       </c>
       <c r="R35" s="8" t="n">
@@ -15169,7 +15377,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="250" customHeight="1">
+    <row r="36" ht="358" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Karekod Nasıl Okutulur?</t>
@@ -15214,10 +15422,14 @@
         <is>
           <t>H2: Karekod Nedir?
 H2: Karekod Nasıl Okutulur?
+H2: Telefondan Karekod Nasıl Okutulur?
 H3: iPhone ile Karekod Okutma
 H3: Android ile Karekod Okutma
 H2: Kamera Karekodu Okutmuyorsa Ne Yapmalı?
 H2: Ekrandaki Karekod Nasıl Okutulur?
+H2: Ders Kitabındaki Karekod Nasıl Okutulur?
+H2: Wifi Karekodu ile Ağa Nasıl Bağlanılır?
+H2: Wi-Fi Karekodu Nasıl Okutulur ve Oluşturulur?
 H2: Sahte Karekodlar Nasıl Ayırt Edilir?
 H2: Karekod Hakkında Sıkça Sorulan Sorular</t>
         </is>
@@ -15244,7 +15456,11 @@
 H3: Karekod Güvenli mi?
 Kodun kendisi bir bağlantıdan ibarettir; açılan adres kontrol edilmeden kişisel bilgi veya ödeme bilgisi girilmemelidir.
 H3: Karekod ile QR Kod Aynı Şey mi?
-Evet. Karekod, QR kodun Türkçe karşılığıdır.</t>
+Evet. Karekod, QR kodun Türkçe karşılığıdır.
+H3: Ders Kitabındaki Karekod Nasıl Okutulur?
+Kitabın sayfasındaki kod telefon kamerasına tutulur; bazı yayınlar kendi uygulamaları üzerinden okutmayı gerektirir.
+H3: Wi-Fi Karekodu Nasıl Okutulur?
+Kamera koda tutulduğunda ağa bağlan seçeneği çıkar ve şifre girilmeden bağlantı kurulur; telefonlarda kayıtlı ağın karekodu da paylaşılabilir.</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -15443,7 +15659,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="209.5" customHeight="1">
+    <row r="38" ht="263.5" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>URL Nedir?</t>
@@ -15511,6 +15727,8 @@
         <is>
           <t>H3: URL Nedir?
 URL, internetteki bir sayfanın veya dosyanın tam adresidir ve tarayıcının hangi kaynağa ulaşacağını belirtir.
+H3: URL Adresi Nedir, Nerede Görülür?
+URL adresi tarayıcının en üstündeki adres çubuğunda görünen tam adrestir; bağlantıya uzun basılarak da kopyalanabilir.
 H3: URL Hangi Bölümlerden Oluşur?
 Protokol, alan adı, yol ve gerektiğinde sorgu parametrelerinden oluşur.
 H3: Güvenli URL Nasıl Anlaşılır?
@@ -15695,7 +15913,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="209.5" customHeight="1">
+    <row r="40" ht="263.5" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>FreeDOS Nedir? İşletim Sistemi Yüklü Olmayan Bilgisayar</t>
@@ -15766,6 +15984,8 @@
 Cihazın Windows veya macOS gibi bir işletim sistemiyle değil, temel bir sistemle geldiğini gösterir; günlük kullanım için ayrıca işletim sistemi kurulması gerekir.
 H3: FreeDOS Bilgisayara Windows Kurulabilir mi?
 Kurulabilir. Lisans satın alındıktan sonra kurulum medyası hazırlanarak sistem yüklenebilir.
+H3: FreeDOS İşletim Sistemi Nedir?
+MS-DOS ile uyumlu, komut satırı tabanlı ve ücretsiz bir işletim sistemidir; günlük masaüstü kullanım için tasarlanmamıştır.
 H3: FreeDOS Bilgisayar Neden Daha Ucuz?
 Fiyat farkı büyük ölçüde işletim sistemi lisans bedelinin cihaza dahil olmamasından kaynaklanır.</t>
         </is>
@@ -16377,7 +16597,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="291" customHeight="1">
+    <row r="4" ht="358" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/isletim-sistemi-nedir-ve-cesitleri-nelerdir</t>
@@ -16485,6 +16705,8 @@
 H3: Linux Nedir, Neden Tercih Edilir?
 H2: İşletim Sistemi Yalnız Bilgisayarlarda mı Bulunur?
 H2: Android ve iOS Arasındaki Farklar Nelerdir?
+H2: Televizyon İşletim Sistemleri: Tizen, webOS ve Vidaa
+H2: Pardus Nedir, Yerli İşletim Sistemi Ne Anlama Gelir?
 H2: İşletim Sistemleri Hakkında Sıkça Sorulan Sorular
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: İşletim Sistemi Özellikleri Nelerdir?</t>
         </is>
@@ -16510,7 +16732,11 @@
 H3: İşletim Sistemi Yalnızca Bilgisayarlarda mı Bulunur?
 Hayır. Telefonlar, akıllı televizyonlar, akıllı saatler ve araç bilgi sistemleri de kendi işletim sistemleriyle çalışır.
 H3: Android ile iOS Arasındaki Fark Nedir?
-Android çok sayıda üreticinin cihazında çalışır ve daha geniş özelleştirme sunar; iOS yalnızca Apple cihazlarında çalışır ve güncellemeleri tüm cihazlara aynı anda ulaşır.</t>
+Android çok sayıda üreticinin cihazında çalışır ve daha geniş özelleştirme sunar; iOS yalnızca Apple cihazlarında çalışır ve güncellemeleri tüm cihazlara aynı anda ulaşır.
+H3: Tizen İşletim Sistemi Nedir?
+Tizen, akıllı televizyonlarda ve giyilebilir cihazlarda kullanılan, Linux tabanlı bir işletim sistemidir.
+H3: Pardus İşletim Sistemi Nedir?
+Pardus, Türkiye'de geliştirilen ve kamu kurumlarında da kullanılan Linux tabanlı açık kaynaklı bir işletim sistemidir.</t>
         </is>
       </c>
       <c r="X4" s="4" t="inlineStr">
@@ -16818,7 +17044,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="317.5" customHeight="1">
+    <row r="6" ht="409" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/nfc-nedir-nfc-ile-neler-yapilabilir</t>
@@ -16965,6 +17191,7 @@
 H3: Xiaomi ve Redmi Cihazlarda NFC Nasıl Açılır?
 H2: NFC Özelliği Olan Telefonlar Hangileri?
 H2: Telefonda NFC Alanı Neresi?
+H2: Bu NFC Etiketi İçin Desteklenen Uygulama Yok Hatası Ne Anlama Gelir?
 H2: NFC Hakkında Sıkça Sorulan Sorular
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: NFC Nedir, NFC ile Neler Yapılabilir?</t>
           </r>
@@ -16994,7 +17221,11 @@
 H3: Telefonumda NFC Var mı, Nasıl Anlarım?
 Cihaz ayarlarında bağlantılar bölümünde NFC seçeneğinin bulunması desteklendiğini gösterir; seçenek yoksa cihaz NFC desteklemiyor demektir.
 H3: Telefonda NFC Alanı Nerede?
-NFC anteni çoğu modelde cihazın arka yüzünün üst bölümünde yer alır; okutma sırasında bu bölgenin okuyucuya temas etmesi gerekir.</t>
+NFC anteni çoğu modelde cihazın arka yüzünün üst bölümünde yer alır; okutma sırasında bu bölgenin okuyucuya temas etmesi gerekir.
+H3: NFC Desteği Ne Demek?
+Cihazın NFC donanımına sahip olduğunu ve temassız veri alışverişi ile ödeme yapabildiğini ifade eder.
+H3: Bu NFC Etiketi İçin Desteklenen Uygulama Yok Hatası Neden Alınır?
+Okutulan etiketin içeriğini açabilecek bir uygulama telefonda kurulu değildir; etiketin yönlendirdiği uygulamanın kurulması ya da etiketin yeniden yazılması gerekir.</t>
         </is>
       </c>
       <c r="X6" s="4" t="inlineStr">
@@ -17115,7 +17346,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="276" customHeight="1">
+    <row r="7" ht="371.5" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/gemini-nedir-googlein-yapay-zeka-uygulamasina-genel-bakis</t>
@@ -17210,6 +17441,7 @@
       <c r="U7" s="4" t="inlineStr">
         <is>
           <t>H2: Gemini Yapay Zeka Ne İşe Yarar?
+H2: Google Gemini Uygulaması Nasıl Kullanılır?
 H2: Gemini Türkçe Destekliyor mu?
 H2: Gemini ile ChatGPT Arasındaki Fark Nedir?
 H2: Gemini Ücretsiz mi?
@@ -17239,7 +17471,11 @@
 H3: Gemini Ücretsiz mi?
 Temel sürüm ücretsiz kullanılabilir; gelişmiş modeller ve ek özellikler ücretli abonelikle sunulur.
 H3: Gemini ile ChatGPT Arasındaki Fark Nedir?
-İki servis de yapay zeka sohbet asistanıdır; farklar güncel bilgiye erişim biçimi, entegre oldukları uygulama ekosistemi ve ücretsiz sürüm sınırlarında ortaya çıkar.</t>
+İki servis de yapay zeka sohbet asistanıdır; farklar güncel bilgiye erişim biçimi, entegre oldukları uygulama ekosistemi ve ücretsiz sürüm sınırlarında ortaya çıkar.
+H3: Google Gemini Uygulaması Nedir?
+Gemini'nin telefon ve tablet için sunulan uygulamasıdır; sesli soru sorma, görsel yükleme ve diğer Google uygulamalarıyla birlikte çalışma özelliklerini taşır.
+H3: Gemini Nedir, Ne İşe Yarar?
+Metin yazma ve özetleme, görsel yorumlama, kod yardımı ve Google uygulamalarıyla birlikte çalışma gibi işlerde kullanılan yapay zeka asistanıdır.</t>
         </is>
       </c>
       <c r="X7" s="4" t="inlineStr">
@@ -17290,7 +17526,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="263.5" customHeight="1">
+    <row r="8" ht="358" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/ping-internette-gecikmenin-gercek-nedeni</t>
@@ -17390,6 +17626,7 @@
 H3: Komut Satırından Ping Testi
 H3: Hız Testi Siteleriyle Ping Ölçümü
 H2: İdeal Ping Değerleri Tablosu
+H2: Ping Atmak Ne Demek?
 H2: Ping Nasıl Düşürülür? Dört Adım
 H2: Ping Hakkında Sıkça Sorulan Sorular
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Ping Testi Nedir? Nasıl Yapılır?</t>
@@ -17438,6 +17675,10 @@
 Komut satırından ping komutu çalıştırılarak ya da bir hız testi sitesi üzerinden ölçüm yapılarak test edilir.
 H3: Ping Nasıl Düşürülür?
 Kablolu bağlantıya geçilmesi, 5 GHz bandın kullanılması, arka plan indirmelerinin durdurulması ve yakın sunucu bölgesinin seçilmesi gecikmeyi azaltır.
+H3: Ping Atmak Ne Demek?
+Bir adrese küçük bir veri paketi gönderip yanıt süresini ölçmeyi ifade eder; bağlantının çalışıp çalışmadığını ve gecikmesini gösterir.
+H3: Ping ve Jitter Nedir, Farkı Nedir?
+Ping gecikmenin süresini, jitter ise bu sürenin ne kadar dalgalandığını ölçer.
 H3: Yüksek Ping Neden Olur?
 Ağ yoğunluğu, kablosuz bağlantı kalitesi, uzak sunucu konumu ve arka planda çalışan indirmeler yüksek pingin başlıca nedenleridir.</t>
         </is>
@@ -17542,7 +17783,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="236.5" customHeight="1">
+    <row r="9" ht="290.5" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/type-c-teknolojisi-ne-ise-yarar-neden-bu-kadar-yaygin</t>
@@ -17654,6 +17895,7 @@
             <t xml:space="preserve">H2: Type-C Nedir, Ne Demek?
 H2: USB 3.2, USB4 ve Thunderbolt Arasındaki Fark Nedir?
 H2: Type-C ile Hızlı Şarj Nasıl Çalışır?
+H2: Type-C Şarj Aleti Nedir, Nasıl Seçilir?
 H2: Kablo Kalitesi Aktarım Hızını Nasıl Etkiler?
 H2: Type-C Hakkında Sıkça Sorulan Sorular
 Rakip yazıda bulunup bu yazıda karşılığı olmayan ara başlıklar: Type C Nedir? · Type C Girişe Sahip Olan Cihazlar Hangileridir? · USB Type-C’nin diğer USB türlerinden Farkı · USB Type-C’nin Avantajları ve USB Type-C’nin Dezavantajları · Type-C Girişli Telefonlara </t>
@@ -17697,6 +17939,8 @@
 Değildir. Konnektör aynı olsa da desteklenen USB standardı ve kablo sertifikasyonu aktarım hızını belirler.
 H3: Type-C ile Hızlı Şarj Nasıl Çalışır?
 Power Delivery protokolü sayesinde şarj cihazı ile telefon anlaşır ve cihazın desteklediği en yüksek güç kademesinde şarj yapılır.
+H3: Type-C Şarj Aleti Nedir?
+Type-C çıkışlı, Power Delivery destekleyen şarj adaptörünü tanımlar; cihazın desteklediği güç kademesine kadar hızlı şarj sağlar.
 H3: Type-C Girişten Görüntü Aktarılır mı?
 Cihaz ve kablo destekliyorsa aktarılır; her Type-C girişte görüntü çıkışı bulunmaz.</t>
         </is>

</xml_diff>

<commit_message>
İçerik yönergesi ile içerik kurgusu tek sütunda birleştirildi
- 02 ve 03 sekmelerindeki "İçerik Yönergesi" / "Güncelleme Yönergesi" sütunları kaldırıldı
- Kurgu sütunu "İçerik Kurgusu ve Yönergesi" adını aldı; yönergedeki tekrar eden maddeler düştü
- Yönergede olup kurguda bulunmayan yedi ayrıntı kurgu metinlerine işlendi
- HTML raporda tek blok: "İçerik kurgusu ve yönergesi"; rakip bloğu sağ sütuna alınarak düzen dengelendi

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -12810,7 +12810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -12828,13 +12828,12 @@
     <col width="110" customWidth="1" min="13" max="13"/>
     <col width="62" customWidth="1" min="14" max="14"/>
     <col width="52" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
-    <col width="44" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="52" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="52" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -12863,9 +12862,8 @@
       <c r="S1" s="2" t="n"/>
       <c r="T1" s="2" t="n"/>
       <c r="U1" s="2" t="n"/>
-      <c r="V1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="81" customHeight="1">
+    </row>
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <r>
@@ -12947,6 +12945,24 @@
               <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">
+Kurgu sütunu: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>İçerik yönergesi ayrı bir sütun değildir: hangi bölümün yazılacağı ve o bölümün nasıl yazılacağı "İçerik Kurgusu ve Yönergesi" sütununda birlikte verilmektedir. Sütun bölüm bölüm ilerler: ton, giriş, her H2 ve H3 için biçim (tablo, adım listesi, madde listesi), derinlik, rakip yazının aynı bölümü nasıl işlediği ve hangi PAA sorusunun nerede karşılandığı.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00FF7B52"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">
 Uzun hücreler: </t>
           </r>
           <r>
@@ -12979,7 +12995,6 @@
       <c r="S2" s="4" t="n"/>
       <c r="T2" s="4" t="n"/>
       <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -13003,7 +13018,6 @@
       <c r="S3" s="2" t="n"/>
       <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="n"/>
-      <c r="V3" s="2" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -13063,7 +13077,7 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>İçerik Kurgusu</t>
+          <t>İçerik Kurgusu ve Yönergesi</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
@@ -13083,35 +13097,30 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>İçerik Yönergesi</t>
+          <t>Dikkat Edilecek</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>Dikkat Edilecek</t>
+          <t>Puan</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Puan</t>
+          <t>Öncelik</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>Öncelik</t>
+          <t>Peak Ayı</t>
         </is>
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>Peak Ayı</t>
+          <t>Önerilen Yayın Ayı</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>Önerilen Yayın Ayı</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>Ne Anlama Geliyor</t>
         </is>
@@ -13260,37 +13269,28 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>1. 192.168.1.1 ve 192.168.0.1 farkı açıklanır
-2. Marka bazında varsayılan kullanıcı adı ve şifre tablosu verilir
-3. Arayüze girilemediğinde kontrol listesi verilir
-4. WiFi adı ve şifresi değiştirme adım adım anlatılır
-5. Modem sıfırlama adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q5" s="6" t="inlineStr">
-        <is>
           <t>Turkcell modem modelleri için varsayılan bilgiler ürün ekibiyle doğrulanmalıdır.</t>
         </is>
       </c>
-      <c r="R5" s="9" t="n">
+      <c r="Q5" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="S5" s="10" t="inlineStr">
+      <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>Ocak</t>
+        </is>
+      </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Ocak</t>
-        </is>
-      </c>
-      <c r="U5" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V5" s="6" t="inlineStr">
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>Modem şifresini değiştirmek isteyen kişi önce arayüze girmeye çalışıyor. Bu adım rakipte en çok trafik getiren sayfa.</t>
         </is>
@@ -13519,37 +13519,28 @@
       </c>
       <c r="P6" s="6" t="inlineStr">
         <is>
-          <t>1. Numara gizleme kodu ve operatör ayarı açıklanır
-2. Gizli numaradan gelen aramayı engelleme adım adım anlatılır
-3. IPhone ve Android ayrı adımlar adım adım anlatılır
-4. Operatör servisiyle kalıcı engelleme adım adım anlatılır
-5. Yasal sınırlar açıklanır</t>
-        </is>
-      </c>
-      <c r="Q6" s="6" t="inlineStr">
-        <is>
           <t>Numarayı gizleme ve gizli numarayı engelleme zıt niyetlerdir; başlık ve ara başlıklar ikisini de karşılamalıdır.</t>
         </is>
       </c>
-      <c r="R6" s="9" t="n">
+      <c r="Q6" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="S6" s="10" t="inlineStr">
+      <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U6" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V6" s="6" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>Kullanıcı ya numarasını gizlemek ya da gizli aramadan kurtulmak istiyor. İki ihtiyaç aynı sayfada karşılanırsa iki arama da aynı yere geliyor.</t>
         </is>
@@ -13771,37 +13762,28 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>1. Kayıt ücreti ve geçerli yılın harç tutarı tablo hâlinde açıklanır
-2. E-Devlet ve BTK üzerinden sorgulama adımları adım adım anlatılır
-3. Kayıtsız telefonun kaç gün kullanılabildiği açıklanır
-4. IMEI numarasının telefondan öğrenilmesi adım adım anlatılır
-5. Kayıt sonrası bekleme süresi açıklanır</t>
-        </is>
-      </c>
-      <c r="Q7" s="6" t="inlineStr">
-        <is>
           <t>Ücret ve süre bilgileri yıl içinde değişmektedir; sayfanın güncellenme tarihi görünür tutulabilir.</t>
         </is>
       </c>
-      <c r="R7" s="9" t="n">
+      <c r="Q7" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="S7" s="10" t="inlineStr">
+      <c r="R7" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>Eylül</t>
+        </is>
+      </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>Eylül</t>
-        </is>
-      </c>
-      <c r="U7" s="7" t="inlineStr">
-        <is>
           <t>Temmuz</t>
         </is>
       </c>
-      <c r="V7" s="6" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>Yurt dışından telefon getiren kişi ücreti ve süreyi arıyor. Bu bilgiyi tek sayfada toplayan taraf aramanın tamamını karşılıyor.</t>
         </is>
@@ -14032,36 +14014,28 @@
       </c>
       <c r="P8" s="6" t="inlineStr">
         <is>
-          <t>1. Google güvenli aramanın ne yaptığı açıklanır
-2. Açma ve kapatma adımları adım adım anlatılır
-3. Kilitli olduğunda yapılabilecekler açıklanır
-4. Çocuk hesaplarında aile bağlantısı ayarı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q8" s="6" t="inlineStr">
-        <is>
           <t>Operatör tarafındaki güvenli internet hizmetiyle karıştırılmaması için ikisi ayrı ara başlıkta ele alınabilir.</t>
         </is>
       </c>
-      <c r="R8" s="9" t="n">
+      <c r="Q8" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="S8" s="10" t="inlineStr">
+      <c r="R8" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>Nisan</t>
+        </is>
+      </c>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>Nisan</t>
-        </is>
-      </c>
-      <c r="U8" s="7" t="inlineStr">
-        <is>
           <t>Şubat</t>
         </is>
       </c>
-      <c r="V8" s="6" t="inlineStr">
+      <c r="U8" s="6" t="inlineStr">
         <is>
           <t>Arama sonuçlarındaki filtreyi açmak veya kapatmak isteyen kullanıcı adım arıyor. Basit ama sürekli aranan bir konu.</t>
         </is>
@@ -14200,36 +14174,28 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>1. PUK kodunun nereden öğrenileceği açıklanır
-2. PIN değiştirme ve kaldırma adım adım anlatılır
-3. Üç kez yanlış PIN girildiğinde izlenecek yol açıklanır
-4. SIM blokesinin kaldırılması adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q9" s="6" t="inlineStr">
-        <is>
           <t>Abone doğrulaması gerektiren adımlarda self servis kanallara yönlendirme yapılabilir.</t>
         </is>
       </c>
-      <c r="R9" s="9" t="n">
+      <c r="Q9" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="S9" s="10" t="inlineStr">
+      <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V9" s="6" t="inlineStr">
+      <c r="U9" s="6" t="inlineStr">
         <is>
           <t>SIM kartı kilitlenen kişi acil çözüm arıyor. Bu anda doğru adımı veren sayfa ziyaret alıyor.</t>
         </is>
@@ -14438,36 +14404,28 @@
       </c>
       <c r="P10" s="6" t="inlineStr">
         <is>
-          <t>1. Kablosuz yansıtma için gereken koşullar açıklanır
-2. IPhone ve Android adımları adım adım anlatılır
-3. Kablo ile yansıtma adım adım anlatılır
-4. Televizyon bulunamadığında kontrol listesi verilir</t>
-        </is>
-      </c>
-      <c r="Q10" s="6" t="inlineStr">
-        <is>
           <t>Yansıtma kalitesi ev ağına bağlıdır; bağlantı bölümüne kısa bir not eklenebilir.</t>
         </is>
       </c>
-      <c r="R10" s="9" t="n">
+      <c r="Q10" s="9" t="n">
         <v>88</v>
       </c>
-      <c r="S10" s="10" t="inlineStr">
+      <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U10" s="7" t="inlineStr">
-        <is>
           <t>Ekim</t>
         </is>
       </c>
-      <c r="V10" s="6" t="inlineStr">
+      <c r="U10" s="6" t="inlineStr">
         <is>
           <t>Telefondaki görüntüyü televizyona aktarmak isteyen kişi adım arıyor. Cihaz farkları netleşince arama karşılanıyor.</t>
         </is>
@@ -14624,36 +14582,28 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>1. IP adresinin tanımı açıklanır
-2. Kendi IP adresinin öğrenilmesi adım adım anlatılır
-3. Statik ve dinamik IP farkı açıklanır
-4. IP adresinin gizlenmesi ve değiştirilmesi adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q11" s="6" t="inlineStr">
-        <is>
           <t>Sonuç sayfasında IP gösteren araçlar öndedir; yazının bir sorgulama aracına bağlanması değerlendirilebilir.</t>
         </is>
       </c>
-      <c r="R11" s="9" t="n">
+      <c r="Q11" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S11" s="10" t="inlineStr">
+      <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>Ocak</t>
+        </is>
+      </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Ocak</t>
-        </is>
-      </c>
-      <c r="U11" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V11" s="6" t="inlineStr">
+      <c r="U11" s="6" t="inlineStr">
         <is>
           <t>Kendi IP adresini öğrenmek isteyen kişi hızlı yanıt arıyor. Sonuç sayfasında araçlar önde, açıklama katmanı boş.</t>
         </is>
@@ -14818,36 +14768,28 @@
       </c>
       <c r="P12" s="6" t="inlineStr">
         <is>
-          <t>1. Android ve iPhone'da indirilenler klasörünün yeri açıklanır
-2. Tarayıcıya göre değişen konumlar açıklanır
-3. Indirilen dosyanın bulunamaması durumu açıklanır
-4. Depolama temizliği açıklanır</t>
-        </is>
-      </c>
-      <c r="Q12" s="6" t="inlineStr">
-        <is>
           <t>Cihaz ve sürüm farkları ekran görüntüsüyle desteklenebilir.</t>
         </is>
       </c>
-      <c r="R12" s="9" t="n">
+      <c r="Q12" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S12" s="10" t="inlineStr">
+      <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>Ekim</t>
+        </is>
+      </c>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>Ekim</t>
-        </is>
-      </c>
-      <c r="U12" s="7" t="inlineStr">
-        <is>
           <t>Ağustos</t>
         </is>
       </c>
-      <c r="V12" s="6" t="inlineStr">
+      <c r="U12" s="6" t="inlineStr">
         <is>
           <t>İndirdiği dosyayı bulamayan kişi klasörün yerini arıyor. Cihaza göre değişen bir bilgi, tek sayfada toplanabilir.</t>
         </is>
@@ -14997,37 +14939,28 @@
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>1. Hesabı geçici dondurma adımları ve kalıcı silmeden farkı açıklanır
-2. Dondurulan hesabın geri açılması adım adım anlatılır
-3. Uygulama açılmadığında kontrol listesi verilir
-4. Giriş yapılamadığında doğrulama adımları adım adım anlatılır
-5. Gönderilen takip isteklerinin görülmesi adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q13" s="6" t="inlineStr">
-        <is>
           <t>Uygulama arayüzü sık değiştiğinden adımların ekran görüntüsüyle desteklenmesi ve güncellenme tarihinin görünür tutulması önerilir.</t>
         </is>
       </c>
-      <c r="R13" s="9" t="n">
+      <c r="Q13" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S13" s="10" t="inlineStr">
+      <c r="R13" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>Eylül</t>
+        </is>
+      </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Eylül</t>
-        </is>
-      </c>
-      <c r="U13" s="7" t="inlineStr">
-        <is>
           <t>Temmuz</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
+      <c r="U13" s="6" t="inlineStr">
         <is>
           <t>Hesabını donduran ya da uygulamaya giremeyen kişi hızlı yanıt arıyor. Rakiplerde konu ayrı yazılara bölünmüş durumda.</t>
         </is>
@@ -15186,35 +15119,28 @@
       </c>
       <c r="P14" s="6" t="inlineStr">
         <is>
-          <t>1. Spam tanımı açıklanır
-2. Spam mesaj ve arama engelleme adımları adım adım anlatılır
-3. Operatör tarafındaki engelleme servisleri açıklanır</t>
-        </is>
-      </c>
-      <c r="Q14" s="6" t="inlineStr">
-        <is>
           <t>Kısa ve doğrudan yanıt veren bir yapı önerilmektedir; sorgu tanım niyetlidir.</t>
         </is>
       </c>
-      <c r="R14" s="9" t="n">
+      <c r="Q14" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S14" s="10" t="inlineStr">
+      <c r="R14" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T14" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U14" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V14" s="6" t="inlineStr">
+      <c r="U14" s="6" t="inlineStr">
         <is>
           <t>Spam kelimesinin anlamını ve engelleme yolunu arayan kişi kısa yanıt istiyor.</t>
         </is>
@@ -15366,38 +15292,29 @@
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>1. SSD ile HDD farkı açıklanır
-2. RAM'in görevi ve yeterli kapasite açıklanır
-3. Ekran kartının ne işe yaradığı açıklanır
-4. Anakartın rolü açıklanır
-5. Bilgisayar yavaşladığında hangi bileşene bakılacağı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q15" s="6" t="inlineStr">
-        <is>
           <t>Ürün önerisi verilmemeli; bilgi katmanında kalınmalıdır.
 NİYET NOTU: 'ram krizi' (500) bellek fiyatlarına ilişkin haber niyetlidir ve bu yazının kapsamı dışındadır.</t>
         </is>
       </c>
-      <c r="R15" s="9" t="n">
+      <c r="Q15" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S15" s="10" t="inlineStr">
+      <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U15" s="7" t="inlineStr">
-        <is>
           <t>Ekim</t>
         </is>
       </c>
-      <c r="V15" s="6" t="inlineStr">
+      <c r="U15" s="6" t="inlineStr">
         <is>
           <t>Bilgisayar alacak veya yükseltecek kişi bileşenlerin ne işe yaradığını soruyor. Tek rehber birden çok aramayı karşılıyor.</t>
         </is>
@@ -15548,35 +15465,28 @@
       </c>
       <c r="P16" s="6" t="inlineStr">
         <is>
-          <t>1. E-imza tanımı açıklanır
-2. Başvuru adımları adım adım anlatılır
-3. Mobil imza ile farkı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q16" s="6" t="inlineStr">
-        <is>
           <t>Turkcell Mobil İmza hizmetiyle bağ kurulabilir; karşılaştırma bölümü ayırt edici olmaktadır.</t>
         </is>
       </c>
-      <c r="R16" s="9" t="n">
+      <c r="Q16" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S16" s="10" t="inlineStr">
+      <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S16" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T16" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U16" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V16" s="6" t="inlineStr">
+      <c r="U16" s="6" t="inlineStr">
         <is>
           <t>E-imza almak isteyen kişi başvuru adımını arıyor. Mobil imza karşılaştırması markaya bağlanıyor.</t>
         </is>
@@ -15727,36 +15637,28 @@
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>1. Taahhüdün tanımı açıklanır
-2. Taahhütlü ve taahhütsüz farkı açıklanır
-3. Taahhüt süresi dolmadan çıkışta ne olduğu açıklanır
-4. Taahhüt süresinin öğrenilmesi adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q17" s="6" t="inlineStr">
-        <is>
           <t>Tanım sorgusudur; ilk paragrafta tek cümlelik karşılık verilmesi önerilir. Kampanya koşulları ürün ekibiyle doğrulanmalıdır.</t>
         </is>
       </c>
-      <c r="R17" s="9" t="n">
+      <c r="Q17" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="S17" s="10" t="inlineStr">
+      <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S17" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U17" s="7" t="inlineStr">
-        <is>
           <t>Ekim</t>
         </is>
       </c>
-      <c r="V17" s="6" t="inlineStr">
+      <c r="U17" s="6" t="inlineStr">
         <is>
           <t>Taahhüt kelimesinin ne anlama geldiğini soran kişi tek cümlelik karşılık bekliyor.</t>
         </is>
@@ -15838,7 +15740,7 @@
             </rPr>
             <t>TON: Uygulamalı ve dürüst. Kritik bölüm numaradan konum bulma; rakip yazılar net yanıt vermiyor, ayırt edici yan burada.
 H2 · Konum Paylaşma Nedir: Kısaca; anlık ve canlı konum farkı.
-H2 · Konum Nasıl Atılır: Detaylı; üç H3 (WhatsApp, Google Haritalar, iPhone), her biri kısa adım listesi. Rakip yazılar (</t>
+H2 · Konum Nasıl Atılır: Detaylı; üç H3 (WhatsApp, Google Haritalar, iPhone'da Mesajlar/iMessage), her biri kısa adım listesi. Rakip yazılar (</t>
           </r>
           <r>
             <rPr>
@@ -15935,36 +15837,28 @@
       </c>
       <c r="P18" s="6" t="inlineStr">
         <is>
-          <t>1. WhatsApp, Google Haritalar ve iMessage üzerinden konum paylaşma adım adım anlatılır
-2. Canlı konum paylaşımı süresi açıklanır
-3. Numaradan konum bulmanın gerçekte mümkün olup olmadığı açıklanır
-4. Konum servislerinin pil etkisi açıklanır</t>
-        </is>
-      </c>
-      <c r="Q18" s="6" t="inlineStr">
-        <is>
           <t>Numaradan konum bulma başlığı yanıltıcı vaatlere açıktır; yasal çerçeve ve gerçek sınırlar açıkça yazılmalıdır.</t>
         </is>
       </c>
-      <c r="R18" s="9" t="n">
+      <c r="Q18" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="S18" s="11" t="inlineStr">
+      <c r="R18" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U18" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V18" s="6" t="inlineStr">
+      <c r="U18" s="6" t="inlineStr">
         <is>
           <t>Konum paylaşmak isteyen çok kişi var; numaradan konum bulma ise beklentisi yanlış kurulmuş bir arama. İkisini dürüstçe ayıran sayfa güven kazanıyor.</t>
         </is>
@@ -16116,37 +16010,28 @@
       </c>
       <c r="P19" s="6" t="inlineStr">
         <is>
-          <t>1. Android'den iPhone'a aktarma adım adım anlatılır
-2. IPhone'dan iPhone'a hızlı başlangıç açıklanır
-3. Android'den Android'e aktarma adım adım anlatılır
-4. WhatsApp geçmişinin taşınması adım adım anlatılır
-5. Aktarma sırasında sık karşılaşılan durumlar açıklanır</t>
-        </is>
-      </c>
-      <c r="Q19" s="6" t="inlineStr">
-        <is>
           <t>Numara taşıma ile veri aktarma farklı işlemlerdir; ikisinin karıştırılmaması için kısa bir ayrım notu eklenebilir.</t>
         </is>
       </c>
-      <c r="R19" s="9" t="n">
+      <c r="Q19" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="S19" s="11" t="inlineStr">
+      <c r="R19" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
+          <t>Ocak</t>
+        </is>
+      </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Ocak</t>
-        </is>
-      </c>
-      <c r="U19" s="7" t="inlineStr">
-        <is>
           <t>Kasım</t>
         </is>
       </c>
-      <c r="V19" s="6" t="inlineStr">
+      <c r="U19" s="6" t="inlineStr">
         <is>
           <t>Telefon değiştiren kişi verisini kaybetmeden taşımak istiyor. Android ve iPhone ayrımını tek sayfada veren içerik bulunmuyor.</t>
         </is>
@@ -16222,7 +16107,7 @@
             </rPr>
             <t>TON: Seçki formatı. Sonuç sayfası liste bekliyor; kurulum adımları listenin sonuna alınır.
 H2 · Chrome Eklentileri Nedir: Kısaca; uzantı ve eklenti kelimelerinin aynı şeyi anlattığı belirtilir.
-H2-H4 · Üç kategori: Her kategoride dört-beş eklenti, her eklenti aynı şablonla: ad, ne işe yaradığı, kime uygun olduğu. Puanlama yapılmaz. Rakip yazılar (</t>
+H2-H4 · Üç kategori (üretkenlik, güvenlik, alışveriş): Her kategoride dört-beş eklenti, her eklenti aynı şablonla: ad, ne işe yaradığı, kime uygun olduğu. Puanlama yapılmaz. Rakip yazılar (</t>
           </r>
           <r>
             <rPr>
@@ -16304,36 +16189,28 @@
       </c>
       <c r="P20" s="6" t="inlineStr">
         <is>
-          <t>1. Kullanım alanına göre eklenti seçkisi: üretkenlik, güvenlik, alışveriş açıklanır
-2. Her eklenti için tek cümlelik ne işe yaradığı açıklanır
-3. Eklentinin eklenmesi ve kaldırılması adım adım anlatılır
-4. Eklenti izinlerinin görülmesi ve güvenilir eklentinin ayırt edilmesi adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q20" s="6" t="inlineStr">
-        <is>
           <t>Seçki formatı sonuç sayfasıyla uyumludur; kurulum adımları listenin sonunda kısa bir bölüm olarak verilebilir.</t>
         </is>
       </c>
-      <c r="R20" s="9" t="n">
+      <c r="Q20" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="S20" s="11" t="inlineStr">
+      <c r="R20" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S20" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T20" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U20" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V20" s="6" t="inlineStr">
+      <c r="U20" s="6" t="inlineStr">
         <is>
           <t>Eklenti arayan kişi tek bir kurulum adımı değil, hangi eklentinin ne işe yaradığını gösteren bir seçki bekliyor.</t>
         </is>
@@ -16481,36 +16358,28 @@
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>1. E-posta adresi oluşturma adımları adım adım anlatılır
-2. Telefonda hesap kurulumu adım adım anlatılır
-3. E-posta yazarken dikkat edilecekler açıklanır
-4. Iki adımlı doğrulama adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q21" s="6" t="inlineStr">
-        <is>
           <t>Sağlayıcı adımları değişmektedir; adımlar sağlayıcı bazında ayrılabilir.</t>
         </is>
       </c>
-      <c r="R21" s="9" t="n">
+      <c r="Q21" s="9" t="n">
         <v>84</v>
       </c>
-      <c r="S21" s="11" t="inlineStr">
+      <c r="R21" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S21" s="7" t="inlineStr">
+        <is>
+          <t>Eylül</t>
+        </is>
+      </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Eylül</t>
-        </is>
-      </c>
-      <c r="U21" s="7" t="inlineStr">
-        <is>
           <t>Temmuz</t>
         </is>
       </c>
-      <c r="V21" s="6" t="inlineStr">
+      <c r="U21" s="6" t="inlineStr">
         <is>
           <t>E-posta hesabı açmak veya telefona kurmak isteyen kişi adım arıyor.</t>
         </is>
@@ -16632,36 +16501,28 @@
       </c>
       <c r="P22" s="6" t="inlineStr">
         <is>
-          <t>1. Android ve iOS için güncelleme adımları adım adım anlatılır
-2. Güncelleme görünmüyorsa yapılabilecekler açıklanır
-3. Güncelleme öncesi yedekleme adım adım anlatılır
-4. Depolama alanı yetmediğinde izlenecek yol açıklanır</t>
-        </is>
-      </c>
-      <c r="Q22" s="6" t="inlineStr">
-        <is>
           <t>Tek soruya odaklı içeriktir; yanıt açılış paragrafında verilip adımlar numaralı listeye alınabilir.</t>
         </is>
       </c>
-      <c r="R22" s="9" t="n">
+      <c r="Q22" s="9" t="n">
         <v>84</v>
       </c>
-      <c r="S22" s="11" t="inlineStr">
+      <c r="R22" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S22" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U22" s="7" t="inlineStr">
-        <is>
           <t>Eylül</t>
         </is>
       </c>
-      <c r="V22" s="6" t="inlineStr">
+      <c r="U22" s="6" t="inlineStr">
         <is>
           <t>Telefonunu güncellemek isteyen kişi adım arıyor; tek soruya odaklı kısa içerik yeterli oluyor.</t>
         </is>
@@ -16735,7 +16596,7 @@
         <is>
           <t>TON: Kısayol rehberi. Kısayol tablosu yazının merkezinde, sayfanın üst yarısında.
 H2 · Nedir: Kısaca; ekran görüntüsü ve ekran kaydı farkı tek ayrımla. PAA'daki "ekran kaydı hangi tuş" sorusu bu ayrımda karşılanır.
-H2 · Windows: Üç H3, her yöntem için ne zaman tercih edileceği tek satırla.
+H2 · Windows: Üç H3 (PrtScn tuşu, Windows+Shift+S, Ekran Alıntısı Aracı), her yöntem için ne zaman tercih edileceği tek satırla.
 H2 · Mac: Kısayollar madde listesi.
 H2 · Kısayollar Tablosu: İşletim sistemi / iş / kısayol / kaydedilen yer sütunları; alıntılanabilir blok.
 H2 · Nereye Kaydedilir: Pano ve dosya ayrımı; varsayılan klasörler.
@@ -16809,37 +16670,28 @@
       </c>
       <c r="P23" s="6" t="inlineStr">
         <is>
-          <t>1. Windows'ta üç yöntem: PrtScn, Windows+Shift+S, Ekran Alıntısı Aracı açıklanır
-2. Mac kısayolları adım adım anlatılır
-3. Kısayol tablosu verilir
-4. Görüntünün kaydedildiği klasör açıklanır
-5. Ekran görüntüsünün düzenlenmesi ve paylaşılması adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q23" s="6" t="inlineStr">
-        <is>
           <t>Kısayol tablosu alıntılanabilir bir blok olarak kurgulanabilir.</t>
         </is>
       </c>
-      <c r="R23" s="9" t="n">
+      <c r="Q23" s="9" t="n">
         <v>83</v>
       </c>
-      <c r="S23" s="11" t="inlineStr">
+      <c r="R23" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S23" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U23" s="7" t="inlineStr">
-        <is>
           <t>Ekim</t>
         </is>
       </c>
-      <c r="V23" s="6" t="inlineStr">
+      <c r="U23" s="6" t="inlineStr">
         <is>
           <t>Bilgisayarda ekran görüntüsü almak isteyen kişi kısayol arıyor; Windows ve Mac karşılığını tek sayfada veren içerik sonuç sayfasında sınırlı.</t>
         </is>
@@ -16969,36 +16821,28 @@
       </c>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>1. ESIM ile fiziksel SIM farkı açıklanır
-2. ESIM destekleyen telefon listesi verilir
-3. Mevcut hattı eSIM'e taşıma adımları adım adım anlatılır
-4. Yurt dışında eSIM kullanımı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q24" s="6" t="inlineStr">
-        <is>
           <t>Destekleyen cihaz listesi hızla değişmektedir; güncellenebilir tablo olarak kurgulanabilir.</t>
         </is>
       </c>
-      <c r="R24" s="9" t="n">
+      <c r="Q24" s="9" t="n">
         <v>82</v>
       </c>
-      <c r="S24" s="10" t="inlineStr">
+      <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
+      <c r="S24" s="7" t="inlineStr">
+        <is>
+          <t>Eylül</t>
+        </is>
+      </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>Eylül</t>
-        </is>
-      </c>
-      <c r="U24" s="7" t="inlineStr">
-        <is>
           <t>Temmuz</t>
         </is>
       </c>
-      <c r="V24" s="6" t="inlineStr">
+      <c r="U24" s="6" t="inlineStr">
         <is>
           <t>eSIM'e geçmek isteyen kişi önce telefonunun desteklediğini doğrulamak istiyor. Cihaz listesi sayfayı vazgeçilmez kılıyor. Telco AI Overview takip listesi: bu başlık Telco AI Overview takibindeki eSIM kümesiyle örtüşmektedir ve Öncelik 2 bandından yükseltilmiştir; ayrıntısı 06B sekmesindedir.</t>
         </is>
@@ -17179,36 +17023,28 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>1. Sıfırlama öncesi yedekleme adım adım anlatılır
-2. Android'de fabrika ayarlarına dönüş adımları adım adım anlatılır
-3. IPhone'da sıfırlama adımları adım adım anlatılır
-4. Sıfırlama sonrası hesap doğrulama adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q25" s="6" t="inlineStr">
-        <is>
           <t>Veri kaybı uyarısının açılışta verilmesi önerilir; adımlar cihaz sürümüne göre değiştiğinden güncellenme tarihi görünür tutulabilir.</t>
         </is>
       </c>
-      <c r="R25" s="9" t="n">
+      <c r="Q25" s="9" t="n">
         <v>82</v>
       </c>
-      <c r="S25" s="11" t="inlineStr">
+      <c r="R25" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S25" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U25" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V25" s="6" t="inlineStr">
+      <c r="U25" s="6" t="inlineStr">
         <is>
           <t>Telefonunu satmadan ya da sorun gidermek için sıfırlamak isteyen kişi adım arıyor.</t>
         </is>
@@ -17352,35 +17188,28 @@
       </c>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>1. Deepfake tanımı açıklanır
-2. Sahte içeriğin anlaşılma yolları adım adım anlatılır
-3. Dolandırıcılık senaryoları açıklanır</t>
-        </is>
-      </c>
-      <c r="Q26" s="6" t="inlineStr">
-        <is>
           <t>Blogun mevcut yapay zeka içerikleriyle iç bağlantı kurulabilir.</t>
         </is>
       </c>
-      <c r="R26" s="9" t="n">
+      <c r="Q26" s="9" t="n">
         <v>82</v>
       </c>
-      <c r="S26" s="11" t="inlineStr">
+      <c r="R26" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S26" s="7" t="inlineStr">
+        <is>
+          <t>Ocak</t>
+        </is>
+      </c>
       <c r="T26" s="7" t="inlineStr">
         <is>
-          <t>Ocak</t>
-        </is>
-      </c>
-      <c r="U26" s="7" t="inlineStr">
-        <is>
           <t>Kasım</t>
         </is>
       </c>
-      <c r="V26" s="6" t="inlineStr">
+      <c r="U26" s="6" t="inlineStr">
         <is>
           <t>Sahte video ve ses içeriklerinin nasıl anlaşıldığını merak eden kişi tanım arıyor.</t>
         </is>
@@ -17448,7 +17277,7 @@
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>TON: Karar yardımı; satış yapmaz.
-H2 · Ne Demek: Kısaca.
+H2 · Ne Demek: Kısaca; yenileme yetkisinin yönetmelikle tanımlı olduğu ve yetkili yenileme merkezi kavramı tek cümleyle verilir.
 H2 · İkinci El Farkı: Dört satırlık tablo. PAA'da "2. el mi yenilenmiş mi" doğrudan soruluyor; tablo bu soruyu karşılar.
 H2 · Kalite Sınıfları: Tablo; A/B/C ve G1/G2 adlandırmaları açıklanır, satıcıya göre değişebildiği notu. Soru kelimesi taramasında sınıf bazlı aramalar ayrı hacim taşıyor.
 H2 · Garanti Süresi: Kısaca; kapsam ve dışında kalanlar.
@@ -17511,36 +17340,28 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>1. Yenilenmiş telefon tanımı ve yasal çerçeve açıklanır
-2. Kalite sınıfları açıklanır
-3. Garanti süresi ve kapsamı açıklanır
-4. Satın almadan önce kontrol listesi verilir</t>
-        </is>
-      </c>
-      <c r="Q27" s="6" t="inlineStr">
-        <is>
           <t>Yenilenmiş cihaz satışıyla ilgili güncel mevzuat doğrulanmalıdır.</t>
         </is>
       </c>
-      <c r="R27" s="9" t="n">
+      <c r="Q27" s="9" t="n">
         <v>82</v>
       </c>
-      <c r="S27" s="11" t="inlineStr">
+      <c r="R27" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
+          <t>Ağustos</t>
+        </is>
+      </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Ağustos</t>
-        </is>
-      </c>
-      <c r="U27" s="7" t="inlineStr">
-        <is>
           <t>Haziran</t>
         </is>
       </c>
-      <c r="V27" s="6" t="inlineStr">
+      <c r="U27" s="6" t="inlineStr">
         <is>
           <t>Yenilenmiş telefon almayı düşünen kişi garanti ve kalite soruyor. Satın alma kararına yakın bir arama.</t>
         </is>
@@ -17691,35 +17512,28 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>1. AirTag tanımı ve çalışma mantığı açıklanır
-2. Kurulum adımları adım adım anlatılır
-3. Takip edilme uyarısı ve gizlilik açıklanır</t>
-        </is>
-      </c>
-      <c r="Q28" s="6" t="inlineStr">
-        <is>
           <t>Gizlilik uyarısı bölümü rakip sayfalarda eksiktir.</t>
         </is>
       </c>
-      <c r="R28" s="9" t="n">
+      <c r="Q28" s="9" t="n">
         <v>81</v>
       </c>
-      <c r="S28" s="11" t="inlineStr">
+      <c r="R28" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S28" s="7" t="inlineStr">
+        <is>
+          <t>Haziran</t>
+        </is>
+      </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>Haziran</t>
-        </is>
-      </c>
-      <c r="U28" s="7" t="inlineStr">
-        <is>
           <t>Nisan</t>
         </is>
       </c>
-      <c r="V28" s="6" t="inlineStr">
+      <c r="U28" s="6" t="inlineStr">
         <is>
           <t>Eşya takip cihazı alan veya takip edildiğinden şüphelenen kişi bilgi arıyor.</t>
         </is>
@@ -17835,35 +17649,28 @@
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>1. OEM tanımı açıklanır
-2. OEM ürün ile orijinal ürün farkı açıklanır
-3. Telefon ve donanımda OEM kullanımı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q29" s="6" t="inlineStr">
-        <is>
           <t>Tanım sorgusudur; kısa ve alıntılanabilir bir açılış paragrafı önerilmektedir.</t>
         </is>
       </c>
-      <c r="R29" s="9" t="n">
+      <c r="Q29" s="9" t="n">
         <v>81</v>
       </c>
-      <c r="S29" s="11" t="inlineStr">
+      <c r="R29" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S29" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U29" s="7" t="inlineStr">
-        <is>
           <t>Eylül</t>
         </is>
       </c>
-      <c r="V29" s="6" t="inlineStr">
+      <c r="U29" s="6" t="inlineStr">
         <is>
           <t>Ürün açıklamalarında gördüğü OEM ifadesinin anlamını arayan kişi tek cümlelik yanıt istiyor.</t>
         </is>
@@ -17994,35 +17801,28 @@
       </c>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>1. KVKK tanımı açıklanır
-2. Kişisel veri türleri açıklanır
-3. Veri sahibinin hakları açıklanır</t>
-        </is>
-      </c>
-      <c r="Q30" s="6" t="inlineStr">
-        <is>
           <t>Hukuki metin niteliği taşımamalıdır; bilgilendirme sınırında kalınmalıdır.</t>
         </is>
       </c>
-      <c r="R30" s="9" t="n">
+      <c r="Q30" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="S30" s="11" t="inlineStr">
+      <c r="R30" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S30" s="7" t="inlineStr">
+        <is>
+          <t>Aralık</t>
+        </is>
+      </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>Aralık</t>
-        </is>
-      </c>
-      <c r="U30" s="7" t="inlineStr">
-        <is>
           <t>Ekim</t>
         </is>
       </c>
-      <c r="V30" s="6" t="inlineStr">
+      <c r="U30" s="6" t="inlineStr">
         <is>
           <t>Kişisel verilerle ilgili hakkını merak eden kişi kısa açıklama arıyor.</t>
         </is>
@@ -18193,36 +17993,28 @@
       </c>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>1. Isınmanın yaygın nedenleri açıklanır
-2. Şarj sırasında ısınma adım adım anlatılır
-3. Isınmayı azaltan ayarlar açıklanır
-4. Servise götürmeyi gerektiren durumlar açıklanır</t>
-        </is>
-      </c>
-      <c r="Q31" s="6" t="inlineStr">
-        <is>
           <t>Tek soruya odaklı içeriktir; yanıt açılış paragrafında üç nedenle özetlenebilir.</t>
         </is>
       </c>
-      <c r="R31" s="9" t="n">
+      <c r="Q31" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="S31" s="11" t="inlineStr">
+      <c r="R31" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S31" s="7" t="inlineStr">
+        <is>
+          <t>Temmuz</t>
+        </is>
+      </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>Temmuz</t>
-        </is>
-      </c>
-      <c r="U31" s="7" t="inlineStr">
-        <is>
           <t>Mayıs</t>
         </is>
       </c>
-      <c r="V31" s="6" t="inlineStr">
+      <c r="U31" s="6" t="inlineStr">
         <is>
           <t>Telefonu ısınan kişi nedenini ve ne yapacağını soruyor; yanıt kısa ve doğrudan verilebilir.</t>
         </is>
@@ -18354,36 +18146,29 @@
       </c>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>1. Müşteri numarasının tanımı açıklanır
-2. Faturada ve uygulamada nereden görüldüğü açıklanır
-3. Abone numarası ile farkı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q32" s="6" t="inlineStr">
-        <is>
           <t>Tanım sorgusudur; hesap ekranına yönlendirme ürün ekibiyle doğrulanmalıdır.
 NİYET NOTU: Jenerik 'müşteri numarası' hacminin büyük bölümü bankacılık aramalarından gelmektedir (yapı kredi 2.400, banka 600, firma 500, halkbank 450, ziraat ve akbank 250'şer). Banka markası içeren aramalar bu yazıyla karşılanamaz. Yazı bankacılık ve telekom kullanımını ayrı bölümlerde ele almakta, aynı ayrımı rakip blog da yapmaktadır.</t>
         </is>
       </c>
-      <c r="R32" s="9" t="n">
+      <c r="Q32" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="S32" s="11" t="inlineStr">
+      <c r="R32" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
+      <c r="S32" s="7" t="inlineStr">
+        <is>
+          <t>Mart</t>
+        </is>
+      </c>
       <c r="T32" s="7" t="inlineStr">
         <is>
-          <t>Mart</t>
-        </is>
-      </c>
-      <c r="U32" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V32" s="6" t="inlineStr">
+      <c r="U32" s="6" t="inlineStr">
         <is>
           <t>Müşteri numarasını nereden bulacağını arayan abone kısa ve net yanıt bekliyor.</t>
         </is>
@@ -18531,36 +18316,28 @@
       </c>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>1. OTP tanımı açıklanır
-2. SMS ile gelen tek kullanımlık şifrenin nasıl çalıştığı açıklanır
-3. OTP paylaşımının riskleri açıklanır
-4. OTP gelmediğinde yapılabilecekler açıklanır</t>
-        </is>
-      </c>
-      <c r="Q33" s="6" t="inlineStr">
-        <is>
           <t>Dolandırıcılık uyarısı bölümü marka güvenliği açısından değerli olabilir.</t>
         </is>
       </c>
-      <c r="R33" s="9" t="n">
+      <c r="Q33" s="9" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="12" t="inlineStr">
+      <c r="R33" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S33" s="7" t="inlineStr">
+        <is>
+          <t>Mart</t>
+        </is>
+      </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>Mart</t>
-        </is>
-      </c>
-      <c r="U33" s="7" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="V33" s="6" t="inlineStr">
+      <c r="U33" s="6" t="inlineStr">
         <is>
           <t>Bankadan ya da uygulamadan gelen OTP ifadesinin ne olduğunu soran kişi kısa yanıt bekliyor.</t>
         </is>
@@ -18669,36 +18446,28 @@
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>1. QLED tanımı açıklanır
-2. QLED ve OLED farkı tablo hâlinde açıklanır
-3. Hangi kullanım için hangisi açıklanır
-4. Parlaklık ve ömür karşılaştırması verilir</t>
-        </is>
-      </c>
-      <c r="Q34" s="6" t="inlineStr">
-        <is>
           <t>Ürün önerisi verilmemesi, bilgi katmanında kalınması önerilir.</t>
         </is>
       </c>
-      <c r="R34" s="9" t="n">
+      <c r="Q34" s="9" t="n">
         <v>79</v>
       </c>
-      <c r="S34" s="12" t="inlineStr">
+      <c r="R34" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S34" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T34" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U34" s="7" t="inlineStr">
-        <is>
           <t>Eylül</t>
         </is>
       </c>
-      <c r="V34" s="6" t="inlineStr">
+      <c r="U34" s="6" t="inlineStr">
         <is>
           <t>Televizyon alacak kişi QLED ile OLED arasındaki farkı soruyor.</t>
         </is>
@@ -18803,36 +18572,28 @@
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>1. Medya okuryazarlığının tanımı açıklanır
-2. Yanlış bilgiyi ayırt etme adımları adım adım anlatılır
-3. Kaynak doğrulama yöntemleri açıklanır
-4. Çocuklar için ipuçları açıklanır</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr">
-        <is>
           <t>Blogun dijital güvenlik yazılarıyla bağlantılandırılması konuyu markanın çizgisine oturtabilir.</t>
         </is>
       </c>
-      <c r="R35" s="9" t="n">
+      <c r="Q35" s="9" t="n">
         <v>79</v>
       </c>
-      <c r="S35" s="12" t="inlineStr">
+      <c r="R35" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S35" s="7" t="inlineStr">
+        <is>
+          <t>Eylül</t>
+        </is>
+      </c>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>Eylül</t>
-        </is>
-      </c>
-      <c r="U35" s="7" t="inlineStr">
-        <is>
           <t>Temmuz</t>
         </is>
       </c>
-      <c r="V35" s="6" t="inlineStr">
+      <c r="U35" s="6" t="inlineStr">
         <is>
           <t>Doğru bilgiyi ayırt etmeyi öğrenmek isteyen kişi tanım ve yöntem arıyor.</t>
         </is>
@@ -18962,37 +18723,29 @@
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>1. TAG teriminin anlamı açıklanır
-2. Sosyal medyada etiketleme adım adım anlatılır
-3. NFC etiketi anlamı açıklanır
-4. Hangi bağlamda hangi anlamın kullanıldığı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q36" s="6" t="inlineStr">
-        <is>
           <t>Kelimenin birden çok anlamı bulunmaktadır; açılışta hangi anlamların ele alındığı belirtilmelidir.
 NİYET NOTU: Jenerik 'tag' hacminin büyük bölümü ulaşım uygulaması (martı tag 6.600, tag taksi 450, tag sürücü 450, tag premium 250) ve takip cihazı (air tag 2.600) aramalarından gelmektedir; skin tag ve Google Tag Manager gibi alan dışı anlamlar da bu hacme dahildir. Yazı, arama hacmine göre sıralanmış anlam bölümleriyle kurgulanmıştır; kümeye atanan hacmin tamamının karşılanması beklenmemelidir.</t>
         </is>
       </c>
-      <c r="R36" s="9" t="n">
+      <c r="Q36" s="9" t="n">
         <v>78</v>
       </c>
-      <c r="S36" s="12" t="inlineStr">
+      <c r="R36" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S36" s="7" t="inlineStr">
+        <is>
+          <t>Ekim</t>
+        </is>
+      </c>
       <c r="T36" s="7" t="inlineStr">
         <is>
-          <t>Ekim</t>
-        </is>
-      </c>
-      <c r="U36" s="7" t="inlineStr">
-        <is>
           <t>Ağustos</t>
         </is>
       </c>
-      <c r="V36" s="6" t="inlineStr">
+      <c r="U36" s="6" t="inlineStr">
         <is>
           <t>TAG kelimesinin karşılığını arayan kişi kısa tanım bekliyor.</t>
         </is>
@@ -19161,35 +18914,28 @@
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>1. Kamerayla karekod okutma adımları adım adım anlatılır
-2. Kamera okutmadığında yapılabilecekler açıklanır
-3. Sahte karekodların ayırt edilmesi adım adım anlatılır</t>
-        </is>
-      </c>
-      <c r="Q37" s="6" t="inlineStr">
-        <is>
           <t>Tek soruya odaklı içeriktir; adımlar numaralı listeye alınabilir.</t>
         </is>
       </c>
-      <c r="R37" s="9" t="n">
+      <c r="Q37" s="9" t="n">
         <v>78</v>
       </c>
-      <c r="S37" s="12" t="inlineStr">
+      <c r="R37" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>Ekim</t>
+        </is>
+      </c>
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>Ekim</t>
-        </is>
-      </c>
-      <c r="U37" s="7" t="inlineStr">
-        <is>
           <t>Ağustos</t>
         </is>
       </c>
-      <c r="V37" s="6" t="inlineStr">
+      <c r="U37" s="6" t="inlineStr">
         <is>
           <t>Karekod okutmayı bilmeyen kişi adım arıyor; soru tek ve nettir.</t>
         </is>
@@ -19319,36 +19065,28 @@
       </c>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>1. Hat devrinin tanımı açıklanır
-2. Devir için gereken belgeler açıklanır
-3. Devir ücreti açıklanır
-4. Devir sonrası fatura ve taahhüt durumu açıklanır</t>
-        </is>
-      </c>
-      <c r="Q38" s="6" t="inlineStr">
-        <is>
           <t>Ücret ve belge bilgileri değişkendir; ürün ekibiyle doğrulanmalı ve güncellenme tarihi görünür tutulmalıdır.</t>
         </is>
       </c>
-      <c r="R38" s="9" t="n">
+      <c r="Q38" s="9" t="n">
         <v>77</v>
       </c>
-      <c r="S38" s="12" t="inlineStr">
+      <c r="R38" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S38" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T38" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U38" s="7" t="inlineStr">
-        <is>
           <t>Eylül</t>
         </is>
       </c>
-      <c r="V38" s="6" t="inlineStr">
+      <c r="U38" s="6" t="inlineStr">
         <is>
           <t>Hattını başkasına devretmek isteyen abone ücreti ve gereken belgeleri arıyor.</t>
         </is>
@@ -19417,7 +19155,7 @@
             </rPr>
             <t>TON: Tanım sorgusu. İlk paragraf tanım, hemen ardından örnek adresin parçalanmış şeması.
 H2 · URL Nedir: Kısaca; açılım parantez içinde. PAA'daki "URL ne demek Türkçe" burada.
-H2 · Bölümleri: Üç H3, örnek adres üzerinden; şema sade metin, görsel yok. Rakip yazı (</t>
+H2 · Bölümleri: Üç H3 (protokol, alan adı, yol), örnek adres üzerinden; şema sade metin, görsel yok. Rakip yazı (</t>
           </r>
           <r>
             <rPr>
@@ -19472,35 +19210,28 @@
       </c>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>1. URL tanımı açıklanır
-2. URL bölümleri: protokol, alan adı, yol açıklanır
-3. Güvenli URL'nin nasıl anlaşıldığı açıklanır</t>
-        </is>
-      </c>
-      <c r="Q39" s="6" t="inlineStr">
-        <is>
           <t>Tanım sorgusudur; ilk paragrafta tek cümlelik karşılık ve ardından bölüm şeması önerilir.</t>
         </is>
       </c>
-      <c r="R39" s="9" t="n">
+      <c r="Q39" s="9" t="n">
         <v>77</v>
       </c>
-      <c r="S39" s="12" t="inlineStr">
+      <c r="R39" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S39" s="7" t="inlineStr">
+        <is>
+          <t>Mart</t>
+        </is>
+      </c>
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>Mart</t>
-        </is>
-      </c>
-      <c r="U39" s="7" t="inlineStr">
-        <is>
           <t>Ocak</t>
         </is>
       </c>
-      <c r="V39" s="6" t="inlineStr">
+      <c r="U39" s="6" t="inlineStr">
         <is>
           <t>URL kelimesinin karşılığını arayan kişi kısa tanım bekliyor.</t>
         </is>
@@ -19625,36 +19356,28 @@
       </c>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>1. Apple Arcade tanımı açıklanır
-2. Abonelik ücreti ve deneme süresi açıklanır
-3. Hangi cihazlarda çalıştığı açıklanır
-4. Oyunların çevrimdışı oynanabilirliği açıklanır</t>
-        </is>
-      </c>
-      <c r="Q40" s="6" t="inlineStr">
-        <is>
           <t>Ücret bilgisi değişkendir; güncellenme tarihi görünür tutulabilir.</t>
         </is>
       </c>
-      <c r="R40" s="9" t="n">
+      <c r="Q40" s="9" t="n">
         <v>76</v>
       </c>
-      <c r="S40" s="12" t="inlineStr">
+      <c r="R40" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S40" s="7" t="inlineStr">
+        <is>
+          <t>Ocak</t>
+        </is>
+      </c>
       <c r="T40" s="7" t="inlineStr">
         <is>
-          <t>Ocak</t>
-        </is>
-      </c>
-      <c r="U40" s="7" t="inlineStr">
-        <is>
           <t>Kasım</t>
         </is>
       </c>
-      <c r="V40" s="6" t="inlineStr">
+      <c r="U40" s="6" t="inlineStr">
         <is>
           <t>Apple Arcade aboneliğini merak eden kişi kapsamı ve ücreti soruyor.</t>
         </is>
@@ -19770,35 +19493,28 @@
       </c>
       <c r="P41" s="6" t="inlineStr">
         <is>
-          <t>1. FreeDOS tanımı açıklanır
-2. Işletim sistemi yüklü olmayan bilgisayarın anlamı açıklanır
-3. Sonrasında yapılabilecekler açıklanır</t>
-        </is>
-      </c>
-      <c r="Q41" s="6" t="inlineStr">
-        <is>
           <t>Blogun işletim sistemi yazısıyla iç bağlantı kurulabilir.</t>
         </is>
       </c>
-      <c r="R41" s="9" t="n">
+      <c r="Q41" s="9" t="n">
         <v>73</v>
       </c>
-      <c r="S41" s="12" t="inlineStr">
+      <c r="R41" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
+      <c r="S41" s="7" t="inlineStr">
+        <is>
+          <t>Kasım</t>
+        </is>
+      </c>
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>Kasım</t>
-        </is>
-      </c>
-      <c r="U41" s="7" t="inlineStr">
-        <is>
           <t>Eylül</t>
         </is>
       </c>
-      <c r="V41" s="6" t="inlineStr">
+      <c r="U41" s="6" t="inlineStr">
         <is>
           <t>İşletim sistemi yüklü olmayan bilgisayar alan kişi ne yapacağını arıyor.</t>
         </is>
@@ -19806,8 +19522,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A2:U2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30994,7 +30710,7 @@
         </is>
       </c>
     </row>
-    <row r="425" ht="51" customHeight="1">
+    <row r="425" ht="66" customHeight="1">
       <c r="A425" s="6" t="inlineStr">
         <is>
           <t>Konum Paylaşma ve Numaradan Konum Bulma</t>
@@ -31023,7 +30739,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t>Detaylı; üç H3 (WhatsApp, Google Haritalar, iPhone), her biri kısa adım listesi. Rakip yazılar (</t>
+            <t>Detaylı; üç H3 (WhatsApp, Google Haritalar, iPhone'da Mesajlar/iMessage), her biri kısa adım listesi. Rakip yazılar (</t>
           </r>
           <r>
             <rPr>
@@ -32397,7 +32113,7 @@
       </c>
       <c r="D476" s="6" t="inlineStr">
         <is>
-          <t>H2-H4 · Üç kategori</t>
+          <t>H2-H4 · Üç kategori (üretkenlik, güvenlik, alışveriş)</t>
         </is>
       </c>
       <c r="E476" s="6" t="inlineStr">
@@ -34182,7 +33898,7 @@
       </c>
       <c r="E544" s="6" t="inlineStr">
         <is>
-          <t>Üç H3, her yöntem için ne zaman tercih edileceği tek satırla.</t>
+          <t>Üç H3 (PrtScn tuşu, Windows+Shift+S, Ekran Alıntısı Aracı), her yöntem için ne zaman tercih edileceği tek satırla.</t>
         </is>
       </c>
     </row>
@@ -36819,7 +36535,7 @@
       </c>
       <c r="E643" s="6" t="inlineStr">
         <is>
-          <t>Kısaca.</t>
+          <t>Kısaca; yenileme yetkisinin yönetmelikle tanımlı olduğu ve yetkili yenileme merkezi kavramı tek cümleyle verilir.</t>
         </is>
       </c>
     </row>
@@ -44443,7 +44159,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t>Üç H3, örnek adres üzerinden; şema sade metin, görsel yok. Rakip yazı (</t>
+            <t>Üç H3 (protokol, alan adı, yol), örnek adres üzerinden; şema sade metin, görsel yok. Rakip yazı (</t>
           </r>
           <r>
             <rPr>
@@ -46630,7 +46346,7 @@
         </is>
       </c>
     </row>
-    <row r="1015" ht="36" customHeight="1">
+    <row r="1015" ht="66" customHeight="1">
       <c r="A1015" s="6" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/web-sitelerinin-altyapisi-hosting-nedir-ne-ise-yarar</t>
@@ -46653,7 +46369,31 @@
       </c>
       <c r="E1015" s="6" t="inlineStr">
         <is>
-          <t>Ziyaretçi bandına göre üç senaryo madde listesi; her senaryoda önerilen tür ve gerekçe. PAA'daki "hosting ücreti nedir" sorusu tutar verilmeden, neye göre değiştiği anlatılarak karşılanır.</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Ziyaretçi bandına göre üç senaryo madde listesi; her senaryoda önerilen tür ve gerekçe. Rakip yazı (</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Türk Telekom</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>, 3. sıra) konuyu tek uzun bölümde veriyor ve bizim yazımız 12 ara başlıkla zaten daha ayrıntılı; eksik olan derinlik değil seçim kriteri, bu yüzden bölüm karar yardımı olarak yazılır. PAA'daki "hosting ücreti nedir" sorusu tutar verilmeden, neye göre değiştiği anlatılarak karşılanır.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -48358,7 +48098,7 @@
         </is>
       </c>
     </row>
-    <row r="1080" ht="36" customHeight="1">
+    <row r="1080" ht="51" customHeight="1">
       <c r="A1080" s="6" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/ping-internette-gecikmenin-gercek-nedeni</t>
@@ -48387,7 +48127,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t xml:space="preserve">İki H3 (komut satırı, hız testi siteleri), kısa adımlar; oyun içi gösterge tek paragraf. </t>
+            <t xml:space="preserve">İki H3 (komut satırı, hız testi siteleri), kısa adımlar; oyun içi gösterge tek paragraf. Mevcut yazıda ölçüm bölümü var, test adımı yok. Rakip yazının başlığı doğrudan "Ping Testi Nedir? Nasıl Yapılır?"; </t>
           </r>
           <r>
             <rPr>
@@ -48404,7 +48144,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t xml:space="preserve"> sıralamayı test aracıyla alıyor; yazı kendi hız testi aracına iç bağlantı verir.</t>
+            <t xml:space="preserve"> sıralamayı test aracıyla alıyor, yazı kendi hız testi aracına iç bağlantı verir.</t>
           </r>
         </is>
       </c>
@@ -51320,7 +51060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -51348,12 +51088,11 @@
     <col width="110" customWidth="1" min="23" max="23"/>
     <col width="58" customWidth="1" min="24" max="24"/>
     <col width="52" customWidth="1" min="25" max="25"/>
-    <col width="58" customWidth="1" min="26" max="26"/>
-    <col width="44" customWidth="1" min="27" max="27"/>
-    <col width="15" customWidth="1" min="28" max="28"/>
-    <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="50" customWidth="1" min="31" max="31"/>
+    <col width="44" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="50" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -51391,9 +51130,8 @@
       <c r="AB1" s="2" t="n"/>
       <c r="AC1" s="2" t="n"/>
       <c r="AD1" s="2" t="n"/>
-      <c r="AE1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="81" customHeight="1">
+    </row>
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <r>
@@ -51475,6 +51213,24 @@
               <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">
+Kurgu sütunu: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Güncelleme yönergesi ayrı bir sütun değildir: eklenecek bölümler, bölümlerin yazıdaki yeri ve gövde düzenlemesi "İçerik Kurgusu ve Yönergesi" sütununda birleştirilmiştir. Kelime yoğunluğu yönergesi ayrı sütunda kalmaktadır.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00FF7B52"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">
 Durum: </t>
           </r>
           <r>
@@ -51516,7 +51272,6 @@
       <c r="AB2" s="4" t="n"/>
       <c r="AC2" s="4" t="n"/>
       <c r="AD2" s="4" t="n"/>
-      <c r="AE2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -51549,7 +51304,6 @@
       <c r="AB3" s="2" t="n"/>
       <c r="AC3" s="2" t="n"/>
       <c r="AD3" s="2" t="n"/>
-      <c r="AE3" s="2" t="n"/>
     </row>
     <row r="4" ht="51" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -51727,7 +51481,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>İçerik Kurgusu</t>
+          <t>İçerik Kurgusu ve Yönergesi</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -51747,30 +51501,25 @@
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
-          <t>Güncelleme Yönergesi</t>
+          <t>Dikkat Edilecek</t>
         </is>
       </c>
       <c r="AA4" s="5" t="inlineStr">
         <is>
-          <t>Dikkat Edilecek</t>
+          <t>Toplam Aylık Arama</t>
         </is>
       </c>
       <c r="AB4" s="5" t="inlineStr">
         <is>
-          <t>Toplam Aylık Arama</t>
+          <t>Puan</t>
         </is>
       </c>
       <c r="AC4" s="5" t="inlineStr">
         <is>
-          <t>Puan</t>
+          <t>Öncelik</t>
         </is>
       </c>
       <c r="AD4" s="5" t="inlineStr">
-        <is>
-          <t>Öncelik</t>
-        </is>
-      </c>
-      <c r="AE4" s="5" t="inlineStr">
         <is>
           <t>Ne Anlama Geliyor</t>
         </is>
@@ -51953,30 +51702,21 @@
       </c>
       <c r="Z5" s="6" t="inlineStr">
         <is>
-          <t>1. 'Windows nedir' sorgusu 1.059 Impression alıyor ancak sayfa 9.7 ortalama sırada kalıyor; Windows, macOS ve Linux için üç ayrı H3 açılıp her birine sürüm adı, tipik kullanıcı profili ve donanım gereksinimi yazılabilir
-2. 'işletim sistemleri sadece bilgisayarlara özgü müdür' sorgusu 646 Impression ile 3.2 sırada geliyor, yani soru soruluyor ama yanıt bölümü yok: telefon, akıllı televizyon, akıllı saat ve araç sistemlerini kapsayan 'İşletim Sistemi Yalnız Bilgisayarlarda mı Bulunur?' başlığı eklenebilir
-3. Mobil tarafta Android ve iOS tek cümlede geçiyor; ikisi ayrı H3 olarak açılıp aralarındaki uygulama mağazası, güncelleme ve donanım farkı üç maddeyle verilebilir
-4. 'bilgisayar işletim sistemleri' ve 'işletim sistemleri nelerdir' kelimeleri gövdede hiç geçmiyor; mevcut 'İşletim Sistemi Çeşitleri Nelerdir?' başlığının açılış cümlesi bu iki kalıbı da karşılayacak biçimde yazılabilir
-5. 'işletim sistemleri hakkında aşağıdakilerden hangisi doğru değildir' sorgusu 4.221 Impression alıyor ve ödev kaynaklı; bu sorguya içerik yazılması önerilmez, ölçüm okunurken hesaba katılması yeterlidir açıklanır</t>
-        </is>
-      </c>
-      <c r="AA5" s="6" t="inlineStr">
-        <is>
           <t>Sürüm adları ve donanım gereksinimleri yıl içinde değişiyor; güncellenme tarihinin görünür tutulması bu yazıda değer taşıyor.</t>
         </is>
       </c>
-      <c r="AB5" s="8" t="n">
+      <c r="AA5" s="8" t="n">
         <v>11870</v>
       </c>
-      <c r="AC5" s="9" t="n">
+      <c r="AB5" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="AD5" s="10" t="inlineStr">
+      <c r="AC5" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
-      <c r="AE5" s="6" t="inlineStr">
+      <c r="AD5" s="6" t="inlineStr">
         <is>
           <t>Rakip aynı soruda üçüncü sırada ve yedi kat trafik alıyor. Mobil ve masaüstü ayrımı eksik.</t>
         </is>
@@ -52098,12 +51838,36 @@
       </c>
       <c r="V6" s="6" t="inlineStr">
         <is>
-          <t>EKLENECEK BÖLÜMLERİN YERİ: Karşılaştırma tablosu mevcut "Hosting Türleri Nelerdir?" başlığının içine; domain bölümü mevcut fark bölümünün yerine; seçim bölümü sona.
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>EKLENECEK BÖLÜMLERİN YERİ: Karşılaştırma tablosu mevcut "Hosting Türleri Nelerdir?" başlığının içine; domain bölümü mevcut fark bölümünün yerine; seçim bölümü sona.
 H2 · Hosting Türleri Karşılaştırma Tablosu: Sayfa "hosting" sorgusunda 31.2 sırada. Mevcut türler bölümü metin; paylaşımlı, VPS, bulut, adanmış satırlarında kaynak paylaşımı, trafik kapasitesi ve kimin için uygun olduğu sütunlu tabloya çevrilir. Rakip yazı (GoDaddy) her tür için avantaj-dezavantaj çifti veriyor; tabloya iki sütun daha eklenir.
 H2 · Domain ve Hosting Ayrı Ayrı mı Alınır: "domain ve hosting nedir" 4.6 sırada 409 Impression. Tek örnek üzerinden ilişki, ardından doğrudan yanıt: ayrı da birlikte de alınabilir.
-H2 · Küçük İşletme İçin Hangi Hosting: Ziyaretçi bandına göre üç senaryo madde listesi; her senaryoda önerilen tür ve gerekçe. PAA'daki "hosting ücreti nedir" sorusu tutar verilmeden, neye göre değiştiği anlatılarak karşılanır.
+H2 · Küçük İşletme İçin Hangi Hosting: Ziyaretçi bandına göre üç senaryo madde listesi; her senaryoda önerilen tür ve gerekçe. Rakip yazı (</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Türk Telekom</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>, 3. sıra) konuyu tek uzun bölümde veriyor ve bizim yazımız 12 ara başlıkla zaten daha ayrıntılı; eksik olan derinlik değil seçim kriteri, bu yüzden bölüm karar yardımı olarak yazılır. PAA'daki "hosting ücreti nedir" sorusu tutar verilmeden, neye göre değiştiği anlatılarak karşılanır.
 GÖVDE DÜZENLEMESİ: "turkcell host" sorgusu 399 Impression ile 5.1 sırada; markanın barındırma hizmetine tek iç bağlantı.
 DİKKAT: Fiyat verilmez; kapasite ve senaryo üzerinden anlatılır.</t>
+          </r>
         </is>
       </c>
       <c r="W6" s="6" t="inlineStr">
@@ -52155,53 +51919,21 @@
       </c>
       <c r="Z6" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. Sayfa 'hosting' sorgusunda 31.2 ortalama sırada; bu sorguda ilk sayfaya girebilmek için mevcut 'Hosting Türleri Nelerdir?' başlığı tabloya çevrilebilir: paylaşımlı, VPS, bulut ve adanmış sunucu satırlarında kaynak paylaşımı, tipik trafik kapasitesi ve kimin için uygun olduğu üç sütunda verilir
-2. 'domain ve hosting nedir' sorgusu 4.6 sırada 409 Impression alıyor; mevcut fark bölümü iki cümlede kalıyor, alan adı ile barındırmanın ilişkisi bir örnek üzerinden anlatılıp 'ikisi ayrı ayrı mı alınır' sorusu yanıtlanabilir
-3. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Türk Telekom</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un aynı sorguda 3. sıradaki yazısı 1.239 kelime ve konuyu tek uzun bölümde veriyor; bizim yazımız 12 ara başlıkla daha ayrıntılı, eksik olan derinlik değil seçim kriteri: 'Küçük İşletme İçin Hangi Hosting Seçilir?' başlığı altında aylık ziyaretçi bandına göre üç senaryo eklenebilir
-4. 'turkcell host' sorgusu 399 Impression ile 5.1 sırada geliyor; markanın barındırma hizmetine tek cümlelik bir bağlantı, arama niyetini karşılar açıklanır</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA6" s="6" t="inlineStr">
-        <is>
           <t>Fiyat bilgisi verilmemesi, kapasite ve kullanım senaryosu üzerinden anlatılması önerilir.</t>
         </is>
       </c>
-      <c r="AB6" s="8" t="n">
+      <c r="AA6" s="8" t="n">
         <v>8640</v>
       </c>
-      <c r="AC6" s="9" t="n">
+      <c r="AB6" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="AD6" s="10" t="inlineStr">
+      <c r="AC6" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
-      <c r="AE6" s="6" t="inlineStr">
+      <c r="AD6" s="6" t="inlineStr">
         <is>
           <t>Bu soruda hosting satan siteler önde. Yazının ilk sıraya çıkması zor; beklenti buna göre kurulmalı.</t>
         </is>
@@ -52498,54 +52230,21 @@
       </c>
       <c r="Z7" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. 'nfc etiketi nedir' sorgusu 3.835 Impression alıyor ancak sayfa 8.7 sırada ve tek click getiriyor; yazıda NFC etiketi hiç geçmiyor. 'NFC Etiketi Nedir, Ne İşe Yarar?' başlığı altında etiketin ne olduğu, telefona nasıl okutulduğu ve ev otomasyonu gibi kullanım örnekleri verilebilir
-2. 'nfc kart nedir' 832 Impression alıyor; temassız kartın NFC ile ilişkisi ayrı bir H3 olarak açılabilir
-3. 'nfc açma', 'iphone nfc açma', 'apple nfc açma' ve 'nfc özelliği nasıl açılır redmi' kelimelerinin hiçbiri gövdede geçmiyor; mevcut 'NFC Nasıl Açılır ve Kullanılır?' başlığı cihaz bazında üçe ayrılabilir: iPhone, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Samsung</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve"> ve Xiaomi/Redmi. Her biri iki-üç adımla anlatılır
-4. 'nfc özelliği olan telefonlar' kelimesi gövdede yok; NFC destekleyen model ailelerini marka bazında listeleyen kısa bir tablo, bu aramayı karşılar açıklanır
-5. 'nfc alanı neresi' aramasının karşılığı da bulunmuyor; NFC anteninin telefonun neresinde olduğu ve nasıl bulunacağı tek paragrafla eklenebilir</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA7" s="6" t="inlineStr">
-        <is>
           <t>Cihaz arayüzleri sürümle değişiyor; adımların model ailesi düzeyinde verilmesi ve güncellenme tarihinin görünür tutulması önerilir.</t>
         </is>
       </c>
-      <c r="AB7" s="8" t="n">
+      <c r="AA7" s="8" t="n">
         <v>145620</v>
       </c>
-      <c r="AC7" s="9" t="n">
+      <c r="AB7" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="AD7" s="10" t="inlineStr">
+      <c r="AC7" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
-      <c r="AE7" s="6" t="inlineStr">
+      <c r="AD7" s="6" t="inlineStr">
         <is>
           <t>Sayfa tanımı veriyor ama kullanıcı NFC'yi telefonunda açmaya çalışıyor. Açma adımları eklenirse arama karşılanmış oluyor.</t>
         </is>
@@ -52703,30 +52402,21 @@
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
-          <t>1. 'gemini yapay zeka' sorgusu 92.496 Impression ile 79 click getiriyor ve kelime gövdede hiç geçmiyor; giriş paragrafında ve bir ara başlıkta bu kalıbın kullanılması, sayfanın hâlihazırda göründüğü aramayı güçlendirir açıklanır
-2. 'gemini türkçe' kelimesi de gövdede yok; 'Gemini Türkçe Destekliyor mu?' başlığı altında dil desteği, Türkçe yanıt kalitesi ve arayüz dili üç maddeyle verilebilir
-3. Mevcut 'Gemini ile Bard Arasındaki Fark' bölümü artık geçerliliğini yitiriyor, Bard adı kullanımdan kalktı; bu bölüm 'Gemini ile ChatGPT Arasındaki Fark' karşılaştırmasına çevrilip yanıt kaynağı, görsel üretimi, dosya yükleme ve ücretsiz sürüm sınırları dört satırlık tabloya alınabilir
-4. Ücretsiz ve ücretli sürüm ayrımı yazıda geçmiyor; 'Gemini Ücretsiz mi?' başlığı, sonuç sayfasındaki soru bloğunda da görünen bir arama adım adım anlatılır
-5. Sayfanın Impression'ı jenerik marka aramasından geliyor ve o aramada sonuç sayfasının ilk beş sırası Google'ın kendi adresleri; kazanım kullanım ve karşılaştırma sorularında olduğu için yeni bölümler bu iki eksende kurgulanmalıdır</t>
-        </is>
-      </c>
-      <c r="AA8" s="6" t="inlineStr">
-        <is>
           <t>Yapay zeka ürünlerinde sürüm ve fiyatlandırma sık değişiyor; tablo değerlerinin tarihiyle birlikte verilmesi önerilir.</t>
         </is>
       </c>
-      <c r="AB8" s="8" t="n">
+      <c r="AA8" s="8" t="n">
         <v>77400</v>
       </c>
-      <c r="AC8" s="9" t="n">
+      <c r="AB8" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="AD8" s="10" t="inlineStr">
+      <c r="AC8" s="10" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
         </is>
       </c>
-      <c r="AE8" s="6" t="inlineStr">
+      <c r="AD8" s="6" t="inlineStr">
         <is>
           <t>Yazı altı ayda 16.3 milyon impression alıp 2.125 click getirmiştir. Sorun içerikte değil, jenerik marka aramasının sonuç sayfasında: üst sıralar Google'ın kendi adreslerinde. Kazanım, kullanım ve karşılaştırma sorularında.</t>
         </is>
@@ -52847,7 +52537,7 @@
               <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">EKLENECEK BÖLÜMLERİN YERİ: Test bölümü mevcut ölçüm bölümünün yerine; değer tablosu tanımın hemen ardına; ping atmak bölümü onun ardına; düşürme bölümü mevcut "Ping Nasıl Düşürülür?" başlığının yerine.
-H2 · Ping Testi Nasıl Yapılır: İki H3 (komut satırı, hız testi siteleri), kısa adımlar; oyun içi gösterge tek paragraf. </t>
+H2 · Ping Testi Nasıl Yapılır: İki H3 (komut satırı, hız testi siteleri), kısa adımlar; oyun içi gösterge tek paragraf. Mevcut yazıda ölçüm bölümü var, test adımı yok. Rakip yazının başlığı doğrudan "Ping Testi Nedir? Nasıl Yapılır?"; </t>
           </r>
           <r>
             <rPr>
@@ -52864,7 +52554,7 @@
               <color rgb="0010332F"/>
               <sz val="10.5"/>
             </rPr>
-            <t xml:space="preserve"> sıralamayı test aracıyla alıyor; yazı kendi hız testi aracına iç bağlantı verir.
+            <t xml:space="preserve"> sıralamayı test aracıyla alıyor, yazı kendi hız testi aracına iç bağlantı verir.
 H2 · İdeal Ping Değerleri Tablosu: "ping nedir" sorgusunda 3.918 Impression'dan 1 click; yanıt sonuç sayfasında veriliyor. Giriş tanımı kısaltılır ve hemen altına değer tablosu (rekabetçi oyun, genel oyun, video görüşme, üzeri) konur; her satırda bağlantı türü. PAA'daki "ping kaç olursa iyi" ve "50 ping iyi mi" soruları tabloyla karşılanır.
 H2 · Ping Atmak Ne Demek: Kısaca.
 H2 · Nasıl Düşürülür: Dört somut adım madde listesi; her adımda beklenen etki. PAA'daki "neden yüksek olur" sorusu bölüm girişinde.
@@ -52940,53 +52630,21 @@
       </c>
       <c r="Z9" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Türk Telekom</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un aynı konudaki yazısının başlığı 'Ping Testi Nedir? Nasıl Yapılır?'; bizim yazımızda ölçüm bölümü var ancak test adımı yok. Komut satırından ping testi, hız testi siteleri ve oyun içi gecikme göstergesi üç adımda anlatılabilir
-2. 'ping nedir' sorgusunda sayfa 3.7 ortalama sırada ancak 3.918 Impression'dan yalnız 1 click geliyor; bu tablo sonuç sayfasının üstünde yanıtın verildiğine işaret ediyor. Giriş paragrafındaki tanımın tek cümleye indirilmesi ve ideal ping aralığının hemen altına tablo olarak konması, alıntılanma ihtimalini artırır açıklanır
-3. Ideal değer aralığı yazıda cümle içinde geçiyor; 'Rekabetçi oyun 0-30 ms, genel oyun 30-60 ms, video görüşme 60-100 ms, üzeri sorunlu' satırlarından oluşan bir tablo hem okuyucuya hem AI yanıtına daha kullanışlı geliyor açıklanır
-4. Mevcut 'Ping Nasıl Düşürülür?' bölümü genel öneriler içeriyor; kablo bağlantısı, 5 GHz bant, arka plan indirmeleri ve sunucu bölgesi seçimi gibi dört somut adıma çevrilebilir</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA9" s="6" t="inlineStr">
-        <is>
           <t>Ping değerleri bağlantı türüne göre değişiyor; verilen aralıkların hangi bağlantı için geçerli olduğu belirtilmelidir.</t>
         </is>
       </c>
-      <c r="AB9" s="8" t="n">
+      <c r="AA9" s="8" t="n">
         <v>4400</v>
       </c>
-      <c r="AC9" s="9" t="n">
+      <c r="AB9" s="9" t="n">
         <v>66</v>
       </c>
-      <c r="AD9" s="11" t="inlineStr">
+      <c r="AC9" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
-      <c r="AE9" s="6" t="inlineStr">
+      <c r="AD9" s="6" t="inlineStr">
         <is>
           <t>Rakip bir test aracıyla sıralanıyor. Yazıya araç bağlantısı eklenmesi aradaki farkı açıklıyor.</t>
         </is>
@@ -53212,29 +52870,21 @@
       </c>
       <c r="Z10" s="6" t="inlineStr">
         <is>
-          <t>1. Sayfa 'type c' sorgusunda 91.693 Impression alıyor ancak 7.8 sırada ve 23 click getiriyor; bu aramada sonuç sayfasının üst sıraları ürün listeleyen mağazalarda olduğu için bilgi tarafında kazanım 'type c nedir' ve 'type c ne demek' kalıplarında. İkisi de gövdede birer kez geçiyor, ara başlığa taşınabilir
-2. USB-C sürümleri yazıda ayrışmıyor; USB 3.2, USB4 ve Thunderbolt 4 için veri hızı, güç aktarımı ve görüntü desteği sütunlarından oluşan bir tablo, konunun en çok karıştırılan yanını karşılar açıklanır
-3. 'Type-C ile hızlı şarj nasıl çalışır' sorusu yazıda yanıtlanmıyor; Power Delivery kademelerinin watt değerleriyle verildiği bir bölüm eklenebilir
-4. Yazıda kablo kalitesinin aktarım hızını nasıl sınırladığı geçmiyor; aynı görünen iki kablonun farklı hız vermesi somut bir okuyucu sorusu ve tek paragrafla karşılanabilir</t>
-        </is>
-      </c>
-      <c r="AA10" s="6" t="inlineStr">
-        <is>
           <t>Ürün önerisi verilmemesi, teknik ayrım katmanında kalınması önerilir; şarj aleti ve kablo aramaları mağaza sayfalarına aittir.</t>
         </is>
       </c>
-      <c r="AB10" s="8" t="n">
+      <c r="AA10" s="8" t="n">
         <v>3400</v>
       </c>
-      <c r="AC10" s="9" t="n">
+      <c r="AB10" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="AD10" s="11" t="inlineStr">
+      <c r="AC10" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
-      <c r="AE10" s="6" t="inlineStr">
+      <c r="AD10" s="6" t="inlineStr">
         <is>
           <t>Arayan kişi çoğunlukla kablo satın alıyor. Yazı bunu karşılamıyor; ürün sayfasına köprü kurmak daha gerçekçi.</t>
         </is>
@@ -53499,59 +53149,27 @@
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. 'adsl vdsl farkı' sorgusu 3.3 ortalama sırada 3.014 Impression alıyor; bu sayfanın en güçlü olduğu alan ve mevcut karşılaştırma metin hâlinde. Hız, mesafe hassasiyeti, upload oranı ve tipik kullanım satırlarından oluşan bir tabloya çevrilmesi ilk üçe girme ihtimalini artırır açıklanır
-2. 'vdsl modem nedir' sorgusu 1.878 Impression ile 4.5 sırada; modem tarafı yazıda tek cümlede geçiyor. 'VDSL Modem Nedir, ADSL Modemden Farkı Ne?' başlığı altında uyumluluk ve değişim gerekliliği anlatılabilir
-3. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Vodafone</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un aynı sorguda 1. sıradaki yazısı 485 kelime; bizim yazımız 1.092 kelimeyle iki katı ve daha kapsamlı. Eksik olan uzunluk değil, tablo ve karar yardımı: 'Hangi Bağlantı Kimin İçin Uygun?' bölümü, ev tipi ve kullanıcı sayısına göre üç senaryo verebilir
-4. Fiber bağlantı yazıda karşılaştırmaya girmiyor; ADSL, VDSL ve fiber üçlüsünün aynı tabloda görülmesi, okuyucunun asıl sorusunu karşılar açıklanır</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA11" s="6" t="inlineStr">
-        <is>
           <t>Altyapı ve hız değerleri bölgeye göre değişiyor; sorgulama işleminin ilgili hizmet sayfasından yapılabileceği belirtilebilir.</t>
         </is>
       </c>
-      <c r="AB11" s="8" t="n">
+      <c r="AA11" s="8" t="n">
         <v>7160</v>
       </c>
-      <c r="AC11" s="9" t="n">
+      <c r="AB11" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="AD11" s="11" t="inlineStr">
+      <c r="AC11" s="11" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
         </is>
       </c>
-      <c r="AE11" s="6" t="inlineStr">
+      <c r="AD11" s="6" t="inlineStr">
         <is>
           <t>Rakipler aynı konuyu daha ayrıntılı işliyor ve dört kat trafik alıyor. Karşılaştırma tablosu farkı kapatabilir.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="263.5" customHeight="1">
+    <row r="12" ht="209.5" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>https://www.turkcell.com.tr/blog/internette-dalgalanma-neden-olur-jitter-degeri-nedir</t>
@@ -53748,54 +53366,21 @@
       </c>
       <c r="Z12" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. 'jitter kaç olmalı' sorgusu 866 Impression ile 7.8 sırada geliyor ve yazıda ideal aralık tablo hâlinde verilmiyor; 'Video görüşme için 30 ms altı, oyun için 20 ms altı, akış için 50 ms altı' satırlarından oluşan bir tablo bu aramayı karşılar açıklanır
-2. 'net jitter ne demek' ve 'net jitter' sorguları birlikte 1.869 Impression alıyor; terim gövdede geçmiyor. Ağ tarafındaki kullanımın ayrı bir cümleyle açıklanması yeterli açıklanır
-3. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Vodafone</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un 1. sıradaki yazısında ana terim 55 kez geçiyor, bizim yazımızda 23; sayının artırılması değil, jitter kelimesinin ara başlıklarda ve tablo satırlarında da kullanılması öneriliyor açıklanır
-4. Jitter ile ping ve paket kaybı arasındaki fark yazıda net ayrılmıyor; üç kavramı yan yana koyan kısa bir bölüm, konunun en sık karıştırılan yanını kapatıyor açıklanır
-5. Jitter düşürme adımları yazıda genel kalıyor; kablolu bağlantı, QoS ayarı, arka plan trafiği ve modem konumu dört somut maddeye çevrilebilir</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA12" s="6" t="inlineStr">
-        <is>
           <t>Değerler bağlantı türüne ve uygulamaya göre değişiyor; aralıkların hangi senaryo için geçerli olduğu yazılmalıdır.</t>
         </is>
       </c>
-      <c r="AB12" s="8" t="n">
+      <c r="AA12" s="8" t="n">
         <v>5350</v>
       </c>
-      <c r="AC12" s="9" t="n">
+      <c r="AB12" s="9" t="n">
         <v>59</v>
       </c>
-      <c r="AD12" s="12" t="inlineStr">
+      <c r="AC12" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
-      <c r="AE12" s="6" t="inlineStr">
+      <c r="AD12" s="6" t="inlineStr">
         <is>
           <t>Rakip aynı formatta ama birinci sırada. Fark, ideal değer tablosu gibi somut bilgide.</t>
         </is>
@@ -54041,53 +53626,21 @@
       </c>
       <c r="Z13" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. 'wifi 6 modem' ve 'wifi 6 modem nedir' sorguları birlikte 4.132 Impression alıyor, sayfa 7.8 ve 4.1 sıralarda; modem tarafı yazıda tek cümlede geçiyor. 'Wi-Fi 6 Modem Nedir, Hangi Modemler Destekler?' başlığı altında uyumluluk, cihaz tarafı gereksinimi ve mevcut modemin yeterli olup olmadığı anlatılabilir
-2. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Vodafone</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un aynı sorguda 1. sıradaki yazısı 1.639 kelime ve 14 ara başlık taşıyor; bizim yazımız 1.146 kelime ve 11 başlık. Fark, kapsam derinliğinde: OFDMA, MU-MIMO ve Target Wake Time gibi teknik kavramların her biri iki cümlelik alt bölüme çevrilebilir
-3. Wi-Fi 6E ve Wi-Fi 7 yazıda geçmiyor; okuyucu Wi-Fi 6 ile Wi-Fi 6E ayrımını sık soruyor, kısa bir bölüm bu boşluğu kapatır açıklanır
-4. 'wifi 6 nedir' sorgusunda sayfa 3.4 sırada ve 48 click alıyor; giriş paragrafındaki tanımın tek cümleye indirilmesi, ilk üçe yaklaşmak için en düşük maliyetli adım açıklanır</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA13" s="6" t="inlineStr">
-        <is>
           <t>Cihaz uyumluluğu marka ve model ailesine göre değişiyor; genel ifadeler yerine standart adları kullanılmalıdır.</t>
         </is>
       </c>
-      <c r="AB13" s="8" t="n">
+      <c r="AA13" s="8" t="n">
         <v>3370</v>
       </c>
-      <c r="AC13" s="9" t="n">
+      <c r="AB13" s="9" t="n">
         <v>57</v>
       </c>
-      <c r="AD13" s="12" t="inlineStr">
+      <c r="AC13" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
-      <c r="AE13" s="6" t="inlineStr">
+      <c r="AD13" s="6" t="inlineStr">
         <is>
           <t>Birinci sırada olmasına rağmen tıklama gelmiyor, çünkü arayan kişi modem arıyor. Cihaz bağlantısı eklenmeli.</t>
         </is>
@@ -54267,53 +53820,21 @@
       </c>
       <c r="Z14" s="6" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t xml:space="preserve">1. 'mac adresi sorgulama' ve 'mac adresi nasıl bulunur' sorguları birlikte 1.800 Impression alıyor, sayfa 6.7 ve 9.2 sıralarda; adım anlatımı yazıda cihaz bazında ayrışmıyor. Windows, macOS, Android, iPhone ve modem arayüzü için beş kısa adım listesi eklenebilir
-2. 'mac adresinden cihaz bulma' sorgusu 237 Impression alıyor ve yazıda karşılığı yok; MAC adresinin ilk üç baytının üretici kodunu taşıdığı ve bu bilgiyle cihaz markasının bulunabildiği tek paragrafla açıklanabilir
-3. 'telefon mac adresi nedir' sorgusu 4.3 sırada 283 Impression alıyor; telefonlarda rastgele MAC kullanımının (privacy MAC) neden devreye girdiği, okuyucunun gördüğü değerin neden değiştiğini açıklar açıklanır
-4. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>Vodafone</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="0010332F"/>
-              <sz val="10.5"/>
-            </rPr>
-            <t>'un 3. sıradaki yazısında ana terim 46 kez geçiyor, bizim yazımızda 43; kelime sıklığı yeterli, eksik olan cihaz bazında adım anlatımı açıklanır</t>
-          </r>
-        </is>
-      </c>
-      <c r="AA14" s="6" t="inlineStr">
-        <is>
           <t>Rastgele MAC kullanımı işletim sistemi sürümüne göre değişiyor; adımların sürüm bilgisiyle verilmesi önerilir.</t>
         </is>
       </c>
-      <c r="AB14" s="8" t="n">
+      <c r="AA14" s="8" t="n">
         <v>2510</v>
       </c>
-      <c r="AC14" s="9" t="n">
+      <c r="AB14" s="9" t="n">
         <v>56</v>
       </c>
-      <c r="AD14" s="12" t="inlineStr">
+      <c r="AC14" s="12" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
         </is>
       </c>
-      <c r="AE14" s="6" t="inlineStr">
+      <c r="AD14" s="6" t="inlineStr">
         <is>
           <t>Kullanıcı MAC adresini bulmaya çalışıyor. Cihaz bazında adım eklenirse sayfa aramayı karşılıyor.</t>
         </is>
@@ -54321,8 +53842,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:AE1"/>
-    <mergeCell ref="A2:AE2"/>
+    <mergeCell ref="A2:AD2"/>
+    <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId1"/>

</xml_diff>

<commit_message>
06 sekmesine Brief sütunu eklendi
- AI Overview kelime listesindeki her satır, karşılık gelen önerinin 02 sekmesindeki satırına gönderme yapıyor
- Sekmenin not bloğuna brief'in nerede olduğunu söyleyen satır eklendi
- 61 eşleşen kelimenin tamamında gönderme doğrulandı

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
+++ b/Turkcell_Blog_Yeni_Trafik_Kaynaklari_Fikir_Hacim.xlsx
@@ -64286,7 +64286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -64295,7 +64295,8 @@
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -64310,8 +64311,9 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="51" customHeight="1">
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="81" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <r>
@@ -64339,6 +64341,24 @@
               <sz val="10.5"/>
             </rPr>
             <t xml:space="preserve">
+Brief: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="0010332F"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t>Bu sekme kelime listesidir, öneri listesi değildir. Karşılık gelen önerinin ayrıntılı brief'i (alt başlıklar, içerik kurgusu ve yönergesi, cevaplanması gereken sorular, iç link önerileri) 02 Blog Önerileri sekmesindedir; Brief sütunu ilgili satırı göstermektedir. Bölüm bölüm okunabilir dökümü 02B Kurgu ve FAQ Detayı sekmesinde bulunmaktadır. Karşılığı çizgiyle işaretli kelimeler öneri kapsamına alınmamıştır: bir bölümü ürün ya da mağaza aramasıdır, bir bölümü blogun kapsamı dışındadır.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00FF7B52"/>
+              <sz val="10.5"/>
+            </rPr>
+            <t xml:space="preserve">
 Yöntem: </t>
           </r>
           <r>
@@ -64357,6 +64377,7 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -64366,6 +64387,7 @@
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -64400,6 +64422,11 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
+          <t>Brief</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
           <t>Not</t>
         </is>
       </c>
@@ -64433,7 +64460,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64468,7 +64500,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64503,7 +64540,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64538,7 +64580,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64573,7 +64620,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64608,7 +64660,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 12</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64643,7 +64700,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64678,7 +64740,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64713,7 +64780,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64748,7 +64820,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64783,7 +64860,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 11</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64818,7 +64900,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64853,7 +64940,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -64888,7 +64980,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 8</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64923,7 +65020,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 8</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64958,7 +65060,12 @@
           <t>eSIM nedir, nasıl aktive edilir?</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 24</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -64993,7 +65100,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65028,7 +65140,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65063,7 +65180,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65098,7 +65220,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65133,7 +65260,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 8</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65168,7 +65300,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65203,7 +65340,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65238,7 +65380,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65273,7 +65420,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65308,7 +65460,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65343,7 +65500,12 @@
           <t>Taahhüt ne demek?</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 17</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65378,7 +65540,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65413,7 +65580,12 @@
           <t>Spam ne demek?</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 14</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65448,7 +65620,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 10</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65483,7 +65660,12 @@
           <t>AirTag nedir ve nasıl çalışır?</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 28</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65518,7 +65700,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65553,7 +65740,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 23</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65588,7 +65780,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65623,7 +65820,12 @@
           <t>Yenilenmiş telefon ne demek?</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 27</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65658,7 +65860,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 18</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65693,7 +65900,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65728,7 +65940,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65763,7 +65980,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 15</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65798,7 +66020,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65833,7 +66060,12 @@
           <t>E-imza nasıl alınır?</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 16</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65868,7 +66100,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -65903,7 +66140,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65938,7 +66180,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 13</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -65973,7 +66220,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66008,7 +66260,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66043,7 +66300,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66078,7 +66340,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66113,7 +66380,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66148,7 +66420,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66183,7 +66460,12 @@
           <t>KVKK nedir?</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 30</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66218,7 +66500,12 @@
           <t>Deepfake nedir ve nasıl anlaşılır?</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 26</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66253,7 +66540,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66288,7 +66580,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66323,7 +66620,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66358,7 +66660,12 @@
           <t>Telefon neden ısınır?</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 31</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66393,7 +66700,12 @@
           <t>eSIM nedir, nasıl aktive edilir?</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 24</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66428,7 +66740,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66463,7 +66780,12 @@
           <t>Deepfake nedir ve nasıl anlaşılır?</t>
         </is>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 26</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66498,7 +66820,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 10</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66533,7 +66860,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 9</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66568,7 +66900,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66603,7 +66940,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66638,7 +66980,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G68" s="6" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66673,7 +67020,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66708,7 +67060,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66743,7 +67100,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 10</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66778,7 +67140,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G72" s="6" t="inlineStr">
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -66813,7 +67180,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G73" s="6" t="inlineStr">
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66848,7 +67220,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 8</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66883,7 +67260,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66918,7 +67300,12 @@
           <t>Apple Arcade nedir?</t>
         </is>
       </c>
-      <c r="G76" s="6" t="inlineStr">
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 40</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66953,7 +67340,12 @@
           <t>Medya okuryazarlığı nedir?</t>
         </is>
       </c>
-      <c r="G77" s="6" t="inlineStr">
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 35</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -66988,7 +67380,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 11</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67023,7 +67420,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67058,7 +67460,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G80" s="6" t="inlineStr">
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 11</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67093,7 +67500,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G81" s="6" t="inlineStr">
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67128,7 +67540,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67163,7 +67580,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67198,7 +67620,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G84" s="6" t="inlineStr">
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 19</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67233,7 +67660,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G85" s="6" t="inlineStr">
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67268,7 +67700,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 9</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67303,7 +67740,12 @@
           <t>OEM ne demek?</t>
         </is>
       </c>
-      <c r="G87" s="6" t="inlineStr">
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 29</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67338,7 +67780,12 @@
           <t>FreeDOS nedir?</t>
         </is>
       </c>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 41</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67373,7 +67820,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G89" s="6" t="inlineStr">
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 15</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67408,7 +67860,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67443,7 +67900,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67478,7 +67940,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G92" s="6" t="inlineStr">
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67513,7 +67980,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G93" s="6" t="inlineStr">
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67548,7 +68020,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G94" s="6" t="inlineStr">
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67583,7 +68060,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G95" s="6" t="inlineStr">
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 13</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67618,7 +68100,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G96" s="6" t="inlineStr">
+      <c r="G96" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67653,7 +68140,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G97" s="6" t="inlineStr">
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67688,7 +68180,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G98" s="6" t="inlineStr">
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67723,7 +68220,12 @@
           <t>TAG nedir?</t>
         </is>
       </c>
-      <c r="G99" s="6" t="inlineStr">
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 36</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67758,7 +68260,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G100" s="6" t="inlineStr">
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67793,7 +68300,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67828,7 +68340,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G102" s="6" t="inlineStr">
+      <c r="G102" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67863,7 +68380,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G103" s="6" t="inlineStr">
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -67898,7 +68420,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G104" s="6" t="inlineStr">
+      <c r="G104" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 12</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67933,7 +68460,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G105" s="6" t="inlineStr">
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -67968,7 +68500,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G106" s="6" t="inlineStr">
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 18</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68003,7 +68540,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G107" s="6" t="inlineStr">
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68038,7 +68580,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G108" s="6" t="inlineStr">
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68073,7 +68620,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G109" s="6" t="inlineStr">
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68108,7 +68660,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G110" s="6" t="inlineStr">
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68143,7 +68700,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G111" s="6" t="inlineStr">
+      <c r="G111" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68178,7 +68740,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G112" s="6" t="inlineStr">
+      <c r="G112" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68213,7 +68780,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G113" s="6" t="inlineStr">
+      <c r="G113" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68248,7 +68820,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G114" s="6" t="inlineStr">
+      <c r="G114" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 6</t>
+        </is>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68283,7 +68860,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G115" s="6" t="inlineStr">
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H115" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68318,7 +68900,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G116" s="6" t="inlineStr">
+      <c r="G116" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 11</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68353,7 +68940,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G117" s="6" t="inlineStr">
+      <c r="G117" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H117" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68388,7 +68980,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G118" s="6" t="inlineStr">
+      <c r="G118" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H118" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68423,7 +69020,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G119" s="6" t="inlineStr">
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 23</t>
+        </is>
+      </c>
+      <c r="H119" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68458,7 +69060,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G120" s="6" t="inlineStr">
+      <c r="G120" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H120" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68493,7 +69100,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G121" s="6" t="inlineStr">
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H121" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68528,7 +69140,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G122" s="6" t="inlineStr">
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H122" s="6" t="inlineStr">
         <is>
           <t>AI Overview yanıtına kaynak olabilecek kısa bölüm değerlendirilebilir</t>
         </is>
@@ -68563,7 +69180,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G123" s="6" t="inlineStr">
+      <c r="G123" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 5</t>
+        </is>
+      </c>
+      <c r="H123" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68598,7 +69220,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G124" s="6" t="inlineStr">
+      <c r="G124" s="7" t="inlineStr">
+        <is>
+          <t>02 Blog Önerileri · satır 7</t>
+        </is>
+      </c>
+      <c r="H124" s="6" t="inlineStr">
         <is>
           <t>Öneri kapsamındadır</t>
         </is>
@@ -68606,8 +69233,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>